<commit_message>
Plan: volver a pedir Moneyman para pagar a Ama el 1 nov y liquidar Vivus por 1500 € el 29 nov
Pagolisto y Crédito Santander 1 pasan a enero–marzo. El Excel se
regenera con el nuevo escenario y una columna de ahorro por liquidar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JEd5Mo2HQL6TrpXUCZoFXP
</commit_message>
<xml_diff>
--- a/excel/plan_de_pagos.xlsx
+++ b/excel/plan_de_pagos.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Supuestos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Calendario'!$A$1:$G$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Calendario'!$A$1:$G$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -110,12 +110,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
+        <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -156,8 +156,8 @@
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -177,8 +177,8 @@
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -281,6 +281,21 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Plan</author>
+  </authors>
+  <commentList>
+    <comment ref="I4" authorId="0" shapeId="0">
+      <text>
+        <t>2.148 € (4 × 537) − 1.500 € de liquidación, según lo que te ofrece Vivus</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -572,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -638,23 +653,23 @@
         <v>46296</v>
       </c>
       <c r="B2" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Ingreso",Calendario!$B$3:$B$69,A2)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A2)</f>
         <v/>
       </c>
       <c r="C2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Gasto",Calendario!$B$3:$B$69,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A2)</f>
         <v/>
       </c>
       <c r="D2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Fijo",Calendario!$B$3:$B$69,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A2)</f>
         <v/>
       </c>
       <c r="E2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Aplazable",Calendario!$B$3:$B$69,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A2)</f>
         <v/>
       </c>
       <c r="F2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Amigo",Calendario!$B$3:$B$69,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A2)</f>
         <v/>
       </c>
       <c r="G2" s="3">
@@ -675,23 +690,23 @@
         <v>46327</v>
       </c>
       <c r="B3" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Ingreso",Calendario!$B$3:$B$69,A3)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A3)</f>
         <v/>
       </c>
       <c r="C3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Gasto",Calendario!$B$3:$B$69,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A3)</f>
         <v/>
       </c>
       <c r="D3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Fijo",Calendario!$B$3:$B$69,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A3)</f>
         <v/>
       </c>
       <c r="E3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Aplazable",Calendario!$B$3:$B$69,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A3)</f>
         <v/>
       </c>
       <c r="F3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Amigo",Calendario!$B$3:$B$69,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A3)</f>
         <v/>
       </c>
       <c r="G3" s="3">
@@ -712,23 +727,23 @@
         <v>46357</v>
       </c>
       <c r="B4" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Ingreso",Calendario!$B$3:$B$69,A4)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A4)</f>
         <v/>
       </c>
       <c r="C4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Gasto",Calendario!$B$3:$B$69,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A4)</f>
         <v/>
       </c>
       <c r="D4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Fijo",Calendario!$B$3:$B$69,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A4)</f>
         <v/>
       </c>
       <c r="E4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Aplazable",Calendario!$B$3:$B$69,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A4)</f>
         <v/>
       </c>
       <c r="F4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Amigo",Calendario!$B$3:$B$69,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A4)</f>
         <v/>
       </c>
       <c r="G4" s="3">
@@ -749,23 +764,23 @@
         <v>46388</v>
       </c>
       <c r="B5" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Ingreso",Calendario!$B$3:$B$69,A5)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A5)</f>
         <v/>
       </c>
       <c r="C5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Gasto",Calendario!$B$3:$B$69,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A5)</f>
         <v/>
       </c>
       <c r="D5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Fijo",Calendario!$B$3:$B$69,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A5)</f>
         <v/>
       </c>
       <c r="E5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Aplazable",Calendario!$B$3:$B$69,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A5)</f>
         <v/>
       </c>
       <c r="F5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Amigo",Calendario!$B$3:$B$69,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A5)</f>
         <v/>
       </c>
       <c r="G5" s="3">
@@ -786,23 +801,23 @@
         <v>46419</v>
       </c>
       <c r="B6" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Ingreso",Calendario!$B$3:$B$69,A6)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A6)</f>
         <v/>
       </c>
       <c r="C6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Gasto",Calendario!$B$3:$B$69,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A6)</f>
         <v/>
       </c>
       <c r="D6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Fijo",Calendario!$B$3:$B$69,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A6)</f>
         <v/>
       </c>
       <c r="E6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Aplazable",Calendario!$B$3:$B$69,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A6)</f>
         <v/>
       </c>
       <c r="F6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Amigo",Calendario!$B$3:$B$69,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A6)</f>
         <v/>
       </c>
       <c r="G6" s="3">
@@ -823,23 +838,23 @@
         <v>46447</v>
       </c>
       <c r="B7" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Ingreso",Calendario!$B$3:$B$69,A7)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A7)</f>
         <v/>
       </c>
       <c r="C7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Gasto",Calendario!$B$3:$B$69,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A7)</f>
         <v/>
       </c>
       <c r="D7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Fijo",Calendario!$B$3:$B$69,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A7)</f>
         <v/>
       </c>
       <c r="E7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Aplazable",Calendario!$B$3:$B$69,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A7)</f>
         <v/>
       </c>
       <c r="F7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Amigo",Calendario!$B$3:$B$69,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A7)</f>
         <v/>
       </c>
       <c r="G7" s="3">
@@ -860,23 +875,23 @@
         <v>46478</v>
       </c>
       <c r="B8" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Ingreso",Calendario!$B$3:$B$69,A8)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A8)</f>
         <v/>
       </c>
       <c r="C8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Gasto",Calendario!$B$3:$B$69,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A8)</f>
         <v/>
       </c>
       <c r="D8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Fijo",Calendario!$B$3:$B$69,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A8)</f>
         <v/>
       </c>
       <c r="E8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Aplazable",Calendario!$B$3:$B$69,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A8)</f>
         <v/>
       </c>
       <c r="F8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Amigo",Calendario!$B$3:$B$69,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A8)</f>
         <v/>
       </c>
       <c r="G8" s="3">
@@ -897,23 +912,23 @@
         <v>46508</v>
       </c>
       <c r="B9" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Ingreso",Calendario!$B$3:$B$69,A9)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A9)</f>
         <v/>
       </c>
       <c r="C9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Gasto",Calendario!$B$3:$B$69,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A9)</f>
         <v/>
       </c>
       <c r="D9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Fijo",Calendario!$B$3:$B$69,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A9)</f>
         <v/>
       </c>
       <c r="E9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Aplazable",Calendario!$B$3:$B$69,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A9)</f>
         <v/>
       </c>
       <c r="F9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Amigo",Calendario!$B$3:$B$69,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A9)</f>
         <v/>
       </c>
       <c r="G9" s="3">
@@ -934,23 +949,23 @@
         <v>46539</v>
       </c>
       <c r="B10" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Ingreso",Calendario!$B$3:$B$69,A10)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A10)</f>
         <v/>
       </c>
       <c r="C10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Gasto",Calendario!$B$3:$B$69,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A10)</f>
         <v/>
       </c>
       <c r="D10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Fijo",Calendario!$B$3:$B$69,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A10)</f>
         <v/>
       </c>
       <c r="E10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Aplazable",Calendario!$B$3:$B$69,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A10)</f>
         <v/>
       </c>
       <c r="F10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Amigo",Calendario!$B$3:$B$69,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A10)</f>
         <v/>
       </c>
       <c r="G10" s="3">
@@ -971,23 +986,23 @@
         <v>46569</v>
       </c>
       <c r="B11" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Ingreso",Calendario!$B$3:$B$69,A11)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A11)</f>
         <v/>
       </c>
       <c r="C11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Gasto",Calendario!$B$3:$B$69,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A11)</f>
         <v/>
       </c>
       <c r="D11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Fijo",Calendario!$B$3:$B$69,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A11)</f>
         <v/>
       </c>
       <c r="E11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Aplazable",Calendario!$B$3:$B$69,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A11)</f>
         <v/>
       </c>
       <c r="F11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Amigo",Calendario!$B$3:$B$69,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A11)</f>
         <v/>
       </c>
       <c r="G11" s="3">
@@ -1008,23 +1023,23 @@
         <v>46600</v>
       </c>
       <c r="B12" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Ingreso",Calendario!$B$3:$B$69,A12)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A12)</f>
         <v/>
       </c>
       <c r="C12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Gasto",Calendario!$B$3:$B$69,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A12)</f>
         <v/>
       </c>
       <c r="D12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Fijo",Calendario!$B$3:$B$69,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A12)</f>
         <v/>
       </c>
       <c r="E12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Aplazable",Calendario!$B$3:$B$69,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A12)</f>
         <v/>
       </c>
       <c r="F12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Amigo",Calendario!$B$3:$B$69,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A12)</f>
         <v/>
       </c>
       <c r="G12" s="3">
@@ -1045,23 +1060,23 @@
         <v>46631</v>
       </c>
       <c r="B13" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Ingreso",Calendario!$B$3:$B$69,A13)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A13)</f>
         <v/>
       </c>
       <c r="C13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Gasto",Calendario!$B$3:$B$69,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A13)</f>
         <v/>
       </c>
       <c r="D13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Fijo",Calendario!$B$3:$B$69,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A13)</f>
         <v/>
       </c>
       <c r="E13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Aplazable",Calendario!$B$3:$B$69,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A13)</f>
         <v/>
       </c>
       <c r="F13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$D$3:$D$69,"Amigo",Calendario!$B$3:$B$69,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A13)</f>
         <v/>
       </c>
       <c r="G13" s="3">
@@ -1078,64 +1093,101 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="2" t="n">
+        <v>46661</v>
+      </c>
+      <c r="B14" s="3">
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A14)</f>
+        <v/>
+      </c>
+      <c r="C14" s="3">
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A14)</f>
+        <v/>
+      </c>
+      <c r="D14" s="3">
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A14)</f>
+        <v/>
+      </c>
+      <c r="E14" s="3">
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="3">
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A14)</f>
+        <v/>
+      </c>
+      <c r="G14" s="3">
+        <f>D14+E14+F14</f>
+        <v/>
+      </c>
+      <c r="H14" s="3">
+        <f>B14-C14-G14</f>
+        <v/>
+      </c>
+      <c r="I14" s="4">
+        <f>Supuestos!$B$5+SUM($H$2:H14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="6">
-        <f>SUM(B2:B13)</f>
-        <v/>
-      </c>
-      <c r="C14" s="6">
-        <f>SUM(C2:C13)</f>
-        <v/>
-      </c>
-      <c r="D14" s="6">
-        <f>SUM(D2:D13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="6">
-        <f>SUM(E2:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="6">
-        <f>SUM(F2:F13)</f>
-        <v/>
-      </c>
-      <c r="G14" s="6">
-        <f>SUM(G2:G13)</f>
-        <v/>
-      </c>
-      <c r="H14" s="6">
-        <f>SUM(H2:H13)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Saldo más bajo del plan</t>
-        </is>
-      </c>
-      <c r="C16" s="4">
-        <f>MIN(Calendario!G2:G69)</f>
+      <c r="B15" s="6">
+        <f>SUM(B2:B14)</f>
+        <v/>
+      </c>
+      <c r="C15" s="6">
+        <f>SUM(C2:C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="6">
+        <f>SUM(D2:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="6">
+        <f>SUM(E2:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="6">
+        <f>SUM(F2:F14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="6">
+        <f>SUM(G2:G14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="6">
+        <f>SUM(H2:H14)</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
+          <t>Saldo más bajo del plan</t>
+        </is>
+      </c>
+      <c r="C17" s="4">
+        <f>MIN(Calendario!G2:G72)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
           <t>Fecha del saldo más bajo</t>
         </is>
       </c>
-      <c r="C17" s="7">
-        <f>INDEX(Calendario!A2:A69,MATCH(C16,Calendario!G2:G69,0))</f>
+      <c r="C18" s="7">
+        <f>INDEX(Calendario!A2:A72,MATCH(C17,Calendario!G2:G72,0))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="H2:I13">
+  <conditionalFormatting sqref="H2:I14">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="0">
       <formula>0</formula>
     </cfRule>
@@ -1150,17 +1202,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="58" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1181,7 +1234,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Pendiente 13 oct (€)</t>
+          <t>Importe a devolver (€)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1202,6 +1255,11 @@
       <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Condiciones</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Ahorro por liquidar (€)</t>
         </is>
       </c>
     </row>
@@ -1225,27 +1283,30 @@
         <v>1400</v>
       </c>
       <c r="E2" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$E$3:$E$69,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A2)</f>
         <v/>
       </c>
       <c r="F2" s="3">
-        <f>D2-E2</f>
+        <f>D2-E2-I2</f>
         <v/>
       </c>
       <c r="G2" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$69,Calendario!$E$3:$E$69,A2)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A2)</f>
         <v/>
       </c>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>Pago único. Te dieron 1.100 €</t>
-        </is>
+          <t>Pago único el 1 nov. Te dieron 1.100 €</t>
+        </is>
+      </c>
+      <c r="I2" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Vivus</t>
+          <t>Moneyman (vuelto a pedir)</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1255,71 +1316,77 @@
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>Vivus</t>
+          <t>Moneyman</t>
         </is>
       </c>
       <c r="D3" s="10" t="n">
-        <v>2148</v>
+        <v>1400</v>
       </c>
       <c r="E3" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$E$3:$E$69,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A3)</f>
         <v/>
       </c>
       <c r="F3" s="3">
-        <f>D3-E3</f>
+        <f>D3-E3-I3</f>
         <v/>
       </c>
       <c r="G3" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$69,Calendario!$E$3:$E$69,A3)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A3)</f>
         <v/>
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>4 cuotas de 537 € desde el 1 nov</t>
-        </is>
+          <t>Nace el 1 nov: recibes 1.100 €, devuelves 1.400 € el 1 dic</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Smartcredito</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Vivus</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Smartcredito</t>
+          <t>Vivus</t>
         </is>
       </c>
       <c r="D4" s="10" t="n">
-        <v>435</v>
+        <v>2148</v>
       </c>
       <c r="E4" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$E$3:$E$69,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A4)</f>
         <v/>
       </c>
       <c r="F4" s="3">
-        <f>D4-E4</f>
+        <f>D4-E4-I4</f>
         <v/>
       </c>
       <c r="G4" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$69,Calendario!$E$3:$E$69,A4)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A4)</f>
         <v/>
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>Pago único, aplazado sin coste al 1 ene</t>
-        </is>
+          <t>4 × 537 €. Plan: aplazar la cuota de nov y liquidar todo el 29 nov por 1.500 €</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="n">
+        <v>648</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Smartcredito</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1329,71 +1396,77 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Santander</t>
+          <t>Smartcredito</t>
         </is>
       </c>
       <c r="D5" s="10" t="n">
-        <v>1994.93</v>
+        <v>435</v>
       </c>
       <c r="E5" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$E$3:$E$69,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A5)</f>
         <v/>
       </c>
       <c r="F5" s="3">
-        <f>D5-E5</f>
+        <f>D5-E5-I5</f>
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$69,Calendario!$E$3:$E$69,A5)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A5)</f>
         <v/>
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>96 €/mes; desde mar 2027 dentro de los 500 €/mes</t>
-        </is>
+          <t>Pago único, aplazado sin coste al 1 ene</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Pagolisto 1</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Pagolisto *6284</t>
+          <t>Santander</t>
         </is>
       </c>
       <c r="D6" s="10" t="n">
-        <v>693.34</v>
+        <v>1994.93</v>
       </c>
       <c r="E6" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$E$3:$E$69,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A6)</f>
         <v/>
       </c>
       <c r="F6" s="3">
-        <f>D6-E6</f>
+        <f>D6-E6-I6</f>
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$69,Calendario!$E$3:$E$69,A6)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A6)</f>
         <v/>
       </c>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>Aplazable sin coste; 3 cuotas dic–feb</t>
-        </is>
+          <t>96 €/mes; desde abr 2027 dentro de los 500 €/mes</t>
+        </is>
+      </c>
+      <c r="I6" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Pagolisto 2</t>
+          <t>Pagolisto 1</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -1403,34 +1476,37 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Pagolisto *6727</t>
+          <t>Pagolisto *6284</t>
         </is>
       </c>
       <c r="D7" s="10" t="n">
-        <v>923.61</v>
+        <v>693.34</v>
       </c>
       <c r="E7" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$E$3:$E$69,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A7)</f>
         <v/>
       </c>
       <c r="F7" s="3">
-        <f>D7-E7</f>
+        <f>D7-E7-I7</f>
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$69,Calendario!$E$3:$E$69,A7)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A7)</f>
         <v/>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Aplazable sin coste; 3 cuotas dic–feb</t>
-        </is>
+          <t>Aplazable sin coste; 3 cuotas ene–mar</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Crédito Santander 1</t>
+          <t>Pagolisto 2</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -1440,34 +1516,37 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Santander *0773</t>
+          <t>Pagolisto *6727</t>
         </is>
       </c>
       <c r="D8" s="10" t="n">
-        <v>1483.63</v>
+        <v>923.61</v>
       </c>
       <c r="E8" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$E$3:$E$69,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A8)</f>
         <v/>
       </c>
       <c r="F8" s="3">
-        <f>D8-E8</f>
+        <f>D8-E8-I8</f>
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$69,Calendario!$E$3:$E$69,A8)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A8)</f>
         <v/>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>Aplazable sin coste; 3 cuotas dic–feb</t>
-        </is>
+          <t>Aplazable sin coste; 3 cuotas ene–mar</t>
+        </is>
+      </c>
+      <c r="I8" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Crédito Santander 1</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -1477,71 +1556,77 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Santander *4475</t>
+          <t>Santander *0773</t>
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>2326.76</v>
+        <v>1483.63</v>
       </c>
       <c r="E9" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$E$3:$E$69,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A9)</f>
         <v/>
       </c>
       <c r="F9" s="3">
-        <f>D9-E9</f>
+        <f>D9-E9-I9</f>
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$69,Calendario!$E$3:$E$69,A9)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A9)</f>
         <v/>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>122,46 €/mes; desde mar 2027 dentro de los 500 €/mes</t>
-        </is>
+          <t>Aplazable sin coste; 3 cuotas ene–mar</t>
+        </is>
+      </c>
+      <c r="I9" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Ama</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>Amigo</t>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Ama</t>
+          <t>Santander *4475</t>
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>600</v>
+        <v>2326.76</v>
       </c>
       <c r="E10" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$E$3:$E$69,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A10)</f>
         <v/>
       </c>
       <c r="F10" s="3">
-        <f>D10-E10</f>
+        <f>D10-E10-I10</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$69,Calendario!$E$3:$E$69,A10)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A10)</f>
         <v/>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>Prioridad: 29 nov</t>
-        </is>
+          <t>122,46 €/mes; desde abr 2027 dentro de los 500 €/mes</t>
+        </is>
+      </c>
+      <c r="I10" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Joserra</t>
+          <t>Ama</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
@@ -1551,34 +1636,37 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Joserra</t>
+          <t>Ama</t>
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="E11" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$E$3:$E$69,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A11)</f>
         <v/>
       </c>
       <c r="F11" s="3">
-        <f>D11-E11</f>
+        <f>D11-E11-I11</f>
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$69,Calendario!$E$3:$E$69,A11)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A11)</f>
         <v/>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>Sin plazo ni interés</t>
-        </is>
+          <t>Prioridad: 1 nov, con lo que vuelves a pedir a Moneyman</t>
+        </is>
+      </c>
+      <c r="I11" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Xabi</t>
+          <t>Joserra</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
@@ -1588,34 +1676,37 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Xabi</t>
+          <t>Joserra</t>
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="E12" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$E$3:$E$69,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A12)</f>
         <v/>
       </c>
       <c r="F12" s="3">
-        <f>D12-E12</f>
+        <f>D12-E12-I12</f>
         <v/>
       </c>
       <c r="G12" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$69,Calendario!$E$3:$E$69,A12)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A12)</f>
         <v/>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
           <t>Sin plazo ni interés</t>
         </is>
+      </c>
+      <c r="I12" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Sergio</t>
+          <t>Xabi</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
@@ -1625,139 +1716,190 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Sergio</t>
+          <t>Xabi</t>
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>1700</v>
+        <v>300</v>
       </c>
       <c r="E13" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$E$3:$E$69,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A13)</f>
         <v/>
       </c>
       <c r="F13" s="3">
-        <f>D13-E13</f>
+        <f>D13-E13-I13</f>
         <v/>
       </c>
       <c r="G13" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$69,Calendario!$E$3:$E$69,A13)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A13)</f>
         <v/>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
           <t>Sin plazo ni interés</t>
         </is>
+      </c>
+      <c r="I13" s="10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
+          <t>Sergio</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
+          <t>Amigo</t>
+        </is>
+      </c>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>Sergio</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>1700</v>
+      </c>
+      <c r="E14" s="11">
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="3">
+        <f>D14-E14-I14</f>
+        <v/>
+      </c>
+      <c r="G14" s="12">
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="13" t="inlineStr">
+        <is>
+          <t>Sin plazo ni interés</t>
+        </is>
+      </c>
+      <c r="I14" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
           <t>Txomin</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>Amigo</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
         <is>
           <t>Txomin</t>
         </is>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="D15" s="10" t="n">
         <v>2500</v>
       </c>
-      <c r="E14" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$69,Calendario!$E$3:$E$69,A14)</f>
-        <v/>
-      </c>
-      <c r="F14" s="3">
-        <f>D14-E14</f>
-        <v/>
-      </c>
-      <c r="G14" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$69,Calendario!$E$3:$E$69,A14)</f>
-        <v/>
-      </c>
-      <c r="H14" s="13" t="inlineStr">
+      <c r="E15" s="11">
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="3">
+        <f>D15-E15-I15</f>
+        <v/>
+      </c>
+      <c r="G15" s="12">
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
         <is>
           <t>Sin plazo ni interés</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="I15" s="10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B15" s="17" t="n"/>
-      <c r="C15" s="17" t="n"/>
-      <c r="D15" s="6">
-        <f>SUM(D2:D14)</f>
-        <v/>
-      </c>
-      <c r="E15" s="6">
-        <f>SUM(E2:E14)</f>
-        <v/>
-      </c>
-      <c r="F15" s="6">
-        <f>SUM(F2:F14)</f>
-        <v/>
-      </c>
-      <c r="G15" s="18">
-        <f>MAX(G2:G14)</f>
-        <v/>
-      </c>
-      <c r="H15" s="19" t="inlineStr">
+      <c r="B16" s="17" t="n"/>
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="6">
+        <f>SUM(D2:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="6">
+        <f>SUM(E2:E15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="6">
+        <f>SUM(F2:F15)</f>
+        <v/>
+      </c>
+      <c r="G16" s="18">
+        <f>MAX(G2:G15)</f>
+        <v/>
+      </c>
+      <c r="H16" s="19" t="inlineStr">
         <is>
           <t>← libre de deudas</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="I16" s="6">
+        <f>SUM(I2:I15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Por bloque</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
       </c>
-      <c r="D18" s="3">
-        <f>SUMIFS(D2:D14,B2:B14,A18)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="D19" s="3">
+        <f>SUMIFS(D2:D15,B2:B15,A19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
-      <c r="D19" s="3">
-        <f>SUMIFS(D2:D14,B2:B14,A19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="D20" s="3">
+        <f>SUMIFS(D2:D15,B2:B15,A20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>Amigo</t>
         </is>
       </c>
-      <c r="D20" s="3">
-        <f>SUMIFS(D2:D14,B2:B14,A20)</f>
+      <c r="D21" s="3">
+        <f>SUMIFS(D2:D15,B2:B15,A21)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 
@@ -1767,7 +1909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1940,27 +2082,23 @@
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>Moneyman</t>
-        </is>
-      </c>
-      <c r="D5" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E5" s="27" t="inlineStr">
-        <is>
-          <t>Moneyman</t>
-        </is>
-      </c>
+          <t>Moneyman: vuelvo a pedir (recibo 1.100 €)</t>
+        </is>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr"/>
       <c r="F5" s="32" t="n">
-        <v>-1400</v>
+        <v>1100</v>
       </c>
       <c r="G5" s="30">
         <f>G4+F5</f>
         <v/>
       </c>
-      <c r="I5" s="34" t="inlineStr">
+      <c r="I5" s="33" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
@@ -1981,21 +2119,21 @@
       </c>
       <c r="C6" s="27" t="inlineStr">
         <is>
-          <t>Vivus · cuota 1/4</t>
-        </is>
-      </c>
-      <c r="D6" s="33" t="inlineStr">
+          <t>Moneyman</t>
+        </is>
+      </c>
+      <c r="D6" s="34" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
       </c>
       <c r="E6" s="27" t="inlineStr">
         <is>
-          <t>Vivus</t>
+          <t>Moneyman</t>
         </is>
       </c>
       <c r="F6" s="32" t="n">
-        <v>-537</v>
+        <v>-1400</v>
       </c>
       <c r="G6" s="30">
         <f>G5+F6</f>
@@ -2022,21 +2160,21 @@
       </c>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D7" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Devolución a Ama</t>
+        </is>
+      </c>
+      <c r="D7" s="36" t="inlineStr">
+        <is>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E7" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Ama</t>
         </is>
       </c>
       <c r="F7" s="32" t="n">
-        <v>-96</v>
+        <v>-600</v>
       </c>
       <c r="G7" s="30">
         <f>G6+F7</f>
@@ -2053,21 +2191,21 @@
       </c>
       <c r="C8" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
-        </is>
-      </c>
-      <c r="D8" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D8" s="34" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E8" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F8" s="32" t="n">
-        <v>-122.46</v>
+        <v>-96</v>
       </c>
       <c r="G8" s="30">
         <f>G7+F8</f>
@@ -2089,18 +2227,21 @@
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D9" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E9" s="27" t="inlineStr"/>
-      <c r="F9" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D9" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F9" s="32" t="n">
+        <v>-122.46</v>
       </c>
       <c r="G9" s="30">
         <f>G8+F9</f>
@@ -2109,7 +2250,7 @@
     </row>
     <row r="10">
       <c r="A10" s="25" t="n">
-        <v>46355</v>
+        <v>46327</v>
       </c>
       <c r="B10" s="26">
         <f>DATE(YEAR(A10),MONTH(A10),1)</f>
@@ -2117,17 +2258,18 @@
       </c>
       <c r="C10" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D10" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D10" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E10" s="27" t="inlineStr"/>
-      <c r="F10" s="32" t="n">
-        <v>3453.01</v>
+      <c r="F10" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G10" s="30">
         <f>G9+F10</f>
@@ -2144,21 +2286,17 @@
       </c>
       <c r="C11" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Ama</t>
-        </is>
-      </c>
-      <c r="D11" s="37" t="inlineStr">
-        <is>
-          <t>Amigo</t>
-        </is>
-      </c>
-      <c r="E11" s="27" t="inlineStr">
-        <is>
-          <t>Ama</t>
-        </is>
-      </c>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D11" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E11" s="27" t="inlineStr"/>
       <c r="F11" s="32" t="n">
-        <v>-600</v>
+        <v>3453.01</v>
       </c>
       <c r="G11" s="30">
         <f>G10+F11</f>
@@ -2167,7 +2305,7 @@
     </row>
     <row r="12">
       <c r="A12" s="25" t="n">
-        <v>46357</v>
+        <v>46355</v>
       </c>
       <c r="B12" s="26">
         <f>DATE(YEAR(A12),MONTH(A12),1)</f>
@@ -2175,12 +2313,12 @@
       </c>
       <c r="C12" s="27" t="inlineStr">
         <is>
-          <t>Vivus · cuota 2/4</t>
-        </is>
-      </c>
-      <c r="D12" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Vivus · liquidación total (en vez de 4 × 537 €)</t>
+        </is>
+      </c>
+      <c r="D12" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E12" s="27" t="inlineStr">
@@ -2189,7 +2327,7 @@
         </is>
       </c>
       <c r="F12" s="32" t="n">
-        <v>-537</v>
+        <v>-1500</v>
       </c>
       <c r="G12" s="30">
         <f>G11+F12</f>
@@ -2206,21 +2344,21 @@
       </c>
       <c r="C13" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D13" s="33" t="inlineStr">
+          <t>Moneyman (vuelto a pedir)</t>
+        </is>
+      </c>
+      <c r="D13" s="34" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
       </c>
       <c r="E13" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Moneyman (vuelto a pedir)</t>
         </is>
       </c>
       <c r="F13" s="32" t="n">
-        <v>-96</v>
+        <v>-1400</v>
       </c>
       <c r="G13" s="30">
         <f>G12+F13</f>
@@ -2237,21 +2375,21 @@
       </c>
       <c r="C14" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
-        </is>
-      </c>
-      <c r="D14" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D14" s="34" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E14" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F14" s="32" t="n">
-        <v>-122.46</v>
+        <v>-96</v>
       </c>
       <c r="G14" s="30">
         <f>G13+F14</f>
@@ -2268,21 +2406,21 @@
       </c>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 1/3</t>
-        </is>
-      </c>
-      <c r="D15" s="36" t="inlineStr">
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D15" s="37" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E15" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1</t>
+          <t>Crédito Santander 2</t>
         </is>
       </c>
       <c r="F15" s="32" t="n">
-        <v>-231.11</v>
+        <v>-122.46</v>
       </c>
       <c r="G15" s="30">
         <f>G14+F15</f>
@@ -2299,21 +2437,18 @@
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 1/3</t>
-        </is>
-      </c>
-      <c r="D16" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E16" s="27" t="inlineStr">
-        <is>
-          <t>Pagolisto 2</t>
-        </is>
-      </c>
-      <c r="F16" s="32" t="n">
-        <v>-307.87</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D16" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E16" s="27" t="inlineStr"/>
+      <c r="F16" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G16" s="30">
         <f>G15+F16</f>
@@ -2322,7 +2457,7 @@
     </row>
     <row r="17">
       <c r="A17" s="25" t="n">
-        <v>46357</v>
+        <v>46385</v>
       </c>
       <c r="B17" s="26">
         <f>DATE(YEAR(A17),MONTH(A17),1)</f>
@@ -2330,21 +2465,17 @@
       </c>
       <c r="C17" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 1/3</t>
-        </is>
-      </c>
-      <c r="D17" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E17" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 1</t>
-        </is>
-      </c>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D17" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E17" s="27" t="inlineStr"/>
       <c r="F17" s="32" t="n">
-        <v>-494.54</v>
+        <v>3453.01</v>
       </c>
       <c r="G17" s="30">
         <f>G16+F17</f>
@@ -2353,7 +2484,7 @@
     </row>
     <row r="18">
       <c r="A18" s="25" t="n">
-        <v>46357</v>
+        <v>46385</v>
       </c>
       <c r="B18" s="26">
         <f>DATE(YEAR(A18),MONTH(A18),1)</f>
@@ -2361,18 +2492,17 @@
       </c>
       <c r="C18" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D18" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Paga extra de diciembre</t>
+        </is>
+      </c>
+      <c r="D18" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E18" s="27" t="inlineStr"/>
-      <c r="F18" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F18" s="32" t="n">
+        <v>2014.69</v>
       </c>
       <c r="G18" s="30">
         <f>G17+F18</f>
@@ -2381,7 +2511,7 @@
     </row>
     <row r="19">
       <c r="A19" s="25" t="n">
-        <v>46385</v>
+        <v>46388</v>
       </c>
       <c r="B19" s="26">
         <f>DATE(YEAR(A19),MONTH(A19),1)</f>
@@ -2389,17 +2519,21 @@
       </c>
       <c r="C19" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D19" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E19" s="27" t="inlineStr"/>
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D19" s="34" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E19" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
       <c r="F19" s="32" t="n">
-        <v>3453.01</v>
+        <v>-96</v>
       </c>
       <c r="G19" s="30">
         <f>G18+F19</f>
@@ -2408,7 +2542,7 @@
     </row>
     <row r="20">
       <c r="A20" s="25" t="n">
-        <v>46385</v>
+        <v>46388</v>
       </c>
       <c r="B20" s="26">
         <f>DATE(YEAR(A20),MONTH(A20),1)</f>
@@ -2416,17 +2550,21 @@
       </c>
       <c r="C20" s="27" t="inlineStr">
         <is>
-          <t>Paga extra de diciembre</t>
-        </is>
-      </c>
-      <c r="D20" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E20" s="27" t="inlineStr"/>
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D20" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
       <c r="F20" s="32" t="n">
-        <v>2014.69</v>
+        <v>-122.46</v>
       </c>
       <c r="G20" s="30">
         <f>G19+F20</f>
@@ -2443,21 +2581,21 @@
       </c>
       <c r="C21" s="27" t="inlineStr">
         <is>
-          <t>Vivus · cuota 3/4</t>
-        </is>
-      </c>
-      <c r="D21" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Pagolisto 1 · cuota 1/3</t>
+        </is>
+      </c>
+      <c r="D21" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E21" s="27" t="inlineStr">
         <is>
-          <t>Vivus</t>
+          <t>Pagolisto 1</t>
         </is>
       </c>
       <c r="F21" s="32" t="n">
-        <v>-537</v>
+        <v>-231.11</v>
       </c>
       <c r="G21" s="30">
         <f>G20+F21</f>
@@ -2474,21 +2612,21 @@
       </c>
       <c r="C22" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D22" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Pagolisto 2 · cuota 1/3</t>
+        </is>
+      </c>
+      <c r="D22" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E22" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Pagolisto 2</t>
         </is>
       </c>
       <c r="F22" s="32" t="n">
-        <v>-96</v>
+        <v>-307.87</v>
       </c>
       <c r="G22" s="30">
         <f>G21+F22</f>
@@ -2505,21 +2643,21 @@
       </c>
       <c r="C23" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
-        </is>
-      </c>
-      <c r="D23" s="36" t="inlineStr">
+          <t>Crédito Santander 1 · cuota 1/3</t>
+        </is>
+      </c>
+      <c r="D23" s="37" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E23" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Crédito Santander 1</t>
         </is>
       </c>
       <c r="F23" s="32" t="n">
-        <v>-122.46</v>
+        <v>-494.54</v>
       </c>
       <c r="G23" s="30">
         <f>G22+F23</f>
@@ -2536,21 +2674,21 @@
       </c>
       <c r="C24" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 2/3</t>
-        </is>
-      </c>
-      <c r="D24" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Smartcredito</t>
+        </is>
+      </c>
+      <c r="D24" s="34" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E24" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1</t>
+          <t>Smartcredito</t>
         </is>
       </c>
       <c r="F24" s="32" t="n">
-        <v>-231.11</v>
+        <v>-435</v>
       </c>
       <c r="G24" s="30">
         <f>G23+F24</f>
@@ -2567,21 +2705,21 @@
       </c>
       <c r="C25" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 2/3</t>
+          <t>Devolución a Joserra</t>
         </is>
       </c>
       <c r="D25" s="36" t="inlineStr">
         <is>
-          <t>Aplazable</t>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E25" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2</t>
+          <t>Joserra</t>
         </is>
       </c>
       <c r="F25" s="32" t="n">
-        <v>-307.87</v>
+        <v>-400</v>
       </c>
       <c r="G25" s="30">
         <f>G24+F25</f>
@@ -2598,21 +2736,21 @@
       </c>
       <c r="C26" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 2/3</t>
+          <t>Devolución a Xabi</t>
         </is>
       </c>
       <c r="D26" s="36" t="inlineStr">
         <is>
-          <t>Aplazable</t>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E26" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1</t>
+          <t>Xabi</t>
         </is>
       </c>
       <c r="F26" s="32" t="n">
-        <v>-494.54</v>
+        <v>-300</v>
       </c>
       <c r="G26" s="30">
         <f>G25+F26</f>
@@ -2629,21 +2767,18 @@
       </c>
       <c r="C27" s="27" t="inlineStr">
         <is>
-          <t>Smartcredito</t>
-        </is>
-      </c>
-      <c r="D27" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E27" s="27" t="inlineStr">
-        <is>
-          <t>Smartcredito</t>
-        </is>
-      </c>
-      <c r="F27" s="32" t="n">
-        <v>-435</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D27" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E27" s="27" t="inlineStr"/>
+      <c r="F27" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G27" s="30">
         <f>G26+F27</f>
@@ -2652,7 +2787,7 @@
     </row>
     <row r="28">
       <c r="A28" s="25" t="n">
-        <v>46388</v>
+        <v>46416</v>
       </c>
       <c r="B28" s="26">
         <f>DATE(YEAR(A28),MONTH(A28),1)</f>
@@ -2660,21 +2795,17 @@
       </c>
       <c r="C28" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Joserra</t>
-        </is>
-      </c>
-      <c r="D28" s="37" t="inlineStr">
-        <is>
-          <t>Amigo</t>
-        </is>
-      </c>
-      <c r="E28" s="27" t="inlineStr">
-        <is>
-          <t>Joserra</t>
-        </is>
-      </c>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D28" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E28" s="27" t="inlineStr"/>
       <c r="F28" s="32" t="n">
-        <v>-400</v>
+        <v>3173.56</v>
       </c>
       <c r="G28" s="30">
         <f>G27+F28</f>
@@ -2683,7 +2814,7 @@
     </row>
     <row r="29">
       <c r="A29" s="25" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="B29" s="26">
         <f>DATE(YEAR(A29),MONTH(A29),1)</f>
@@ -2691,21 +2822,21 @@
       </c>
       <c r="C29" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Xabi</t>
-        </is>
-      </c>
-      <c r="D29" s="37" t="inlineStr">
-        <is>
-          <t>Amigo</t>
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D29" s="34" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E29" s="27" t="inlineStr">
         <is>
-          <t>Xabi</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F29" s="32" t="n">
-        <v>-300</v>
+        <v>-96</v>
       </c>
       <c r="G29" s="30">
         <f>G28+F29</f>
@@ -2714,7 +2845,7 @@
     </row>
     <row r="30">
       <c r="A30" s="25" t="n">
-        <v>46388</v>
+        <v>46419</v>
       </c>
       <c r="B30" s="26">
         <f>DATE(YEAR(A30),MONTH(A30),1)</f>
@@ -2722,18 +2853,21 @@
       </c>
       <c r="C30" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D30" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E30" s="27" t="inlineStr"/>
-      <c r="F30" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D30" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E30" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F30" s="32" t="n">
+        <v>-122.46</v>
       </c>
       <c r="G30" s="30">
         <f>G29+F30</f>
@@ -2742,7 +2876,7 @@
     </row>
     <row r="31">
       <c r="A31" s="25" t="n">
-        <v>46416</v>
+        <v>46419</v>
       </c>
       <c r="B31" s="26">
         <f>DATE(YEAR(A31),MONTH(A31),1)</f>
@@ -2750,17 +2884,21 @@
       </c>
       <c r="C31" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D31" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E31" s="27" t="inlineStr"/>
+          <t>Pagolisto 1 · cuota 2/3</t>
+        </is>
+      </c>
+      <c r="D31" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E31" s="27" t="inlineStr">
+        <is>
+          <t>Pagolisto 1</t>
+        </is>
+      </c>
       <c r="F31" s="32" t="n">
-        <v>3173.56</v>
+        <v>-231.11</v>
       </c>
       <c r="G31" s="30">
         <f>G30+F31</f>
@@ -2777,21 +2915,21 @@
       </c>
       <c r="C32" s="27" t="inlineStr">
         <is>
-          <t>Vivus · cuota 4/4</t>
-        </is>
-      </c>
-      <c r="D32" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Pagolisto 2 · cuota 2/3</t>
+        </is>
+      </c>
+      <c r="D32" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E32" s="27" t="inlineStr">
         <is>
-          <t>Vivus</t>
+          <t>Pagolisto 2</t>
         </is>
       </c>
       <c r="F32" s="32" t="n">
-        <v>-537</v>
+        <v>-307.87</v>
       </c>
       <c r="G32" s="30">
         <f>G31+F32</f>
@@ -2808,21 +2946,21 @@
       </c>
       <c r="C33" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D33" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 1 · cuota 2/3</t>
+        </is>
+      </c>
+      <c r="D33" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E33" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Crédito Santander 1</t>
         </is>
       </c>
       <c r="F33" s="32" t="n">
-        <v>-96</v>
+        <v>-494.54</v>
       </c>
       <c r="G33" s="30">
         <f>G32+F33</f>
@@ -2839,21 +2977,21 @@
       </c>
       <c r="C34" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
+          <t>Devolución a Sergio</t>
         </is>
       </c>
       <c r="D34" s="36" t="inlineStr">
         <is>
-          <t>Aplazable</t>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E34" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Sergio</t>
         </is>
       </c>
       <c r="F34" s="32" t="n">
-        <v>-122.46</v>
+        <v>-1700</v>
       </c>
       <c r="G34" s="30">
         <f>G33+F34</f>
@@ -2870,21 +3008,18 @@
       </c>
       <c r="C35" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 3/3</t>
-        </is>
-      </c>
-      <c r="D35" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E35" s="27" t="inlineStr">
-        <is>
-          <t>Pagolisto 1</t>
-        </is>
-      </c>
-      <c r="F35" s="32" t="n">
-        <v>-231.12</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D35" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E35" s="27" t="inlineStr"/>
+      <c r="F35" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G35" s="30">
         <f>G34+F35</f>
@@ -2893,7 +3028,7 @@
     </row>
     <row r="36">
       <c r="A36" s="25" t="n">
-        <v>46419</v>
+        <v>46446</v>
       </c>
       <c r="B36" s="26">
         <f>DATE(YEAR(A36),MONTH(A36),1)</f>
@@ -2901,21 +3036,17 @@
       </c>
       <c r="C36" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 3/3</t>
-        </is>
-      </c>
-      <c r="D36" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E36" s="27" t="inlineStr">
-        <is>
-          <t>Pagolisto 2</t>
-        </is>
-      </c>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D36" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E36" s="27" t="inlineStr"/>
       <c r="F36" s="32" t="n">
-        <v>-307.87</v>
+        <v>3173.56</v>
       </c>
       <c r="G36" s="30">
         <f>G35+F36</f>
@@ -2924,7 +3055,7 @@
     </row>
     <row r="37">
       <c r="A37" s="25" t="n">
-        <v>46419</v>
+        <v>46446</v>
       </c>
       <c r="B37" s="26">
         <f>DATE(YEAR(A37),MONTH(A37),1)</f>
@@ -2932,21 +3063,17 @@
       </c>
       <c r="C37" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 3/3</t>
-        </is>
-      </c>
-      <c r="D37" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E37" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 1</t>
-        </is>
-      </c>
+          <t>Variable de febrero</t>
+        </is>
+      </c>
+      <c r="D37" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E37" s="27" t="inlineStr"/>
       <c r="F37" s="32" t="n">
-        <v>-494.55</v>
+        <v>2114.45</v>
       </c>
       <c r="G37" s="30">
         <f>G36+F37</f>
@@ -2955,7 +3082,7 @@
     </row>
     <row r="38">
       <c r="A38" s="25" t="n">
-        <v>46419</v>
+        <v>46446</v>
       </c>
       <c r="B38" s="26">
         <f>DATE(YEAR(A38),MONTH(A38),1)</f>
@@ -2963,21 +3090,21 @@
       </c>
       <c r="C38" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Sergio</t>
-        </is>
-      </c>
-      <c r="D38" s="37" t="inlineStr">
+          <t>Devolución a Txomin</t>
+        </is>
+      </c>
+      <c r="D38" s="36" t="inlineStr">
         <is>
           <t>Amigo</t>
         </is>
       </c>
       <c r="E38" s="27" t="inlineStr">
         <is>
-          <t>Sergio</t>
+          <t>Txomin</t>
         </is>
       </c>
       <c r="F38" s="32" t="n">
-        <v>-1700</v>
+        <v>-2500</v>
       </c>
       <c r="G38" s="30">
         <f>G37+F38</f>
@@ -2986,7 +3113,7 @@
     </row>
     <row r="39">
       <c r="A39" s="25" t="n">
-        <v>46419</v>
+        <v>46447</v>
       </c>
       <c r="B39" s="26">
         <f>DATE(YEAR(A39),MONTH(A39),1)</f>
@@ -2994,18 +3121,21 @@
       </c>
       <c r="C39" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D39" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E39" s="27" t="inlineStr"/>
-      <c r="F39" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D39" s="34" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E39" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F39" s="32" t="n">
+        <v>-96</v>
       </c>
       <c r="G39" s="30">
         <f>G38+F39</f>
@@ -3014,7 +3144,7 @@
     </row>
     <row r="40">
       <c r="A40" s="25" t="n">
-        <v>46446</v>
+        <v>46447</v>
       </c>
       <c r="B40" s="26">
         <f>DATE(YEAR(A40),MONTH(A40),1)</f>
@@ -3022,17 +3152,21 @@
       </c>
       <c r="C40" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D40" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E40" s="27" t="inlineStr"/>
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D40" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E40" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
       <c r="F40" s="32" t="n">
-        <v>3173.56</v>
+        <v>-122.46</v>
       </c>
       <c r="G40" s="30">
         <f>G39+F40</f>
@@ -3041,7 +3175,7 @@
     </row>
     <row r="41">
       <c r="A41" s="25" t="n">
-        <v>46446</v>
+        <v>46447</v>
       </c>
       <c r="B41" s="26">
         <f>DATE(YEAR(A41),MONTH(A41),1)</f>
@@ -3049,17 +3183,21 @@
       </c>
       <c r="C41" s="27" t="inlineStr">
         <is>
-          <t>Variable de febrero</t>
-        </is>
-      </c>
-      <c r="D41" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E41" s="27" t="inlineStr"/>
+          <t>Pagolisto 1 · cuota 3/3</t>
+        </is>
+      </c>
+      <c r="D41" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E41" s="27" t="inlineStr">
+        <is>
+          <t>Pagolisto 1</t>
+        </is>
+      </c>
       <c r="F41" s="32" t="n">
-        <v>2114.45</v>
+        <v>-231.12</v>
       </c>
       <c r="G41" s="30">
         <f>G40+F41</f>
@@ -3068,7 +3206,7 @@
     </row>
     <row r="42">
       <c r="A42" s="25" t="n">
-        <v>46446</v>
+        <v>46447</v>
       </c>
       <c r="B42" s="26">
         <f>DATE(YEAR(A42),MONTH(A42),1)</f>
@@ -3076,21 +3214,21 @@
       </c>
       <c r="C42" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Txomin</t>
+          <t>Pagolisto 2 · cuota 3/3</t>
         </is>
       </c>
       <c r="D42" s="37" t="inlineStr">
         <is>
-          <t>Amigo</t>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E42" s="27" t="inlineStr">
         <is>
-          <t>Txomin</t>
+          <t>Pagolisto 2</t>
         </is>
       </c>
       <c r="F42" s="32" t="n">
-        <v>-2500</v>
+        <v>-307.87</v>
       </c>
       <c r="G42" s="30">
         <f>G41+F42</f>
@@ -3107,21 +3245,21 @@
       </c>
       <c r="C43" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D43" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 1 · cuota 3/3</t>
+        </is>
+      </c>
+      <c r="D43" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E43" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Crédito Santander 1</t>
         </is>
       </c>
       <c r="F43" s="32" t="n">
-        <v>-96</v>
+        <v>-494.55</v>
       </c>
       <c r="G43" s="30">
         <f>G42+F43</f>
@@ -3138,21 +3276,18 @@
       </c>
       <c r="C44" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D44" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E44" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F44" s="32" t="n">
-        <v>-404</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D44" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E44" s="27" t="inlineStr"/>
+      <c r="F44" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G44" s="30">
         <f>G43+F44</f>
@@ -3161,7 +3296,7 @@
     </row>
     <row r="45">
       <c r="A45" s="25" t="n">
-        <v>46447</v>
+        <v>46475</v>
       </c>
       <c r="B45" s="26">
         <f>DATE(YEAR(A45),MONTH(A45),1)</f>
@@ -3169,18 +3304,17 @@
       </c>
       <c r="C45" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D45" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D45" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E45" s="27" t="inlineStr"/>
-      <c r="F45" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F45" s="32" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G45" s="30">
         <f>G44+F45</f>
@@ -3189,7 +3323,7 @@
     </row>
     <row r="46">
       <c r="A46" s="25" t="n">
-        <v>46475</v>
+        <v>46478</v>
       </c>
       <c r="B46" s="26">
         <f>DATE(YEAR(A46),MONTH(A46),1)</f>
@@ -3197,17 +3331,21 @@
       </c>
       <c r="C46" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D46" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E46" s="27" t="inlineStr"/>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D46" s="34" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E46" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
       <c r="F46" s="32" t="n">
-        <v>3173.56</v>
+        <v>-96</v>
       </c>
       <c r="G46" s="30">
         <f>G45+F46</f>
@@ -3224,21 +3362,21 @@
       </c>
       <c r="C47" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D47" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D47" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E47" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Crédito Santander 2</t>
         </is>
       </c>
       <c r="F47" s="32" t="n">
-        <v>-96</v>
+        <v>-404</v>
       </c>
       <c r="G47" s="30">
         <f>G46+F47</f>
@@ -3255,21 +3393,18 @@
       </c>
       <c r="C48" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D48" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E48" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F48" s="32" t="n">
-        <v>-404</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D48" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E48" s="27" t="inlineStr"/>
+      <c r="F48" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G48" s="30">
         <f>G47+F48</f>
@@ -3278,7 +3413,7 @@
     </row>
     <row r="49">
       <c r="A49" s="25" t="n">
-        <v>46478</v>
+        <v>46506</v>
       </c>
       <c r="B49" s="26">
         <f>DATE(YEAR(A49),MONTH(A49),1)</f>
@@ -3286,18 +3421,17 @@
       </c>
       <c r="C49" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D49" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D49" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E49" s="27" t="inlineStr"/>
-      <c r="F49" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F49" s="32" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G49" s="30">
         <f>G48+F49</f>
@@ -3306,7 +3440,7 @@
     </row>
     <row r="50">
       <c r="A50" s="25" t="n">
-        <v>46506</v>
+        <v>46508</v>
       </c>
       <c r="B50" s="26">
         <f>DATE(YEAR(A50),MONTH(A50),1)</f>
@@ -3314,17 +3448,21 @@
       </c>
       <c r="C50" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D50" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E50" s="27" t="inlineStr"/>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D50" s="34" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E50" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
       <c r="F50" s="32" t="n">
-        <v>3173.56</v>
+        <v>-96</v>
       </c>
       <c r="G50" s="30">
         <f>G49+F50</f>
@@ -3341,21 +3479,21 @@
       </c>
       <c r="C51" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D51" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D51" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E51" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Crédito Santander 2</t>
         </is>
       </c>
       <c r="F51" s="32" t="n">
-        <v>-96</v>
+        <v>-404</v>
       </c>
       <c r="G51" s="30">
         <f>G50+F51</f>
@@ -3372,21 +3510,18 @@
       </c>
       <c r="C52" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D52" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E52" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F52" s="32" t="n">
-        <v>-404</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D52" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E52" s="27" t="inlineStr"/>
+      <c r="F52" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G52" s="30">
         <f>G51+F52</f>
@@ -3395,7 +3530,7 @@
     </row>
     <row r="53">
       <c r="A53" s="25" t="n">
-        <v>46508</v>
+        <v>46536</v>
       </c>
       <c r="B53" s="26">
         <f>DATE(YEAR(A53),MONTH(A53),1)</f>
@@ -3403,18 +3538,17 @@
       </c>
       <c r="C53" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D53" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D53" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E53" s="27" t="inlineStr"/>
-      <c r="F53" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F53" s="32" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G53" s="30">
         <f>G52+F53</f>
@@ -3423,7 +3557,7 @@
     </row>
     <row r="54">
       <c r="A54" s="25" t="n">
-        <v>46536</v>
+        <v>46539</v>
       </c>
       <c r="B54" s="26">
         <f>DATE(YEAR(A54),MONTH(A54),1)</f>
@@ -3431,17 +3565,21 @@
       </c>
       <c r="C54" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D54" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E54" s="27" t="inlineStr"/>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D54" s="34" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E54" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
       <c r="F54" s="32" t="n">
-        <v>3173.56</v>
+        <v>-96</v>
       </c>
       <c r="G54" s="30">
         <f>G53+F54</f>
@@ -3458,21 +3596,21 @@
       </c>
       <c r="C55" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D55" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D55" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E55" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Crédito Santander 2</t>
         </is>
       </c>
       <c r="F55" s="32" t="n">
-        <v>-96</v>
+        <v>-404</v>
       </c>
       <c r="G55" s="30">
         <f>G54+F55</f>
@@ -3489,21 +3627,18 @@
       </c>
       <c r="C56" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D56" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E56" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F56" s="32" t="n">
-        <v>-404</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D56" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E56" s="27" t="inlineStr"/>
+      <c r="F56" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G56" s="30">
         <f>G55+F56</f>
@@ -3512,7 +3647,7 @@
     </row>
     <row r="57">
       <c r="A57" s="25" t="n">
-        <v>46539</v>
+        <v>46567</v>
       </c>
       <c r="B57" s="26">
         <f>DATE(YEAR(A57),MONTH(A57),1)</f>
@@ -3520,18 +3655,17 @@
       </c>
       <c r="C57" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D57" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D57" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E57" s="27" t="inlineStr"/>
-      <c r="F57" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F57" s="32" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G57" s="30">
         <f>G56+F57</f>
@@ -3548,7 +3682,7 @@
       </c>
       <c r="C58" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
+          <t>Paga extra de junio</t>
         </is>
       </c>
       <c r="D58" s="31" t="inlineStr">
@@ -3558,7 +3692,7 @@
       </c>
       <c r="E58" s="27" t="inlineStr"/>
       <c r="F58" s="32" t="n">
-        <v>3173.56</v>
+        <v>1989.05</v>
       </c>
       <c r="G58" s="30">
         <f>G57+F58</f>
@@ -3567,7 +3701,7 @@
     </row>
     <row r="59">
       <c r="A59" s="25" t="n">
-        <v>46567</v>
+        <v>46569</v>
       </c>
       <c r="B59" s="26">
         <f>DATE(YEAR(A59),MONTH(A59),1)</f>
@@ -3575,17 +3709,21 @@
       </c>
       <c r="C59" s="27" t="inlineStr">
         <is>
-          <t>Paga extra de junio</t>
-        </is>
-      </c>
-      <c r="D59" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E59" s="27" t="inlineStr"/>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D59" s="34" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E59" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
       <c r="F59" s="32" t="n">
-        <v>1989.05</v>
+        <v>-96</v>
       </c>
       <c r="G59" s="30">
         <f>G58+F59</f>
@@ -3602,21 +3740,21 @@
       </c>
       <c r="C60" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D60" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D60" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E60" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Crédito Santander 2</t>
         </is>
       </c>
       <c r="F60" s="32" t="n">
-        <v>-279.08</v>
+        <v>-404</v>
       </c>
       <c r="G60" s="30">
         <f>G59+F60</f>
@@ -3633,21 +3771,18 @@
       </c>
       <c r="C61" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D61" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E61" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F61" s="32" t="n">
-        <v>-220.92</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D61" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E61" s="27" t="inlineStr"/>
+      <c r="F61" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G61" s="30">
         <f>G60+F61</f>
@@ -3656,7 +3791,7 @@
     </row>
     <row r="62">
       <c r="A62" s="25" t="n">
-        <v>46569</v>
+        <v>46597</v>
       </c>
       <c r="B62" s="26">
         <f>DATE(YEAR(A62),MONTH(A62),1)</f>
@@ -3664,18 +3799,17 @@
       </c>
       <c r="C62" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D62" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D62" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E62" s="27" t="inlineStr"/>
-      <c r="F62" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F62" s="32" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G62" s="30">
         <f>G61+F62</f>
@@ -3684,7 +3818,7 @@
     </row>
     <row r="63">
       <c r="A63" s="25" t="n">
-        <v>46597</v>
+        <v>46600</v>
       </c>
       <c r="B63" s="26">
         <f>DATE(YEAR(A63),MONTH(A63),1)</f>
@@ -3692,17 +3826,21 @@
       </c>
       <c r="C63" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D63" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E63" s="27" t="inlineStr"/>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D63" s="34" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E63" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
       <c r="F63" s="32" t="n">
-        <v>3173.56</v>
+        <v>-401.54</v>
       </c>
       <c r="G63" s="30">
         <f>G62+F63</f>
@@ -3719,21 +3857,21 @@
       </c>
       <c r="C64" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D64" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D64" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E64" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Crédito Santander 2</t>
         </is>
       </c>
       <c r="F64" s="32" t="n">
-        <v>-500</v>
+        <v>-98.45999999999999</v>
       </c>
       <c r="G64" s="30">
         <f>G63+F64</f>
@@ -3808,7 +3946,7 @@
           <t>Santander (préstamo) · plan 500 €/mes</t>
         </is>
       </c>
-      <c r="D67" s="33" t="inlineStr">
+      <c r="D67" s="34" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
@@ -3819,7 +3957,7 @@
         </is>
       </c>
       <c r="F67" s="32" t="n">
-        <v>-447.85</v>
+        <v>-500</v>
       </c>
       <c r="G67" s="30">
         <f>G66+F67</f>
@@ -3881,9 +4019,95 @@
         <v/>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" s="25" t="n">
+        <v>46661</v>
+      </c>
+      <c r="B70" s="26">
+        <f>DATE(YEAR(A70),MONTH(A70),1)</f>
+        <v/>
+      </c>
+      <c r="C70" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D70" s="34" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E70" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F70" s="32" t="n">
+        <v>-229.39</v>
+      </c>
+      <c r="G70" s="30">
+        <f>G69+F70</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="25" t="n">
+        <v>46661</v>
+      </c>
+      <c r="B71" s="26">
+        <f>DATE(YEAR(A71),MONTH(A71),1)</f>
+        <v/>
+      </c>
+      <c r="C71" s="27" t="inlineStr">
+        <is>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D71" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E71" s="27" t="inlineStr"/>
+      <c r="F71" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
+      </c>
+      <c r="G71" s="30">
+        <f>G70+F71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="25" t="n">
+        <v>46689</v>
+      </c>
+      <c r="B72" s="26">
+        <f>DATE(YEAR(A72),MONTH(A72),1)</f>
+        <v/>
+      </c>
+      <c r="C72" s="27" t="inlineStr">
+        <is>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D72" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E72" s="27" t="inlineStr"/>
+      <c r="F72" s="32" t="n">
+        <v>2490.44</v>
+      </c>
+      <c r="G72" s="30">
+        <f>G71+F72</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G69"/>
-  <conditionalFormatting sqref="G2:G69">
+  <autoFilter ref="A1:G72"/>
+  <conditionalFormatting sqref="G2:G72">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="1">
       <formula>0</formula>
     </cfRule>
@@ -3898,7 +4122,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -3983,7 +4207,7 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Pago mensual al bloque Santander desde mar 2027 (€)</t>
+          <t>Pago mensual al bloque Santander desde abr 2027 (€)</t>
         </is>
       </c>
       <c r="B8" s="41" t="n">
@@ -4013,6 +4237,13 @@
       <c r="A12" s="13" t="inlineStr">
         <is>
           <t>Aplazables sin coste: Pagolisto 1 y 2, Crédito Santander 1 y 2, Smartcredito y Vivus. No aplazables: Santander (préstamo) y Moneyman.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Escenario: el 1 nov pagas Moneyman y lo vuelves a pedir (1.100 €) para pagar a Ama; el 29 nov liquidas Vivus por 1.500 €.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan: Smartcredito se paga hoy, Vivus no se aplaza y los aplazables se pagan y se vuelven a pedir
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JEd5Mo2HQL6TrpXUCZoFXP
</commit_message>
<xml_diff>
--- a/excel/plan_de_pagos.xlsx
+++ b/excel/plan_de_pagos.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Supuestos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Calendario'!$A$1:$G$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Calendario'!$A$1:$G$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -95,17 +95,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FDE2E2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DCFCE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FDE2E2"/>
       </patternFill>
     </fill>
     <fill>
@@ -150,7 +150,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -173,13 +173,13 @@
     <xf numFmtId="167" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -653,23 +653,23 @@
         <v>46296</v>
       </c>
       <c r="B2" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A2)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A2)</f>
         <v/>
       </c>
       <c r="C2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A2)</f>
         <v/>
       </c>
       <c r="D2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A2)</f>
         <v/>
       </c>
       <c r="E2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A2)</f>
         <v/>
       </c>
       <c r="F2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A2)</f>
         <v/>
       </c>
       <c r="G2" s="3">
@@ -690,23 +690,23 @@
         <v>46327</v>
       </c>
       <c r="B3" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A3)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A3)</f>
         <v/>
       </c>
       <c r="C3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A3)</f>
         <v/>
       </c>
       <c r="D3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A3)</f>
         <v/>
       </c>
       <c r="E3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A3)</f>
         <v/>
       </c>
       <c r="F3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A3)</f>
         <v/>
       </c>
       <c r="G3" s="3">
@@ -727,23 +727,23 @@
         <v>46357</v>
       </c>
       <c r="B4" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A4)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A4)</f>
         <v/>
       </c>
       <c r="C4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A4)</f>
         <v/>
       </c>
       <c r="D4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A4)</f>
         <v/>
       </c>
       <c r="E4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A4)</f>
         <v/>
       </c>
       <c r="F4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A4)</f>
         <v/>
       </c>
       <c r="G4" s="3">
@@ -764,23 +764,23 @@
         <v>46388</v>
       </c>
       <c r="B5" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A5)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A5)</f>
         <v/>
       </c>
       <c r="C5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A5)</f>
         <v/>
       </c>
       <c r="D5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A5)</f>
         <v/>
       </c>
       <c r="E5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A5)</f>
         <v/>
       </c>
       <c r="F5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A5)</f>
         <v/>
       </c>
       <c r="G5" s="3">
@@ -801,23 +801,23 @@
         <v>46419</v>
       </c>
       <c r="B6" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A6)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A6)</f>
         <v/>
       </c>
       <c r="C6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A6)</f>
         <v/>
       </c>
       <c r="D6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A6)</f>
         <v/>
       </c>
       <c r="E6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A6)</f>
         <v/>
       </c>
       <c r="F6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A6)</f>
         <v/>
       </c>
       <c r="G6" s="3">
@@ -838,23 +838,23 @@
         <v>46447</v>
       </c>
       <c r="B7" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A7)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A7)</f>
         <v/>
       </c>
       <c r="C7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A7)</f>
         <v/>
       </c>
       <c r="D7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A7)</f>
         <v/>
       </c>
       <c r="E7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A7)</f>
         <v/>
       </c>
       <c r="F7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A7)</f>
         <v/>
       </c>
       <c r="G7" s="3">
@@ -875,23 +875,23 @@
         <v>46478</v>
       </c>
       <c r="B8" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A8)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A8)</f>
         <v/>
       </c>
       <c r="C8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A8)</f>
         <v/>
       </c>
       <c r="D8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A8)</f>
         <v/>
       </c>
       <c r="E8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A8)</f>
         <v/>
       </c>
       <c r="F8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A8)</f>
         <v/>
       </c>
       <c r="G8" s="3">
@@ -912,23 +912,23 @@
         <v>46508</v>
       </c>
       <c r="B9" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A9)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A9)</f>
         <v/>
       </c>
       <c r="C9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A9)</f>
         <v/>
       </c>
       <c r="D9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A9)</f>
         <v/>
       </c>
       <c r="E9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A9)</f>
         <v/>
       </c>
       <c r="F9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A9)</f>
         <v/>
       </c>
       <c r="G9" s="3">
@@ -949,23 +949,23 @@
         <v>46539</v>
       </c>
       <c r="B10" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A10)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A10)</f>
         <v/>
       </c>
       <c r="C10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A10)</f>
         <v/>
       </c>
       <c r="D10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A10)</f>
         <v/>
       </c>
       <c r="E10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A10)</f>
         <v/>
       </c>
       <c r="F10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A10)</f>
         <v/>
       </c>
       <c r="G10" s="3">
@@ -986,23 +986,23 @@
         <v>46569</v>
       </c>
       <c r="B11" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A11)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A11)</f>
         <v/>
       </c>
       <c r="C11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A11)</f>
         <v/>
       </c>
       <c r="D11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A11)</f>
         <v/>
       </c>
       <c r="E11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A11)</f>
         <v/>
       </c>
       <c r="F11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A11)</f>
         <v/>
       </c>
       <c r="G11" s="3">
@@ -1023,23 +1023,23 @@
         <v>46600</v>
       </c>
       <c r="B12" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A12)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A12)</f>
         <v/>
       </c>
       <c r="C12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A12)</f>
         <v/>
       </c>
       <c r="D12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A12)</f>
         <v/>
       </c>
       <c r="E12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A12)</f>
         <v/>
       </c>
       <c r="F12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A12)</f>
         <v/>
       </c>
       <c r="G12" s="3">
@@ -1060,23 +1060,23 @@
         <v>46631</v>
       </c>
       <c r="B13" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A13)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A13)</f>
         <v/>
       </c>
       <c r="C13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A13)</f>
         <v/>
       </c>
       <c r="D13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A13)</f>
         <v/>
       </c>
       <c r="E13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A13)</f>
         <v/>
       </c>
       <c r="F13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A13)</f>
         <v/>
       </c>
       <c r="G13" s="3">
@@ -1097,23 +1097,23 @@
         <v>46661</v>
       </c>
       <c r="B14" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A14)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A14)</f>
         <v/>
       </c>
       <c r="C14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A14)</f>
         <v/>
       </c>
       <c r="D14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A14)</f>
         <v/>
       </c>
       <c r="E14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A14)</f>
         <v/>
       </c>
       <c r="F14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A14)</f>
         <v/>
       </c>
       <c r="G14" s="3">
@@ -1171,7 +1171,7 @@
         </is>
       </c>
       <c r="C17" s="4">
-        <f>MIN(Calendario!G2:G72)</f>
+        <f>MIN(Calendario!G2:G79)</f>
         <v/>
       </c>
     </row>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="C18" s="7">
-        <f>INDEX(Calendario!A2:A72,MATCH(C17,Calendario!G2:G72,0))</f>
+        <f>INDEX(Calendario!A2:A79,MATCH(C17,Calendario!G2:G79,0))</f>
         <v/>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
         <v>1400</v>
       </c>
       <c r="E2" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A2)</f>
         <v/>
       </c>
       <c r="F2" s="3">
@@ -1291,7 +1291,7 @@
         <v/>
       </c>
       <c r="G2" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A2)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A2)</f>
         <v/>
       </c>
       <c r="H2" s="13" t="inlineStr">
@@ -1323,7 +1323,7 @@
         <v>1400</v>
       </c>
       <c r="E3" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A3)</f>
         <v/>
       </c>
       <c r="F3" s="3">
@@ -1331,7 +1331,7 @@
         <v/>
       </c>
       <c r="G3" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A3)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A3)</f>
         <v/>
       </c>
       <c r="H3" s="13" t="inlineStr">
@@ -1349,9 +1349,9 @@
           <t>Vivus</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
@@ -1363,7 +1363,7 @@
         <v>2148</v>
       </c>
       <c r="E4" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A4)</f>
         <v/>
       </c>
       <c r="F4" s="3">
@@ -1371,12 +1371,12 @@
         <v/>
       </c>
       <c r="G4" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A4)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A4)</f>
         <v/>
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>4 × 537 €. Plan: aplazar la cuota de nov y liquidar todo el 29 nov por 1.500 €</t>
+          <t>4 × 537 €, no aplazable. Plan: cuota del 1 nov y liquidar el resto el 29 nov (total 1.500 €)</t>
         </is>
       </c>
       <c r="I4" s="10" t="n">
@@ -1403,7 +1403,7 @@
         <v>435</v>
       </c>
       <c r="E5" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A5)</f>
         <v/>
       </c>
       <c r="F5" s="3">
@@ -1411,12 +1411,12 @@
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A5)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A5)</f>
         <v/>
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>Pago único, aplazado sin coste al 1 ene</t>
+          <t>Pago único hoy (13 oct). Volver a pedirlo cuesta: recibes 300 €, devuelves 435 €</t>
         </is>
       </c>
       <c r="I5" s="10" t="n">
@@ -1443,7 +1443,7 @@
         <v>1994.93</v>
       </c>
       <c r="E6" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A6)</f>
         <v/>
       </c>
       <c r="F6" s="3">
@@ -1451,7 +1451,7 @@
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A6)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A6)</f>
         <v/>
       </c>
       <c r="H6" s="13" t="inlineStr">
@@ -1483,7 +1483,7 @@
         <v>693.34</v>
       </c>
       <c r="E7" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A7)</f>
         <v/>
       </c>
       <c r="F7" s="3">
@@ -1491,12 +1491,12 @@
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A7)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A7)</f>
         <v/>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Aplazable sin coste; 3 cuotas ene–mar</t>
+          <t>Aplazable: en nov y dic pagas la cuota y la vuelves a pedir sin intereses; 3 cuotas ene–mar</t>
         </is>
       </c>
       <c r="I7" s="10" t="n">
@@ -1523,7 +1523,7 @@
         <v>923.61</v>
       </c>
       <c r="E8" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A8)</f>
         <v/>
       </c>
       <c r="F8" s="3">
@@ -1531,12 +1531,12 @@
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A8)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A8)</f>
         <v/>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>Aplazable sin coste; 3 cuotas ene–mar</t>
+          <t>Aplazable: en nov y dic pagas la cuota y la vuelves a pedir sin intereses; 3 cuotas ene–mar</t>
         </is>
       </c>
       <c r="I8" s="10" t="n">
@@ -1563,7 +1563,7 @@
         <v>1483.63</v>
       </c>
       <c r="E9" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A9)</f>
         <v/>
       </c>
       <c r="F9" s="3">
@@ -1571,12 +1571,12 @@
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A9)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A9)</f>
         <v/>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Aplazable sin coste; 3 cuotas ene–mar</t>
+          <t>Aplazable: en nov y dic pagas la cuota y la vuelves a pedir sin intereses; 3 cuotas ene–mar</t>
         </is>
       </c>
       <c r="I9" s="10" t="n">
@@ -1603,7 +1603,7 @@
         <v>2326.76</v>
       </c>
       <c r="E10" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A10)</f>
         <v/>
       </c>
       <c r="F10" s="3">
@@ -1611,7 +1611,7 @@
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A10)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A10)</f>
         <v/>
       </c>
       <c r="H10" s="13" t="inlineStr">
@@ -1643,7 +1643,7 @@
         <v>600</v>
       </c>
       <c r="E11" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A11)</f>
         <v/>
       </c>
       <c r="F11" s="3">
@@ -1651,7 +1651,7 @@
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A11)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A11)</f>
         <v/>
       </c>
       <c r="H11" s="13" t="inlineStr">
@@ -1683,7 +1683,7 @@
         <v>400</v>
       </c>
       <c r="E12" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A12)</f>
         <v/>
       </c>
       <c r="F12" s="3">
@@ -1691,7 +1691,7 @@
         <v/>
       </c>
       <c r="G12" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A12)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A12)</f>
         <v/>
       </c>
       <c r="H12" s="13" t="inlineStr">
@@ -1723,7 +1723,7 @@
         <v>300</v>
       </c>
       <c r="E13" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A13)</f>
         <v/>
       </c>
       <c r="F13" s="3">
@@ -1731,7 +1731,7 @@
         <v/>
       </c>
       <c r="G13" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A13)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A13)</f>
         <v/>
       </c>
       <c r="H13" s="13" t="inlineStr">
@@ -1763,7 +1763,7 @@
         <v>1700</v>
       </c>
       <c r="E14" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A14)</f>
         <v/>
       </c>
       <c r="F14" s="3">
@@ -1771,7 +1771,7 @@
         <v/>
       </c>
       <c r="G14" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A14)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A14)</f>
         <v/>
       </c>
       <c r="H14" s="13" t="inlineStr">
@@ -1803,7 +1803,7 @@
         <v>2500</v>
       </c>
       <c r="E15" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A15)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A15)</f>
         <v/>
       </c>
       <c r="F15" s="3">
@@ -1811,7 +1811,7 @@
         <v/>
       </c>
       <c r="G15" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A15)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A15)</f>
         <v/>
       </c>
       <c r="H15" s="13" t="inlineStr">
@@ -1909,7 +1909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1999,7 +1999,7 @@
     </row>
     <row r="3">
       <c r="A3" s="25" t="n">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B3" s="26">
         <f>DATE(YEAR(A3),MONTH(A3),1)</f>
@@ -2007,18 +2007,21 @@
       </c>
       <c r="C3" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida hasta el 29 oct (estimado)</t>
+          <t>Smartcredito · pago hoy</t>
         </is>
       </c>
       <c r="D3" s="28" t="inlineStr">
         <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E3" s="27" t="inlineStr"/>
-      <c r="F3" s="29">
-        <f>-Supuestos!B6</f>
-        <v/>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E3" s="27" t="inlineStr">
+        <is>
+          <t>Smartcredito</t>
+        </is>
+      </c>
+      <c r="F3" s="29" t="n">
+        <v>-435</v>
       </c>
       <c r="G3" s="30">
         <f>G2+F3</f>
@@ -2037,7 +2040,7 @@
     </row>
     <row r="4">
       <c r="A4" s="25" t="n">
-        <v>46324</v>
+        <v>46309</v>
       </c>
       <c r="B4" s="26">
         <f>DATE(YEAR(A4),MONTH(A4),1)</f>
@@ -2045,17 +2048,18 @@
       </c>
       <c r="C4" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
+          <t>Gastos de vida hasta el 29 oct (estimado)</t>
         </is>
       </c>
       <c r="D4" s="31" t="inlineStr">
         <is>
-          <t>Ingreso</t>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E4" s="27" t="inlineStr"/>
-      <c r="F4" s="32" t="n">
-        <v>2645.44</v>
+      <c r="F4" s="32">
+        <f>-Supuestos!B6</f>
+        <v/>
       </c>
       <c r="G4" s="30">
         <f>G3+F4</f>
@@ -2074,7 +2078,7 @@
     </row>
     <row r="5">
       <c r="A5" s="25" t="n">
-        <v>46327</v>
+        <v>46324</v>
       </c>
       <c r="B5" s="26">
         <f>DATE(YEAR(A5),MONTH(A5),1)</f>
@@ -2082,23 +2086,23 @@
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>Moneyman: vuelvo a pedir (recibo 1.100 €)</t>
-        </is>
-      </c>
-      <c r="D5" s="31" t="inlineStr">
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D5" s="33" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
       </c>
       <c r="E5" s="27" t="inlineStr"/>
-      <c r="F5" s="32" t="n">
-        <v>1100</v>
+      <c r="F5" s="29" t="n">
+        <v>2645.44</v>
       </c>
       <c r="G5" s="30">
         <f>G4+F5</f>
         <v/>
       </c>
-      <c r="I5" s="33" t="inlineStr">
+      <c r="I5" s="34" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
@@ -2119,21 +2123,17 @@
       </c>
       <c r="C6" s="27" t="inlineStr">
         <is>
-          <t>Moneyman</t>
-        </is>
-      </c>
-      <c r="D6" s="34" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E6" s="27" t="inlineStr">
-        <is>
-          <t>Moneyman</t>
-        </is>
-      </c>
-      <c r="F6" s="32" t="n">
-        <v>-1400</v>
+          <t>Moneyman: vuelvo a pedir (recibo 1.100 €)</t>
+        </is>
+      </c>
+      <c r="D6" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr"/>
+      <c r="F6" s="29" t="n">
+        <v>1100</v>
       </c>
       <c r="G6" s="30">
         <f>G5+F6</f>
@@ -2160,21 +2160,21 @@
       </c>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Ama</t>
-        </is>
-      </c>
-      <c r="D7" s="36" t="inlineStr">
-        <is>
-          <t>Amigo</t>
+          <t>Moneyman</t>
+        </is>
+      </c>
+      <c r="D7" s="28" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E7" s="27" t="inlineStr">
         <is>
-          <t>Ama</t>
-        </is>
-      </c>
-      <c r="F7" s="32" t="n">
-        <v>-600</v>
+          <t>Moneyman</t>
+        </is>
+      </c>
+      <c r="F7" s="29" t="n">
+        <v>-1400</v>
       </c>
       <c r="G7" s="30">
         <f>G6+F7</f>
@@ -2191,21 +2191,21 @@
       </c>
       <c r="C8" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D8" s="34" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Devolución a Ama</t>
+        </is>
+      </c>
+      <c r="D8" s="36" t="inlineStr">
+        <is>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E8" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F8" s="32" t="n">
-        <v>-96</v>
+          <t>Ama</t>
+        </is>
+      </c>
+      <c r="F8" s="29" t="n">
+        <v>-600</v>
       </c>
       <c r="G8" s="30">
         <f>G7+F8</f>
@@ -2227,21 +2227,21 @@
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
-        </is>
-      </c>
-      <c r="D9" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Vivus · cuota 1/4 (no aplazable)</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E9" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F9" s="32" t="n">
-        <v>-122.46</v>
+          <t>Vivus</t>
+        </is>
+      </c>
+      <c r="F9" s="29" t="n">
+        <v>-537</v>
       </c>
       <c r="G9" s="30">
         <f>G8+F9</f>
@@ -2258,18 +2258,17 @@
       </c>
       <c r="C10" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D10" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Pagolisto 1 · pagas 231,11 € y lo vuelves a pedir (neto 0)</t>
+        </is>
+      </c>
+      <c r="D10" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E10" s="27" t="inlineStr"/>
-      <c r="F10" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F10" s="29" t="n">
+        <v>0</v>
       </c>
       <c r="G10" s="30">
         <f>G9+F10</f>
@@ -2278,7 +2277,7 @@
     </row>
     <row r="11">
       <c r="A11" s="25" t="n">
-        <v>46355</v>
+        <v>46327</v>
       </c>
       <c r="B11" s="26">
         <f>DATE(YEAR(A11),MONTH(A11),1)</f>
@@ -2286,17 +2285,17 @@
       </c>
       <c r="C11" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D11" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Pagolisto 2 · pagas 307,87 € y lo vuelves a pedir (neto 0)</t>
+        </is>
+      </c>
+      <c r="D11" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E11" s="27" t="inlineStr"/>
-      <c r="F11" s="32" t="n">
-        <v>3453.01</v>
+      <c r="F11" s="29" t="n">
+        <v>0</v>
       </c>
       <c r="G11" s="30">
         <f>G10+F11</f>
@@ -2305,7 +2304,7 @@
     </row>
     <row r="12">
       <c r="A12" s="25" t="n">
-        <v>46355</v>
+        <v>46327</v>
       </c>
       <c r="B12" s="26">
         <f>DATE(YEAR(A12),MONTH(A12),1)</f>
@@ -2313,7 +2312,7 @@
       </c>
       <c r="C12" s="27" t="inlineStr">
         <is>
-          <t>Vivus · liquidación total (en vez de 4 × 537 €)</t>
+          <t>Crédito Santander 1 · pagas 494,54 € y lo vuelves a pedir (neto 0)</t>
         </is>
       </c>
       <c r="D12" s="37" t="inlineStr">
@@ -2321,13 +2320,9 @@
           <t>Aplazable</t>
         </is>
       </c>
-      <c r="E12" s="27" t="inlineStr">
-        <is>
-          <t>Vivus</t>
-        </is>
-      </c>
-      <c r="F12" s="32" t="n">
-        <v>-1500</v>
+      <c r="E12" s="27" t="inlineStr"/>
+      <c r="F12" s="29" t="n">
+        <v>0</v>
       </c>
       <c r="G12" s="30">
         <f>G11+F12</f>
@@ -2336,7 +2331,7 @@
     </row>
     <row r="13">
       <c r="A13" s="25" t="n">
-        <v>46357</v>
+        <v>46327</v>
       </c>
       <c r="B13" s="26">
         <f>DATE(YEAR(A13),MONTH(A13),1)</f>
@@ -2344,21 +2339,21 @@
       </c>
       <c r="C13" s="27" t="inlineStr">
         <is>
-          <t>Moneyman (vuelto a pedir)</t>
-        </is>
-      </c>
-      <c r="D13" s="34" t="inlineStr">
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D13" s="28" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
       </c>
       <c r="E13" s="27" t="inlineStr">
         <is>
-          <t>Moneyman (vuelto a pedir)</t>
-        </is>
-      </c>
-      <c r="F13" s="32" t="n">
-        <v>-1400</v>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F13" s="29" t="n">
+        <v>-96</v>
       </c>
       <c r="G13" s="30">
         <f>G12+F13</f>
@@ -2367,7 +2362,7 @@
     </row>
     <row r="14">
       <c r="A14" s="25" t="n">
-        <v>46357</v>
+        <v>46327</v>
       </c>
       <c r="B14" s="26">
         <f>DATE(YEAR(A14),MONTH(A14),1)</f>
@@ -2375,21 +2370,21 @@
       </c>
       <c r="C14" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D14" s="34" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D14" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E14" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F14" s="32" t="n">
-        <v>-96</v>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F14" s="29" t="n">
+        <v>-122.46</v>
       </c>
       <c r="G14" s="30">
         <f>G13+F14</f>
@@ -2398,7 +2393,7 @@
     </row>
     <row r="15">
       <c r="A15" s="25" t="n">
-        <v>46357</v>
+        <v>46327</v>
       </c>
       <c r="B15" s="26">
         <f>DATE(YEAR(A15),MONTH(A15),1)</f>
@@ -2406,21 +2401,18 @@
       </c>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
-        </is>
-      </c>
-      <c r="D15" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E15" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F15" s="32" t="n">
-        <v>-122.46</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D15" s="31" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E15" s="27" t="inlineStr"/>
+      <c r="F15" s="32">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G15" s="30">
         <f>G14+F15</f>
@@ -2429,7 +2421,7 @@
     </row>
     <row r="16">
       <c r="A16" s="25" t="n">
-        <v>46357</v>
+        <v>46355</v>
       </c>
       <c r="B16" s="26">
         <f>DATE(YEAR(A16),MONTH(A16),1)</f>
@@ -2437,18 +2429,17 @@
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D16" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D16" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E16" s="27" t="inlineStr"/>
-      <c r="F16" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F16" s="29" t="n">
+        <v>3453.01</v>
       </c>
       <c r="G16" s="30">
         <f>G15+F16</f>
@@ -2457,7 +2448,7 @@
     </row>
     <row r="17">
       <c r="A17" s="25" t="n">
-        <v>46385</v>
+        <v>46355</v>
       </c>
       <c r="B17" s="26">
         <f>DATE(YEAR(A17),MONTH(A17),1)</f>
@@ -2465,17 +2456,21 @@
       </c>
       <c r="C17" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D17" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E17" s="27" t="inlineStr"/>
-      <c r="F17" s="32" t="n">
-        <v>3453.01</v>
+          <t>Vivus · liquidación del resto (total 1.500 € en vez de 2.148 €)</t>
+        </is>
+      </c>
+      <c r="D17" s="28" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E17" s="27" t="inlineStr">
+        <is>
+          <t>Vivus</t>
+        </is>
+      </c>
+      <c r="F17" s="29" t="n">
+        <v>-963</v>
       </c>
       <c r="G17" s="30">
         <f>G16+F17</f>
@@ -2484,7 +2479,7 @@
     </row>
     <row r="18">
       <c r="A18" s="25" t="n">
-        <v>46385</v>
+        <v>46357</v>
       </c>
       <c r="B18" s="26">
         <f>DATE(YEAR(A18),MONTH(A18),1)</f>
@@ -2492,17 +2487,17 @@
       </c>
       <c r="C18" s="27" t="inlineStr">
         <is>
-          <t>Paga extra de diciembre</t>
-        </is>
-      </c>
-      <c r="D18" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Pagolisto 1 · pagas 231,11 € y lo vuelves a pedir (neto 0)</t>
+        </is>
+      </c>
+      <c r="D18" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E18" s="27" t="inlineStr"/>
-      <c r="F18" s="32" t="n">
-        <v>2014.69</v>
+      <c r="F18" s="29" t="n">
+        <v>0</v>
       </c>
       <c r="G18" s="30">
         <f>G17+F18</f>
@@ -2511,7 +2506,7 @@
     </row>
     <row r="19">
       <c r="A19" s="25" t="n">
-        <v>46388</v>
+        <v>46357</v>
       </c>
       <c r="B19" s="26">
         <f>DATE(YEAR(A19),MONTH(A19),1)</f>
@@ -2519,21 +2514,17 @@
       </c>
       <c r="C19" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D19" s="34" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E19" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F19" s="32" t="n">
-        <v>-96</v>
+          <t>Pagolisto 2 · pagas 307,87 € y lo vuelves a pedir (neto 0)</t>
+        </is>
+      </c>
+      <c r="D19" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E19" s="27" t="inlineStr"/>
+      <c r="F19" s="29" t="n">
+        <v>0</v>
       </c>
       <c r="G19" s="30">
         <f>G18+F19</f>
@@ -2542,7 +2533,7 @@
     </row>
     <row r="20">
       <c r="A20" s="25" t="n">
-        <v>46388</v>
+        <v>46357</v>
       </c>
       <c r="B20" s="26">
         <f>DATE(YEAR(A20),MONTH(A20),1)</f>
@@ -2550,7 +2541,7 @@
       </c>
       <c r="C20" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
+          <t>Crédito Santander 1 · pagas 494,54 € y lo vuelves a pedir (neto 0)</t>
         </is>
       </c>
       <c r="D20" s="37" t="inlineStr">
@@ -2558,13 +2549,9 @@
           <t>Aplazable</t>
         </is>
       </c>
-      <c r="E20" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F20" s="32" t="n">
-        <v>-122.46</v>
+      <c r="E20" s="27" t="inlineStr"/>
+      <c r="F20" s="29" t="n">
+        <v>0</v>
       </c>
       <c r="G20" s="30">
         <f>G19+F20</f>
@@ -2573,7 +2560,7 @@
     </row>
     <row r="21">
       <c r="A21" s="25" t="n">
-        <v>46388</v>
+        <v>46357</v>
       </c>
       <c r="B21" s="26">
         <f>DATE(YEAR(A21),MONTH(A21),1)</f>
@@ -2581,21 +2568,21 @@
       </c>
       <c r="C21" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 1/3</t>
-        </is>
-      </c>
-      <c r="D21" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Moneyman (vuelto a pedir)</t>
+        </is>
+      </c>
+      <c r="D21" s="28" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E21" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1</t>
-        </is>
-      </c>
-      <c r="F21" s="32" t="n">
-        <v>-231.11</v>
+          <t>Moneyman (vuelto a pedir)</t>
+        </is>
+      </c>
+      <c r="F21" s="29" t="n">
+        <v>-1400</v>
       </c>
       <c r="G21" s="30">
         <f>G20+F21</f>
@@ -2604,7 +2591,7 @@
     </row>
     <row r="22">
       <c r="A22" s="25" t="n">
-        <v>46388</v>
+        <v>46357</v>
       </c>
       <c r="B22" s="26">
         <f>DATE(YEAR(A22),MONTH(A22),1)</f>
@@ -2612,21 +2599,21 @@
       </c>
       <c r="C22" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 1/3</t>
-        </is>
-      </c>
-      <c r="D22" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D22" s="28" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E22" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2</t>
-        </is>
-      </c>
-      <c r="F22" s="32" t="n">
-        <v>-307.87</v>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F22" s="29" t="n">
+        <v>-96</v>
       </c>
       <c r="G22" s="30">
         <f>G21+F22</f>
@@ -2635,7 +2622,7 @@
     </row>
     <row r="23">
       <c r="A23" s="25" t="n">
-        <v>46388</v>
+        <v>46357</v>
       </c>
       <c r="B23" s="26">
         <f>DATE(YEAR(A23),MONTH(A23),1)</f>
@@ -2643,7 +2630,7 @@
       </c>
       <c r="C23" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 1/3</t>
+          <t>Crédito Santander 2 · cuota</t>
         </is>
       </c>
       <c r="D23" s="37" t="inlineStr">
@@ -2653,11 +2640,11 @@
       </c>
       <c r="E23" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1</t>
-        </is>
-      </c>
-      <c r="F23" s="32" t="n">
-        <v>-494.54</v>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F23" s="29" t="n">
+        <v>-122.46</v>
       </c>
       <c r="G23" s="30">
         <f>G22+F23</f>
@@ -2666,7 +2653,7 @@
     </row>
     <row r="24">
       <c r="A24" s="25" t="n">
-        <v>46388</v>
+        <v>46357</v>
       </c>
       <c r="B24" s="26">
         <f>DATE(YEAR(A24),MONTH(A24),1)</f>
@@ -2674,21 +2661,18 @@
       </c>
       <c r="C24" s="27" t="inlineStr">
         <is>
-          <t>Smartcredito</t>
-        </is>
-      </c>
-      <c r="D24" s="34" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E24" s="27" t="inlineStr">
-        <is>
-          <t>Smartcredito</t>
-        </is>
-      </c>
-      <c r="F24" s="32" t="n">
-        <v>-435</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D24" s="31" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="inlineStr"/>
+      <c r="F24" s="32">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G24" s="30">
         <f>G23+F24</f>
@@ -2697,7 +2681,7 @@
     </row>
     <row r="25">
       <c r="A25" s="25" t="n">
-        <v>46388</v>
+        <v>46385</v>
       </c>
       <c r="B25" s="26">
         <f>DATE(YEAR(A25),MONTH(A25),1)</f>
@@ -2705,21 +2689,17 @@
       </c>
       <c r="C25" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Joserra</t>
-        </is>
-      </c>
-      <c r="D25" s="36" t="inlineStr">
-        <is>
-          <t>Amigo</t>
-        </is>
-      </c>
-      <c r="E25" s="27" t="inlineStr">
-        <is>
-          <t>Joserra</t>
-        </is>
-      </c>
-      <c r="F25" s="32" t="n">
-        <v>-400</v>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D25" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E25" s="27" t="inlineStr"/>
+      <c r="F25" s="29" t="n">
+        <v>3453.01</v>
       </c>
       <c r="G25" s="30">
         <f>G24+F25</f>
@@ -2728,7 +2708,7 @@
     </row>
     <row r="26">
       <c r="A26" s="25" t="n">
-        <v>46388</v>
+        <v>46385</v>
       </c>
       <c r="B26" s="26">
         <f>DATE(YEAR(A26),MONTH(A26),1)</f>
@@ -2736,21 +2716,17 @@
       </c>
       <c r="C26" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Xabi</t>
-        </is>
-      </c>
-      <c r="D26" s="36" t="inlineStr">
-        <is>
-          <t>Amigo</t>
-        </is>
-      </c>
-      <c r="E26" s="27" t="inlineStr">
-        <is>
-          <t>Xabi</t>
-        </is>
-      </c>
-      <c r="F26" s="32" t="n">
-        <v>-300</v>
+          <t>Paga extra de diciembre</t>
+        </is>
+      </c>
+      <c r="D26" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E26" s="27" t="inlineStr"/>
+      <c r="F26" s="29" t="n">
+        <v>2014.69</v>
       </c>
       <c r="G26" s="30">
         <f>G25+F26</f>
@@ -2767,18 +2743,21 @@
       </c>
       <c r="C27" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
+          <t>Santander (préstamo) · cuota</t>
         </is>
       </c>
       <c r="D27" s="28" t="inlineStr">
         <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E27" s="27" t="inlineStr"/>
-      <c r="F27" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E27" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F27" s="29" t="n">
+        <v>-96</v>
       </c>
       <c r="G27" s="30">
         <f>G26+F27</f>
@@ -2787,7 +2766,7 @@
     </row>
     <row r="28">
       <c r="A28" s="25" t="n">
-        <v>46416</v>
+        <v>46388</v>
       </c>
       <c r="B28" s="26">
         <f>DATE(YEAR(A28),MONTH(A28),1)</f>
@@ -2795,17 +2774,21 @@
       </c>
       <c r="C28" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D28" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E28" s="27" t="inlineStr"/>
-      <c r="F28" s="32" t="n">
-        <v>3173.56</v>
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D28" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E28" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F28" s="29" t="n">
+        <v>-122.46</v>
       </c>
       <c r="G28" s="30">
         <f>G27+F28</f>
@@ -2814,7 +2797,7 @@
     </row>
     <row r="29">
       <c r="A29" s="25" t="n">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="B29" s="26">
         <f>DATE(YEAR(A29),MONTH(A29),1)</f>
@@ -2822,21 +2805,21 @@
       </c>
       <c r="C29" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D29" s="34" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Pagolisto 1 · cuota 1/3</t>
+        </is>
+      </c>
+      <c r="D29" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E29" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F29" s="32" t="n">
-        <v>-96</v>
+          <t>Pagolisto 1</t>
+        </is>
+      </c>
+      <c r="F29" s="29" t="n">
+        <v>-231.11</v>
       </c>
       <c r="G29" s="30">
         <f>G28+F29</f>
@@ -2845,7 +2828,7 @@
     </row>
     <row r="30">
       <c r="A30" s="25" t="n">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="B30" s="26">
         <f>DATE(YEAR(A30),MONTH(A30),1)</f>
@@ -2853,7 +2836,7 @@
       </c>
       <c r="C30" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
+          <t>Pagolisto 2 · cuota 1/3</t>
         </is>
       </c>
       <c r="D30" s="37" t="inlineStr">
@@ -2863,11 +2846,11 @@
       </c>
       <c r="E30" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F30" s="32" t="n">
-        <v>-122.46</v>
+          <t>Pagolisto 2</t>
+        </is>
+      </c>
+      <c r="F30" s="29" t="n">
+        <v>-307.87</v>
       </c>
       <c r="G30" s="30">
         <f>G29+F30</f>
@@ -2876,7 +2859,7 @@
     </row>
     <row r="31">
       <c r="A31" s="25" t="n">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="B31" s="26">
         <f>DATE(YEAR(A31),MONTH(A31),1)</f>
@@ -2884,7 +2867,7 @@
       </c>
       <c r="C31" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 2/3</t>
+          <t>Crédito Santander 1 · cuota 1/3</t>
         </is>
       </c>
       <c r="D31" s="37" t="inlineStr">
@@ -2894,11 +2877,11 @@
       </c>
       <c r="E31" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1</t>
-        </is>
-      </c>
-      <c r="F31" s="32" t="n">
-        <v>-231.11</v>
+          <t>Crédito Santander 1</t>
+        </is>
+      </c>
+      <c r="F31" s="29" t="n">
+        <v>-494.54</v>
       </c>
       <c r="G31" s="30">
         <f>G30+F31</f>
@@ -2907,7 +2890,7 @@
     </row>
     <row r="32">
       <c r="A32" s="25" t="n">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="B32" s="26">
         <f>DATE(YEAR(A32),MONTH(A32),1)</f>
@@ -2915,21 +2898,21 @@
       </c>
       <c r="C32" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 2/3</t>
-        </is>
-      </c>
-      <c r="D32" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Devolución a Joserra</t>
+        </is>
+      </c>
+      <c r="D32" s="36" t="inlineStr">
+        <is>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E32" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2</t>
-        </is>
-      </c>
-      <c r="F32" s="32" t="n">
-        <v>-307.87</v>
+          <t>Joserra</t>
+        </is>
+      </c>
+      <c r="F32" s="29" t="n">
+        <v>-400</v>
       </c>
       <c r="G32" s="30">
         <f>G31+F32</f>
@@ -2938,7 +2921,7 @@
     </row>
     <row r="33">
       <c r="A33" s="25" t="n">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="B33" s="26">
         <f>DATE(YEAR(A33),MONTH(A33),1)</f>
@@ -2946,21 +2929,21 @@
       </c>
       <c r="C33" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 2/3</t>
-        </is>
-      </c>
-      <c r="D33" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Devolución a Xabi</t>
+        </is>
+      </c>
+      <c r="D33" s="36" t="inlineStr">
+        <is>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E33" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1</t>
-        </is>
-      </c>
-      <c r="F33" s="32" t="n">
-        <v>-494.54</v>
+          <t>Xabi</t>
+        </is>
+      </c>
+      <c r="F33" s="29" t="n">
+        <v>-300</v>
       </c>
       <c r="G33" s="30">
         <f>G32+F33</f>
@@ -2969,7 +2952,7 @@
     </row>
     <row r="34">
       <c r="A34" s="25" t="n">
-        <v>46419</v>
+        <v>46388</v>
       </c>
       <c r="B34" s="26">
         <f>DATE(YEAR(A34),MONTH(A34),1)</f>
@@ -2977,21 +2960,18 @@
       </c>
       <c r="C34" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Sergio</t>
-        </is>
-      </c>
-      <c r="D34" s="36" t="inlineStr">
-        <is>
-          <t>Amigo</t>
-        </is>
-      </c>
-      <c r="E34" s="27" t="inlineStr">
-        <is>
-          <t>Sergio</t>
-        </is>
-      </c>
-      <c r="F34" s="32" t="n">
-        <v>-1700</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D34" s="31" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E34" s="27" t="inlineStr"/>
+      <c r="F34" s="32">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G34" s="30">
         <f>G33+F34</f>
@@ -3000,7 +2980,7 @@
     </row>
     <row r="35">
       <c r="A35" s="25" t="n">
-        <v>46419</v>
+        <v>46416</v>
       </c>
       <c r="B35" s="26">
         <f>DATE(YEAR(A35),MONTH(A35),1)</f>
@@ -3008,18 +2988,17 @@
       </c>
       <c r="C35" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D35" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D35" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E35" s="27" t="inlineStr"/>
-      <c r="F35" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F35" s="29" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G35" s="30">
         <f>G34+F35</f>
@@ -3028,7 +3007,7 @@
     </row>
     <row r="36">
       <c r="A36" s="25" t="n">
-        <v>46446</v>
+        <v>46419</v>
       </c>
       <c r="B36" s="26">
         <f>DATE(YEAR(A36),MONTH(A36),1)</f>
@@ -3036,17 +3015,21 @@
       </c>
       <c r="C36" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D36" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E36" s="27" t="inlineStr"/>
-      <c r="F36" s="32" t="n">
-        <v>3173.56</v>
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D36" s="28" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E36" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F36" s="29" t="n">
+        <v>-96</v>
       </c>
       <c r="G36" s="30">
         <f>G35+F36</f>
@@ -3055,7 +3038,7 @@
     </row>
     <row r="37">
       <c r="A37" s="25" t="n">
-        <v>46446</v>
+        <v>46419</v>
       </c>
       <c r="B37" s="26">
         <f>DATE(YEAR(A37),MONTH(A37),1)</f>
@@ -3063,17 +3046,21 @@
       </c>
       <c r="C37" s="27" t="inlineStr">
         <is>
-          <t>Variable de febrero</t>
-        </is>
-      </c>
-      <c r="D37" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E37" s="27" t="inlineStr"/>
-      <c r="F37" s="32" t="n">
-        <v>2114.45</v>
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D37" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E37" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F37" s="29" t="n">
+        <v>-122.46</v>
       </c>
       <c r="G37" s="30">
         <f>G36+F37</f>
@@ -3082,7 +3069,7 @@
     </row>
     <row r="38">
       <c r="A38" s="25" t="n">
-        <v>46446</v>
+        <v>46419</v>
       </c>
       <c r="B38" s="26">
         <f>DATE(YEAR(A38),MONTH(A38),1)</f>
@@ -3090,21 +3077,21 @@
       </c>
       <c r="C38" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Txomin</t>
-        </is>
-      </c>
-      <c r="D38" s="36" t="inlineStr">
-        <is>
-          <t>Amigo</t>
+          <t>Pagolisto 1 · cuota 2/3</t>
+        </is>
+      </c>
+      <c r="D38" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E38" s="27" t="inlineStr">
         <is>
-          <t>Txomin</t>
-        </is>
-      </c>
-      <c r="F38" s="32" t="n">
-        <v>-2500</v>
+          <t>Pagolisto 1</t>
+        </is>
+      </c>
+      <c r="F38" s="29" t="n">
+        <v>-231.11</v>
       </c>
       <c r="G38" s="30">
         <f>G37+F38</f>
@@ -3113,7 +3100,7 @@
     </row>
     <row r="39">
       <c r="A39" s="25" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="B39" s="26">
         <f>DATE(YEAR(A39),MONTH(A39),1)</f>
@@ -3121,21 +3108,21 @@
       </c>
       <c r="C39" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D39" s="34" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Pagolisto 2 · cuota 2/3</t>
+        </is>
+      </c>
+      <c r="D39" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E39" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F39" s="32" t="n">
-        <v>-96</v>
+          <t>Pagolisto 2</t>
+        </is>
+      </c>
+      <c r="F39" s="29" t="n">
+        <v>-307.87</v>
       </c>
       <c r="G39" s="30">
         <f>G38+F39</f>
@@ -3144,7 +3131,7 @@
     </row>
     <row r="40">
       <c r="A40" s="25" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="B40" s="26">
         <f>DATE(YEAR(A40),MONTH(A40),1)</f>
@@ -3152,7 +3139,7 @@
       </c>
       <c r="C40" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
+          <t>Crédito Santander 1 · cuota 2/3</t>
         </is>
       </c>
       <c r="D40" s="37" t="inlineStr">
@@ -3162,11 +3149,11 @@
       </c>
       <c r="E40" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F40" s="32" t="n">
-        <v>-122.46</v>
+          <t>Crédito Santander 1</t>
+        </is>
+      </c>
+      <c r="F40" s="29" t="n">
+        <v>-494.54</v>
       </c>
       <c r="G40" s="30">
         <f>G39+F40</f>
@@ -3175,7 +3162,7 @@
     </row>
     <row r="41">
       <c r="A41" s="25" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="B41" s="26">
         <f>DATE(YEAR(A41),MONTH(A41),1)</f>
@@ -3183,21 +3170,21 @@
       </c>
       <c r="C41" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 3/3</t>
-        </is>
-      </c>
-      <c r="D41" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Devolución a Sergio</t>
+        </is>
+      </c>
+      <c r="D41" s="36" t="inlineStr">
+        <is>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E41" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1</t>
-        </is>
-      </c>
-      <c r="F41" s="32" t="n">
-        <v>-231.12</v>
+          <t>Sergio</t>
+        </is>
+      </c>
+      <c r="F41" s="29" t="n">
+        <v>-1700</v>
       </c>
       <c r="G41" s="30">
         <f>G40+F41</f>
@@ -3206,7 +3193,7 @@
     </row>
     <row r="42">
       <c r="A42" s="25" t="n">
-        <v>46447</v>
+        <v>46419</v>
       </c>
       <c r="B42" s="26">
         <f>DATE(YEAR(A42),MONTH(A42),1)</f>
@@ -3214,21 +3201,18 @@
       </c>
       <c r="C42" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 3/3</t>
-        </is>
-      </c>
-      <c r="D42" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E42" s="27" t="inlineStr">
-        <is>
-          <t>Pagolisto 2</t>
-        </is>
-      </c>
-      <c r="F42" s="32" t="n">
-        <v>-307.87</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D42" s="31" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E42" s="27" t="inlineStr"/>
+      <c r="F42" s="32">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G42" s="30">
         <f>G41+F42</f>
@@ -3237,7 +3221,7 @@
     </row>
     <row r="43">
       <c r="A43" s="25" t="n">
-        <v>46447</v>
+        <v>46446</v>
       </c>
       <c r="B43" s="26">
         <f>DATE(YEAR(A43),MONTH(A43),1)</f>
@@ -3245,21 +3229,17 @@
       </c>
       <c r="C43" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 3/3</t>
-        </is>
-      </c>
-      <c r="D43" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E43" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 1</t>
-        </is>
-      </c>
-      <c r="F43" s="32" t="n">
-        <v>-494.55</v>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D43" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E43" s="27" t="inlineStr"/>
+      <c r="F43" s="29" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G43" s="30">
         <f>G42+F43</f>
@@ -3268,7 +3248,7 @@
     </row>
     <row r="44">
       <c r="A44" s="25" t="n">
-        <v>46447</v>
+        <v>46446</v>
       </c>
       <c r="B44" s="26">
         <f>DATE(YEAR(A44),MONTH(A44),1)</f>
@@ -3276,18 +3256,17 @@
       </c>
       <c r="C44" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D44" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Variable de febrero</t>
+        </is>
+      </c>
+      <c r="D44" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E44" s="27" t="inlineStr"/>
-      <c r="F44" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F44" s="29" t="n">
+        <v>2114.45</v>
       </c>
       <c r="G44" s="30">
         <f>G43+F44</f>
@@ -3296,7 +3275,7 @@
     </row>
     <row r="45">
       <c r="A45" s="25" t="n">
-        <v>46475</v>
+        <v>46446</v>
       </c>
       <c r="B45" s="26">
         <f>DATE(YEAR(A45),MONTH(A45),1)</f>
@@ -3304,17 +3283,21 @@
       </c>
       <c r="C45" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D45" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E45" s="27" t="inlineStr"/>
-      <c r="F45" s="32" t="n">
-        <v>3173.56</v>
+          <t>Devolución a Txomin</t>
+        </is>
+      </c>
+      <c r="D45" s="36" t="inlineStr">
+        <is>
+          <t>Amigo</t>
+        </is>
+      </c>
+      <c r="E45" s="27" t="inlineStr">
+        <is>
+          <t>Txomin</t>
+        </is>
+      </c>
+      <c r="F45" s="29" t="n">
+        <v>-2500</v>
       </c>
       <c r="G45" s="30">
         <f>G44+F45</f>
@@ -3323,7 +3306,7 @@
     </row>
     <row r="46">
       <c r="A46" s="25" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="B46" s="26">
         <f>DATE(YEAR(A46),MONTH(A46),1)</f>
@@ -3331,10 +3314,10 @@
       </c>
       <c r="C46" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D46" s="34" t="inlineStr">
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D46" s="28" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
@@ -3344,7 +3327,7 @@
           <t>Santander (préstamo)</t>
         </is>
       </c>
-      <c r="F46" s="32" t="n">
+      <c r="F46" s="29" t="n">
         <v>-96</v>
       </c>
       <c r="G46" s="30">
@@ -3354,7 +3337,7 @@
     </row>
     <row r="47">
       <c r="A47" s="25" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="B47" s="26">
         <f>DATE(YEAR(A47),MONTH(A47),1)</f>
@@ -3362,7 +3345,7 @@
       </c>
       <c r="C47" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
+          <t>Crédito Santander 2 · cuota</t>
         </is>
       </c>
       <c r="D47" s="37" t="inlineStr">
@@ -3375,8 +3358,8 @@
           <t>Crédito Santander 2</t>
         </is>
       </c>
-      <c r="F47" s="32" t="n">
-        <v>-404</v>
+      <c r="F47" s="29" t="n">
+        <v>-122.46</v>
       </c>
       <c r="G47" s="30">
         <f>G46+F47</f>
@@ -3385,7 +3368,7 @@
     </row>
     <row r="48">
       <c r="A48" s="25" t="n">
-        <v>46478</v>
+        <v>46447</v>
       </c>
       <c r="B48" s="26">
         <f>DATE(YEAR(A48),MONTH(A48),1)</f>
@@ -3393,18 +3376,21 @@
       </c>
       <c r="C48" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D48" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E48" s="27" t="inlineStr"/>
-      <c r="F48" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Pagolisto 1 · cuota 3/3</t>
+        </is>
+      </c>
+      <c r="D48" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E48" s="27" t="inlineStr">
+        <is>
+          <t>Pagolisto 1</t>
+        </is>
+      </c>
+      <c r="F48" s="29" t="n">
+        <v>-231.12</v>
       </c>
       <c r="G48" s="30">
         <f>G47+F48</f>
@@ -3413,7 +3399,7 @@
     </row>
     <row r="49">
       <c r="A49" s="25" t="n">
-        <v>46506</v>
+        <v>46447</v>
       </c>
       <c r="B49" s="26">
         <f>DATE(YEAR(A49),MONTH(A49),1)</f>
@@ -3421,17 +3407,21 @@
       </c>
       <c r="C49" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D49" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E49" s="27" t="inlineStr"/>
-      <c r="F49" s="32" t="n">
-        <v>3173.56</v>
+          <t>Pagolisto 2 · cuota 3/3</t>
+        </is>
+      </c>
+      <c r="D49" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E49" s="27" t="inlineStr">
+        <is>
+          <t>Pagolisto 2</t>
+        </is>
+      </c>
+      <c r="F49" s="29" t="n">
+        <v>-307.87</v>
       </c>
       <c r="G49" s="30">
         <f>G48+F49</f>
@@ -3440,7 +3430,7 @@
     </row>
     <row r="50">
       <c r="A50" s="25" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="B50" s="26">
         <f>DATE(YEAR(A50),MONTH(A50),1)</f>
@@ -3448,21 +3438,21 @@
       </c>
       <c r="C50" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D50" s="34" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 1 · cuota 3/3</t>
+        </is>
+      </c>
+      <c r="D50" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E50" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F50" s="32" t="n">
-        <v>-96</v>
+          <t>Crédito Santander 1</t>
+        </is>
+      </c>
+      <c r="F50" s="29" t="n">
+        <v>-494.55</v>
       </c>
       <c r="G50" s="30">
         <f>G49+F50</f>
@@ -3471,7 +3461,7 @@
     </row>
     <row r="51">
       <c r="A51" s="25" t="n">
-        <v>46508</v>
+        <v>46447</v>
       </c>
       <c r="B51" s="26">
         <f>DATE(YEAR(A51),MONTH(A51),1)</f>
@@ -3479,21 +3469,18 @@
       </c>
       <c r="C51" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D51" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E51" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F51" s="32" t="n">
-        <v>-404</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D51" s="31" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E51" s="27" t="inlineStr"/>
+      <c r="F51" s="32">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G51" s="30">
         <f>G50+F51</f>
@@ -3502,7 +3489,7 @@
     </row>
     <row r="52">
       <c r="A52" s="25" t="n">
-        <v>46508</v>
+        <v>46475</v>
       </c>
       <c r="B52" s="26">
         <f>DATE(YEAR(A52),MONTH(A52),1)</f>
@@ -3510,18 +3497,17 @@
       </c>
       <c r="C52" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D52" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D52" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E52" s="27" t="inlineStr"/>
-      <c r="F52" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F52" s="29" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G52" s="30">
         <f>G51+F52</f>
@@ -3530,7 +3516,7 @@
     </row>
     <row r="53">
       <c r="A53" s="25" t="n">
-        <v>46536</v>
+        <v>46478</v>
       </c>
       <c r="B53" s="26">
         <f>DATE(YEAR(A53),MONTH(A53),1)</f>
@@ -3538,17 +3524,21 @@
       </c>
       <c r="C53" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D53" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E53" s="27" t="inlineStr"/>
-      <c r="F53" s="32" t="n">
-        <v>3173.56</v>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D53" s="28" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E53" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F53" s="29" t="n">
+        <v>-96</v>
       </c>
       <c r="G53" s="30">
         <f>G52+F53</f>
@@ -3557,7 +3547,7 @@
     </row>
     <row r="54">
       <c r="A54" s="25" t="n">
-        <v>46539</v>
+        <v>46478</v>
       </c>
       <c r="B54" s="26">
         <f>DATE(YEAR(A54),MONTH(A54),1)</f>
@@ -3565,21 +3555,21 @@
       </c>
       <c r="C54" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D54" s="34" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D54" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E54" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F54" s="32" t="n">
-        <v>-96</v>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F54" s="29" t="n">
+        <v>-404</v>
       </c>
       <c r="G54" s="30">
         <f>G53+F54</f>
@@ -3588,7 +3578,7 @@
     </row>
     <row r="55">
       <c r="A55" s="25" t="n">
-        <v>46539</v>
+        <v>46478</v>
       </c>
       <c r="B55" s="26">
         <f>DATE(YEAR(A55),MONTH(A55),1)</f>
@@ -3596,21 +3586,18 @@
       </c>
       <c r="C55" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D55" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E55" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F55" s="32" t="n">
-        <v>-404</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D55" s="31" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E55" s="27" t="inlineStr"/>
+      <c r="F55" s="32">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G55" s="30">
         <f>G54+F55</f>
@@ -3619,7 +3606,7 @@
     </row>
     <row r="56">
       <c r="A56" s="25" t="n">
-        <v>46539</v>
+        <v>46506</v>
       </c>
       <c r="B56" s="26">
         <f>DATE(YEAR(A56),MONTH(A56),1)</f>
@@ -3627,18 +3614,17 @@
       </c>
       <c r="C56" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D56" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D56" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E56" s="27" t="inlineStr"/>
-      <c r="F56" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F56" s="29" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G56" s="30">
         <f>G55+F56</f>
@@ -3647,7 +3633,7 @@
     </row>
     <row r="57">
       <c r="A57" s="25" t="n">
-        <v>46567</v>
+        <v>46508</v>
       </c>
       <c r="B57" s="26">
         <f>DATE(YEAR(A57),MONTH(A57),1)</f>
@@ -3655,17 +3641,21 @@
       </c>
       <c r="C57" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D57" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E57" s="27" t="inlineStr"/>
-      <c r="F57" s="32" t="n">
-        <v>3173.56</v>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D57" s="28" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E57" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F57" s="29" t="n">
+        <v>-96</v>
       </c>
       <c r="G57" s="30">
         <f>G56+F57</f>
@@ -3674,7 +3664,7 @@
     </row>
     <row r="58">
       <c r="A58" s="25" t="n">
-        <v>46567</v>
+        <v>46508</v>
       </c>
       <c r="B58" s="26">
         <f>DATE(YEAR(A58),MONTH(A58),1)</f>
@@ -3682,17 +3672,21 @@
       </c>
       <c r="C58" s="27" t="inlineStr">
         <is>
-          <t>Paga extra de junio</t>
-        </is>
-      </c>
-      <c r="D58" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E58" s="27" t="inlineStr"/>
-      <c r="F58" s="32" t="n">
-        <v>1989.05</v>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D58" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E58" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F58" s="29" t="n">
+        <v>-404</v>
       </c>
       <c r="G58" s="30">
         <f>G57+F58</f>
@@ -3701,7 +3695,7 @@
     </row>
     <row r="59">
       <c r="A59" s="25" t="n">
-        <v>46569</v>
+        <v>46508</v>
       </c>
       <c r="B59" s="26">
         <f>DATE(YEAR(A59),MONTH(A59),1)</f>
@@ -3709,21 +3703,18 @@
       </c>
       <c r="C59" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D59" s="34" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E59" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F59" s="32" t="n">
-        <v>-96</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D59" s="31" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E59" s="27" t="inlineStr"/>
+      <c r="F59" s="32">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G59" s="30">
         <f>G58+F59</f>
@@ -3732,7 +3723,7 @@
     </row>
     <row r="60">
       <c r="A60" s="25" t="n">
-        <v>46569</v>
+        <v>46536</v>
       </c>
       <c r="B60" s="26">
         <f>DATE(YEAR(A60),MONTH(A60),1)</f>
@@ -3740,21 +3731,17 @@
       </c>
       <c r="C60" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D60" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E60" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F60" s="32" t="n">
-        <v>-404</v>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D60" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E60" s="27" t="inlineStr"/>
+      <c r="F60" s="29" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G60" s="30">
         <f>G59+F60</f>
@@ -3763,7 +3750,7 @@
     </row>
     <row r="61">
       <c r="A61" s="25" t="n">
-        <v>46569</v>
+        <v>46539</v>
       </c>
       <c r="B61" s="26">
         <f>DATE(YEAR(A61),MONTH(A61),1)</f>
@@ -3771,18 +3758,21 @@
       </c>
       <c r="C61" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
         </is>
       </c>
       <c r="D61" s="28" t="inlineStr">
         <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E61" s="27" t="inlineStr"/>
-      <c r="F61" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E61" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F61" s="29" t="n">
+        <v>-96</v>
       </c>
       <c r="G61" s="30">
         <f>G60+F61</f>
@@ -3791,7 +3781,7 @@
     </row>
     <row r="62">
       <c r="A62" s="25" t="n">
-        <v>46597</v>
+        <v>46539</v>
       </c>
       <c r="B62" s="26">
         <f>DATE(YEAR(A62),MONTH(A62),1)</f>
@@ -3799,17 +3789,21 @@
       </c>
       <c r="C62" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D62" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E62" s="27" t="inlineStr"/>
-      <c r="F62" s="32" t="n">
-        <v>3173.56</v>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D62" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E62" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F62" s="29" t="n">
+        <v>-404</v>
       </c>
       <c r="G62" s="30">
         <f>G61+F62</f>
@@ -3818,7 +3812,7 @@
     </row>
     <row r="63">
       <c r="A63" s="25" t="n">
-        <v>46600</v>
+        <v>46539</v>
       </c>
       <c r="B63" s="26">
         <f>DATE(YEAR(A63),MONTH(A63),1)</f>
@@ -3826,21 +3820,18 @@
       </c>
       <c r="C63" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D63" s="34" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E63" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F63" s="32" t="n">
-        <v>-401.54</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D63" s="31" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E63" s="27" t="inlineStr"/>
+      <c r="F63" s="32">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G63" s="30">
         <f>G62+F63</f>
@@ -3849,7 +3840,7 @@
     </row>
     <row r="64">
       <c r="A64" s="25" t="n">
-        <v>46600</v>
+        <v>46567</v>
       </c>
       <c r="B64" s="26">
         <f>DATE(YEAR(A64),MONTH(A64),1)</f>
@@ -3857,21 +3848,17 @@
       </c>
       <c r="C64" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D64" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E64" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F64" s="32" t="n">
-        <v>-98.45999999999999</v>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D64" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E64" s="27" t="inlineStr"/>
+      <c r="F64" s="29" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G64" s="30">
         <f>G63+F64</f>
@@ -3880,7 +3867,7 @@
     </row>
     <row r="65">
       <c r="A65" s="25" t="n">
-        <v>46600</v>
+        <v>46567</v>
       </c>
       <c r="B65" s="26">
         <f>DATE(YEAR(A65),MONTH(A65),1)</f>
@@ -3888,18 +3875,17 @@
       </c>
       <c r="C65" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D65" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Paga extra de junio</t>
+        </is>
+      </c>
+      <c r="D65" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E65" s="27" t="inlineStr"/>
-      <c r="F65" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F65" s="29" t="n">
+        <v>1989.05</v>
       </c>
       <c r="G65" s="30">
         <f>G64+F65</f>
@@ -3908,7 +3894,7 @@
     </row>
     <row r="66">
       <c r="A66" s="25" t="n">
-        <v>46628</v>
+        <v>46569</v>
       </c>
       <c r="B66" s="26">
         <f>DATE(YEAR(A66),MONTH(A66),1)</f>
@@ -3916,17 +3902,21 @@
       </c>
       <c r="C66" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D66" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E66" s="27" t="inlineStr"/>
-      <c r="F66" s="32" t="n">
-        <v>2280.25</v>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D66" s="28" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E66" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F66" s="29" t="n">
+        <v>-96</v>
       </c>
       <c r="G66" s="30">
         <f>G65+F66</f>
@@ -3935,7 +3925,7 @@
     </row>
     <row r="67">
       <c r="A67" s="25" t="n">
-        <v>46631</v>
+        <v>46569</v>
       </c>
       <c r="B67" s="26">
         <f>DATE(YEAR(A67),MONTH(A67),1)</f>
@@ -3943,21 +3933,21 @@
       </c>
       <c r="C67" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D67" s="34" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D67" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E67" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F67" s="32" t="n">
-        <v>-500</v>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F67" s="29" t="n">
+        <v>-404</v>
       </c>
       <c r="G67" s="30">
         <f>G66+F67</f>
@@ -3966,7 +3956,7 @@
     </row>
     <row r="68">
       <c r="A68" s="25" t="n">
-        <v>46631</v>
+        <v>46569</v>
       </c>
       <c r="B68" s="26">
         <f>DATE(YEAR(A68),MONTH(A68),1)</f>
@@ -3977,13 +3967,13 @@
           <t>Gastos de vida</t>
         </is>
       </c>
-      <c r="D68" s="28" t="inlineStr">
+      <c r="D68" s="31" t="inlineStr">
         <is>
           <t>Gasto</t>
         </is>
       </c>
       <c r="E68" s="27" t="inlineStr"/>
-      <c r="F68" s="29">
+      <c r="F68" s="32">
         <f>-Supuestos!B7</f>
         <v/>
       </c>
@@ -3994,7 +3984,7 @@
     </row>
     <row r="69">
       <c r="A69" s="25" t="n">
-        <v>46659</v>
+        <v>46597</v>
       </c>
       <c r="B69" s="26">
         <f>DATE(YEAR(A69),MONTH(A69),1)</f>
@@ -4005,13 +3995,13 @@
           <t>Nómina</t>
         </is>
       </c>
-      <c r="D69" s="31" t="inlineStr">
+      <c r="D69" s="33" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
       </c>
       <c r="E69" s="27" t="inlineStr"/>
-      <c r="F69" s="32" t="n">
+      <c r="F69" s="29" t="n">
         <v>3173.56</v>
       </c>
       <c r="G69" s="30">
@@ -4021,7 +4011,7 @@
     </row>
     <row r="70">
       <c r="A70" s="25" t="n">
-        <v>46661</v>
+        <v>46600</v>
       </c>
       <c r="B70" s="26">
         <f>DATE(YEAR(A70),MONTH(A70),1)</f>
@@ -4032,7 +4022,7 @@
           <t>Santander (préstamo) · plan 500 €/mes</t>
         </is>
       </c>
-      <c r="D70" s="34" t="inlineStr">
+      <c r="D70" s="28" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
@@ -4042,8 +4032,8 @@
           <t>Santander (préstamo)</t>
         </is>
       </c>
-      <c r="F70" s="32" t="n">
-        <v>-229.39</v>
+      <c r="F70" s="29" t="n">
+        <v>-401.54</v>
       </c>
       <c r="G70" s="30">
         <f>G69+F70</f>
@@ -4052,7 +4042,7 @@
     </row>
     <row r="71">
       <c r="A71" s="25" t="n">
-        <v>46661</v>
+        <v>46600</v>
       </c>
       <c r="B71" s="26">
         <f>DATE(YEAR(A71),MONTH(A71),1)</f>
@@ -4060,18 +4050,21 @@
       </c>
       <c r="C71" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D71" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E71" s="27" t="inlineStr"/>
-      <c r="F71" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D71" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E71" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F71" s="29" t="n">
+        <v>-98.45999999999999</v>
       </c>
       <c r="G71" s="30">
         <f>G70+F71</f>
@@ -4080,7 +4073,7 @@
     </row>
     <row r="72">
       <c r="A72" s="25" t="n">
-        <v>46689</v>
+        <v>46600</v>
       </c>
       <c r="B72" s="26">
         <f>DATE(YEAR(A72),MONTH(A72),1)</f>
@@ -4088,26 +4081,226 @@
       </c>
       <c r="C72" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
+          <t>Gastos de vida</t>
         </is>
       </c>
       <c r="D72" s="31" t="inlineStr">
         <is>
-          <t>Ingreso</t>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E72" s="27" t="inlineStr"/>
-      <c r="F72" s="32" t="n">
-        <v>2490.44</v>
+      <c r="F72" s="32">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G72" s="30">
         <f>G71+F72</f>
         <v/>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="25" t="n">
+        <v>46628</v>
+      </c>
+      <c r="B73" s="26">
+        <f>DATE(YEAR(A73),MONTH(A73),1)</f>
+        <v/>
+      </c>
+      <c r="C73" s="27" t="inlineStr">
+        <is>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D73" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E73" s="27" t="inlineStr"/>
+      <c r="F73" s="29" t="n">
+        <v>2280.25</v>
+      </c>
+      <c r="G73" s="30">
+        <f>G72+F73</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="25" t="n">
+        <v>46631</v>
+      </c>
+      <c r="B74" s="26">
+        <f>DATE(YEAR(A74),MONTH(A74),1)</f>
+        <v/>
+      </c>
+      <c r="C74" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D74" s="28" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E74" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F74" s="29" t="n">
+        <v>-500</v>
+      </c>
+      <c r="G74" s="30">
+        <f>G73+F74</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="25" t="n">
+        <v>46631</v>
+      </c>
+      <c r="B75" s="26">
+        <f>DATE(YEAR(A75),MONTH(A75),1)</f>
+        <v/>
+      </c>
+      <c r="C75" s="27" t="inlineStr">
+        <is>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D75" s="31" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E75" s="27" t="inlineStr"/>
+      <c r="F75" s="32">
+        <f>-Supuestos!B7</f>
+        <v/>
+      </c>
+      <c r="G75" s="30">
+        <f>G74+F75</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="25" t="n">
+        <v>46659</v>
+      </c>
+      <c r="B76" s="26">
+        <f>DATE(YEAR(A76),MONTH(A76),1)</f>
+        <v/>
+      </c>
+      <c r="C76" s="27" t="inlineStr">
+        <is>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D76" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E76" s="27" t="inlineStr"/>
+      <c r="F76" s="29" t="n">
+        <v>3173.56</v>
+      </c>
+      <c r="G76" s="30">
+        <f>G75+F76</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="25" t="n">
+        <v>46661</v>
+      </c>
+      <c r="B77" s="26">
+        <f>DATE(YEAR(A77),MONTH(A77),1)</f>
+        <v/>
+      </c>
+      <c r="C77" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D77" s="28" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E77" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F77" s="29" t="n">
+        <v>-229.39</v>
+      </c>
+      <c r="G77" s="30">
+        <f>G76+F77</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="25" t="n">
+        <v>46661</v>
+      </c>
+      <c r="B78" s="26">
+        <f>DATE(YEAR(A78),MONTH(A78),1)</f>
+        <v/>
+      </c>
+      <c r="C78" s="27" t="inlineStr">
+        <is>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D78" s="31" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E78" s="27" t="inlineStr"/>
+      <c r="F78" s="32">
+        <f>-Supuestos!B7</f>
+        <v/>
+      </c>
+      <c r="G78" s="30">
+        <f>G77+F78</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="25" t="n">
+        <v>46689</v>
+      </c>
+      <c r="B79" s="26">
+        <f>DATE(YEAR(A79),MONTH(A79),1)</f>
+        <v/>
+      </c>
+      <c r="C79" s="27" t="inlineStr">
+        <is>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D79" s="33" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E79" s="27" t="inlineStr"/>
+      <c r="F79" s="29" t="n">
+        <v>2490.44</v>
+      </c>
+      <c r="G79" s="30">
+        <f>G78+F79</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G72"/>
-  <conditionalFormatting sqref="G2:G72">
+  <autoFilter ref="A1:G79"/>
+  <conditionalFormatting sqref="G2:G79">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="1">
       <formula>0</formula>
     </cfRule>
@@ -4181,11 +4374,11 @@
         </is>
       </c>
       <c r="B6" s="41" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>Estimación: para llegar al 1 nov sin volver a pedir, máximo ~390 €</t>
+          <t>Tras pagar Smartcredito te quedan 165 €: máximo disponible hasta la nómina</t>
         </is>
       </c>
     </row>
@@ -4236,14 +4429,14 @@
     <row r="12">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Aplazables sin coste: Pagolisto 1 y 2, Crédito Santander 1 y 2, Smartcredito y Vivus. No aplazables: Santander (préstamo) y Moneyman.</t>
+          <t>Aplazables (se pagan y se vuelven a pedir sin intereses): Pagolisto 1 y 2, Crédito Santander 1 y 2. No aplazables: Santander (préstamo), Moneyman, Vivus y Smartcredito.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Escenario: el 1 nov pagas Moneyman y lo vuelves a pedir (1.100 €) para pagar a Ama; el 29 nov liquidas Vivus por 1.500 €.</t>
+          <t>Escenario: hoy pagas Smartcredito; el 1 nov pagas Moneyman y lo vuelves a pedir (1.100 €) para pagar a Ama y la cuota de Vivus; el 29 nov liquidas el resto de Vivus. Aplazables: pagar y volver a pedir en nov y dic.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel: plan con puente de 600 € de Joserra (sin volver a pedir Moneyman ni Smartcredito)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JEd5Mo2HQL6TrpXUCZoFXP
</commit_message>
<xml_diff>
--- a/excel/plan_de_pagos.xlsx
+++ b/excel/plan_de_pagos.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Supuestos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Calendario'!$A$1:$G$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Calendario'!$A$1:$G$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -95,6 +95,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00DCFCE7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FDE2E2"/>
       </patternFill>
     </fill>
@@ -105,17 +110,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCFCE7"/>
+        <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -150,14 +150,14 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -176,10 +176,10 @@
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -289,7 +289,7 @@
     <author>Plan</author>
   </authors>
   <commentList>
-    <comment ref="I4" authorId="0" shapeId="0">
+    <comment ref="I3" authorId="0" shapeId="0">
       <text>
         <t>2.148 € (4 × 537) − 1.500 € de liquidación, según lo que te ofrece Vivus</t>
       </text>
@@ -653,23 +653,23 @@
         <v>46296</v>
       </c>
       <c r="B2" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A2)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A2)</f>
         <v/>
       </c>
       <c r="C2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A2)</f>
         <v/>
       </c>
       <c r="D2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A2)</f>
         <v/>
       </c>
       <c r="E2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A2)</f>
         <v/>
       </c>
       <c r="F2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A2)</f>
         <v/>
       </c>
       <c r="G2" s="3">
@@ -690,23 +690,23 @@
         <v>46327</v>
       </c>
       <c r="B3" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A3)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A3)</f>
         <v/>
       </c>
       <c r="C3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A3)</f>
         <v/>
       </c>
       <c r="D3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A3)</f>
         <v/>
       </c>
       <c r="E3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A3)</f>
         <v/>
       </c>
       <c r="F3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A3)</f>
         <v/>
       </c>
       <c r="G3" s="3">
@@ -727,23 +727,23 @@
         <v>46357</v>
       </c>
       <c r="B4" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A4)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A4)</f>
         <v/>
       </c>
       <c r="C4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A4)</f>
         <v/>
       </c>
       <c r="D4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A4)</f>
         <v/>
       </c>
       <c r="E4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A4)</f>
         <v/>
       </c>
       <c r="F4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A4)</f>
         <v/>
       </c>
       <c r="G4" s="3">
@@ -764,23 +764,23 @@
         <v>46388</v>
       </c>
       <c r="B5" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A5)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A5)</f>
         <v/>
       </c>
       <c r="C5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A5)</f>
         <v/>
       </c>
       <c r="D5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A5)</f>
         <v/>
       </c>
       <c r="E5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A5)</f>
         <v/>
       </c>
       <c r="F5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A5)</f>
         <v/>
       </c>
       <c r="G5" s="3">
@@ -801,23 +801,23 @@
         <v>46419</v>
       </c>
       <c r="B6" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A6)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A6)</f>
         <v/>
       </c>
       <c r="C6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A6)</f>
         <v/>
       </c>
       <c r="D6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A6)</f>
         <v/>
       </c>
       <c r="E6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A6)</f>
         <v/>
       </c>
       <c r="F6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A6)</f>
         <v/>
       </c>
       <c r="G6" s="3">
@@ -838,23 +838,23 @@
         <v>46447</v>
       </c>
       <c r="B7" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A7)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A7)</f>
         <v/>
       </c>
       <c r="C7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A7)</f>
         <v/>
       </c>
       <c r="D7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A7)</f>
         <v/>
       </c>
       <c r="E7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A7)</f>
         <v/>
       </c>
       <c r="F7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A7)</f>
         <v/>
       </c>
       <c r="G7" s="3">
@@ -875,23 +875,23 @@
         <v>46478</v>
       </c>
       <c r="B8" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A8)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A8)</f>
         <v/>
       </c>
       <c r="C8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A8)</f>
         <v/>
       </c>
       <c r="D8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A8)</f>
         <v/>
       </c>
       <c r="E8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A8)</f>
         <v/>
       </c>
       <c r="F8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A8)</f>
         <v/>
       </c>
       <c r="G8" s="3">
@@ -912,23 +912,23 @@
         <v>46508</v>
       </c>
       <c r="B9" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A9)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A9)</f>
         <v/>
       </c>
       <c r="C9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A9)</f>
         <v/>
       </c>
       <c r="D9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A9)</f>
         <v/>
       </c>
       <c r="E9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A9)</f>
         <v/>
       </c>
       <c r="F9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A9)</f>
         <v/>
       </c>
       <c r="G9" s="3">
@@ -949,23 +949,23 @@
         <v>46539</v>
       </c>
       <c r="B10" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A10)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A10)</f>
         <v/>
       </c>
       <c r="C10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A10)</f>
         <v/>
       </c>
       <c r="D10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A10)</f>
         <v/>
       </c>
       <c r="E10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A10)</f>
         <v/>
       </c>
       <c r="F10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A10)</f>
         <v/>
       </c>
       <c r="G10" s="3">
@@ -986,23 +986,23 @@
         <v>46569</v>
       </c>
       <c r="B11" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A11)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A11)</f>
         <v/>
       </c>
       <c r="C11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A11)</f>
         <v/>
       </c>
       <c r="D11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A11)</f>
         <v/>
       </c>
       <c r="E11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A11)</f>
         <v/>
       </c>
       <c r="F11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A11)</f>
         <v/>
       </c>
       <c r="G11" s="3">
@@ -1023,23 +1023,23 @@
         <v>46600</v>
       </c>
       <c r="B12" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A12)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A12)</f>
         <v/>
       </c>
       <c r="C12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A12)</f>
         <v/>
       </c>
       <c r="D12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A12)</f>
         <v/>
       </c>
       <c r="E12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A12)</f>
         <v/>
       </c>
       <c r="F12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A12)</f>
         <v/>
       </c>
       <c r="G12" s="3">
@@ -1060,23 +1060,23 @@
         <v>46631</v>
       </c>
       <c r="B13" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A13)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A13)</f>
         <v/>
       </c>
       <c r="C13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A13)</f>
         <v/>
       </c>
       <c r="D13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A13)</f>
         <v/>
       </c>
       <c r="E13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A13)</f>
         <v/>
       </c>
       <c r="F13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A13)</f>
         <v/>
       </c>
       <c r="G13" s="3">
@@ -1097,23 +1097,23 @@
         <v>46661</v>
       </c>
       <c r="B14" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Ingreso",Calendario!$B$3:$B$79,A14)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A14)</f>
         <v/>
       </c>
       <c r="C14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Gasto",Calendario!$B$3:$B$79,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A14)</f>
         <v/>
       </c>
       <c r="D14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Fijo",Calendario!$B$3:$B$79,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A14)</f>
         <v/>
       </c>
       <c r="E14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Aplazable",Calendario!$B$3:$B$79,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A14)</f>
         <v/>
       </c>
       <c r="F14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$D$3:$D$79,"Amigo",Calendario!$B$3:$B$79,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A14)</f>
         <v/>
       </c>
       <c r="G14" s="3">
@@ -1171,7 +1171,7 @@
         </is>
       </c>
       <c r="C17" s="4">
-        <f>MIN(Calendario!G2:G79)</f>
+        <f>MIN(Calendario!G2:G73)</f>
         <v/>
       </c>
     </row>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="C18" s="7">
-        <f>INDEX(Calendario!A2:A79,MATCH(C17,Calendario!G2:G79,0))</f>
+        <f>INDEX(Calendario!A2:A73,MATCH(C17,Calendario!G2:G73,0))</f>
         <v/>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1283,7 +1283,7 @@
         <v>1400</v>
       </c>
       <c r="E2" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A2)</f>
         <v/>
       </c>
       <c r="F2" s="3">
@@ -1291,12 +1291,12 @@
         <v/>
       </c>
       <c r="G2" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A2)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A2)</f>
         <v/>
       </c>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>Pago único el 1 nov. Te dieron 1.100 €</t>
+          <t>Pago único el 1 nov, sin volver a pedirlo. Te dieron 1.100 €</t>
         </is>
       </c>
       <c r="I2" s="10" t="n">
@@ -1306,7 +1306,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Moneyman (vuelto a pedir)</t>
+          <t>Vivus</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
@@ -1316,14 +1316,14 @@
       </c>
       <c r="C3" s="9" t="inlineStr">
         <is>
-          <t>Moneyman</t>
+          <t>Vivus</t>
         </is>
       </c>
       <c r="D3" s="10" t="n">
-        <v>1400</v>
+        <v>2148</v>
       </c>
       <c r="E3" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A3)</f>
         <v/>
       </c>
       <c r="F3" s="3">
@@ -1331,22 +1331,22 @@
         <v/>
       </c>
       <c r="G3" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A3)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A3)</f>
         <v/>
       </c>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>Nace el 1 nov: recibes 1.100 €, devuelves 1.400 € el 1 dic</t>
+          <t>4 × 537 €, no aplazable. Plan: cuota del 1 nov y liquidar el resto el 29 nov (total 1.500 €)</t>
         </is>
       </c>
       <c r="I3" s="10" t="n">
-        <v>0</v>
+        <v>648</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Vivus</t>
+          <t>Smartcredito</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -1356,14 +1356,14 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>Vivus</t>
+          <t>Smartcredito</t>
         </is>
       </c>
       <c r="D4" s="10" t="n">
-        <v>2148</v>
+        <v>435</v>
       </c>
       <c r="E4" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A4)</f>
         <v/>
       </c>
       <c r="F4" s="3">
@@ -1371,22 +1371,22 @@
         <v/>
       </c>
       <c r="G4" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A4)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A4)</f>
         <v/>
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>4 × 537 €, no aplazable. Plan: cuota del 1 nov y liquidar el resto el 29 nov (total 1.500 €)</t>
+          <t>Pago único hoy (13 oct). Volver a pedirlo cuesta: recibes 300 €, devuelves 435 €</t>
         </is>
       </c>
       <c r="I4" s="10" t="n">
-        <v>648</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Smartcredito</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
@@ -1396,14 +1396,14 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>Smartcredito</t>
+          <t>Santander</t>
         </is>
       </c>
       <c r="D5" s="10" t="n">
-        <v>435</v>
+        <v>1994.93</v>
       </c>
       <c r="E5" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A5)</f>
         <v/>
       </c>
       <c r="F5" s="3">
@@ -1411,12 +1411,12 @@
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A5)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A5)</f>
         <v/>
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t>Pago único hoy (13 oct). Volver a pedirlo cuesta: recibes 300 €, devuelves 435 €</t>
+          <t>96 €/mes; desde mar 2027 dentro de los 500 €/mes</t>
         </is>
       </c>
       <c r="I5" s="10" t="n">
@@ -1426,24 +1426,24 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Pagolisto 1</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Santander</t>
+          <t>Pagolisto *6284</t>
         </is>
       </c>
       <c r="D6" s="10" t="n">
-        <v>1994.93</v>
+        <v>693.34</v>
       </c>
       <c r="E6" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A6)</f>
         <v/>
       </c>
       <c r="F6" s="3">
@@ -1451,12 +1451,12 @@
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A6)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A6)</f>
         <v/>
       </c>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>96 €/mes; desde abr 2027 dentro de los 500 €/mes</t>
+          <t>Aplazable: en nov pagas la cuota y la vuelves a pedir sin intereses; 3 cuotas dic–feb</t>
         </is>
       </c>
       <c r="I6" s="10" t="n">
@@ -1466,7 +1466,7 @@
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Pagolisto 1</t>
+          <t>Pagolisto 2</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
@@ -1476,14 +1476,14 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Pagolisto *6284</t>
+          <t>Pagolisto *6727</t>
         </is>
       </c>
       <c r="D7" s="10" t="n">
-        <v>693.34</v>
+        <v>923.61</v>
       </c>
       <c r="E7" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A7)</f>
         <v/>
       </c>
       <c r="F7" s="3">
@@ -1491,12 +1491,12 @@
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A7)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A7)</f>
         <v/>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Aplazable: en nov y dic pagas la cuota y la vuelves a pedir sin intereses; 3 cuotas ene–mar</t>
+          <t>Aplazable: en nov pagas la cuota y la vuelves a pedir sin intereses; 3 cuotas dic–feb</t>
         </is>
       </c>
       <c r="I7" s="10" t="n">
@@ -1506,7 +1506,7 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Pagolisto 2</t>
+          <t>Crédito Santander 1</t>
         </is>
       </c>
       <c r="B8" s="14" t="inlineStr">
@@ -1516,14 +1516,14 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Pagolisto *6727</t>
+          <t>Santander *0773</t>
         </is>
       </c>
       <c r="D8" s="10" t="n">
-        <v>923.61</v>
+        <v>1483.63</v>
       </c>
       <c r="E8" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A8)</f>
         <v/>
       </c>
       <c r="F8" s="3">
@@ -1531,12 +1531,12 @@
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A8)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A8)</f>
         <v/>
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>Aplazable: en nov y dic pagas la cuota y la vuelves a pedir sin intereses; 3 cuotas ene–mar</t>
+          <t>Aplazable: en nov pagas la cuota y la vuelves a pedir sin intereses; 3 cuotas dic–feb</t>
         </is>
       </c>
       <c r="I8" s="10" t="n">
@@ -1546,7 +1546,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Crédito Santander 1</t>
+          <t>Crédito Santander 2</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr">
@@ -1556,14 +1556,14 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>Santander *0773</t>
+          <t>Santander *4475</t>
         </is>
       </c>
       <c r="D9" s="10" t="n">
-        <v>1483.63</v>
+        <v>2326.76</v>
       </c>
       <c r="E9" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A9)</f>
         <v/>
       </c>
       <c r="F9" s="3">
@@ -1571,12 +1571,12 @@
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A9)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A9)</f>
         <v/>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Aplazable: en nov y dic pagas la cuota y la vuelves a pedir sin intereses; 3 cuotas ene–mar</t>
+          <t>122,46 €/mes; desde mar 2027 dentro de los 500 €/mes</t>
         </is>
       </c>
       <c r="I9" s="10" t="n">
@@ -1586,24 +1586,24 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Ama</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Santander *4475</t>
+          <t>Ama</t>
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>2326.76</v>
+        <v>600</v>
       </c>
       <c r="E10" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A10)</f>
         <v/>
       </c>
       <c r="F10" s="3">
@@ -1611,12 +1611,12 @@
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A10)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A10)</f>
         <v/>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>122,46 €/mes; desde abr 2027 dentro de los 500 €/mes</t>
+          <t>Prioridad: 29 nov, con la nómina</t>
         </is>
       </c>
       <c r="I10" s="10" t="n">
@@ -1626,7 +1626,7 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Ama</t>
+          <t>Joserra</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
@@ -1636,14 +1636,14 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>Ama</t>
+          <t>Joserra</t>
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>600</v>
+        <v>1000</v>
       </c>
       <c r="E11" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A11)</f>
         <v/>
       </c>
       <c r="F11" s="3">
@@ -1651,12 +1651,12 @@
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A11)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A11)</f>
         <v/>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>Prioridad: 1 nov, con lo que vuelves a pedir a Moneyman</t>
+          <t>400 € anteriores + 600 € de puente el 13 oct. Se devuelve todo antes de fin de año</t>
         </is>
       </c>
       <c r="I11" s="10" t="n">
@@ -1666,7 +1666,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Joserra</t>
+          <t>Xabi</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
@@ -1676,14 +1676,14 @@
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Joserra</t>
+          <t>Xabi</t>
         </is>
       </c>
       <c r="D12" s="10" t="n">
-        <v>400</v>
+        <v>300</v>
       </c>
       <c r="E12" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A12)</f>
         <v/>
       </c>
       <c r="F12" s="3">
@@ -1691,7 +1691,7 @@
         <v/>
       </c>
       <c r="G12" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A12)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A12)</f>
         <v/>
       </c>
       <c r="H12" s="13" t="inlineStr">
@@ -1706,7 +1706,7 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Xabi</t>
+          <t>Sergio</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
@@ -1716,14 +1716,14 @@
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>Xabi</t>
+          <t>Sergio</t>
         </is>
       </c>
       <c r="D13" s="10" t="n">
-        <v>300</v>
+        <v>1700</v>
       </c>
       <c r="E13" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A13)</f>
         <v/>
       </c>
       <c r="F13" s="3">
@@ -1731,7 +1731,7 @@
         <v/>
       </c>
       <c r="G13" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A13)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A13)</f>
         <v/>
       </c>
       <c r="H13" s="13" t="inlineStr">
@@ -1746,7 +1746,7 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Sergio</t>
+          <t>Txomin</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
@@ -1756,14 +1756,14 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Sergio</t>
+          <t>Txomin</t>
         </is>
       </c>
       <c r="D14" s="10" t="n">
-        <v>1700</v>
+        <v>2500</v>
       </c>
       <c r="E14" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A14)</f>
         <v/>
       </c>
       <c r="F14" s="3">
@@ -1771,7 +1771,7 @@
         <v/>
       </c>
       <c r="G14" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A14)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A14)</f>
         <v/>
       </c>
       <c r="H14" s="13" t="inlineStr">
@@ -1784,116 +1784,76 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Txomin</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="n"/>
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="6">
+        <f>SUM(D2:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="6">
+        <f>SUM(E2:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="6">
+        <f>SUM(F2:F14)</f>
+        <v/>
+      </c>
+      <c r="G15" s="18">
+        <f>MAX(G2:G14)</f>
+        <v/>
+      </c>
+      <c r="H15" s="19" t="inlineStr">
+        <is>
+          <t>← libre de deudas</t>
+        </is>
+      </c>
+      <c r="I15" s="6">
+        <f>SUM(I2:I14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Por bloque</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="D18" s="3">
+        <f>SUMIFS(D2:D14,B2:B14,A18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="D19" s="3">
+        <f>SUMIFS(D2:D14,B2:B14,A19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>Amigo</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>Txomin</t>
-        </is>
-      </c>
-      <c r="D15" s="10" t="n">
-        <v>2500</v>
-      </c>
-      <c r="E15" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$79,Calendario!$E$3:$E$79,A15)</f>
-        <v/>
-      </c>
-      <c r="F15" s="3">
-        <f>D15-E15-I15</f>
-        <v/>
-      </c>
-      <c r="G15" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$79,Calendario!$E$3:$E$79,A15)</f>
-        <v/>
-      </c>
-      <c r="H15" s="13" t="inlineStr">
-        <is>
-          <t>Sin plazo ni interés</t>
-        </is>
-      </c>
-      <c r="I15" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B16" s="17" t="n"/>
-      <c r="C16" s="17" t="n"/>
-      <c r="D16" s="6">
-        <f>SUM(D2:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="6">
-        <f>SUM(E2:E15)</f>
-        <v/>
-      </c>
-      <c r="F16" s="6">
-        <f>SUM(F2:F15)</f>
-        <v/>
-      </c>
-      <c r="G16" s="18">
-        <f>MAX(G2:G15)</f>
-        <v/>
-      </c>
-      <c r="H16" s="19" t="inlineStr">
-        <is>
-          <t>← libre de deudas</t>
-        </is>
-      </c>
-      <c r="I16" s="6">
-        <f>SUM(I2:I15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>Por bloque</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="D19" s="3">
-        <f>SUMIFS(D2:D15,B2:B15,A19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
       <c r="D20" s="3">
-        <f>SUMIFS(D2:D15,B2:B15,A20)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>Amigo</t>
-        </is>
-      </c>
-      <c r="D21" s="3">
-        <f>SUMIFS(D2:D15,B2:B15,A21)</f>
+        <f>SUMIFS(D2:D14,B2:B14,A20)</f>
         <v/>
       </c>
     </row>
@@ -1909,7 +1869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J79"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2007,21 +1967,17 @@
       </c>
       <c r="C3" s="27" t="inlineStr">
         <is>
-          <t>Smartcredito · pago hoy</t>
+          <t>Préstamo puente de Joserra (sin intereses)</t>
         </is>
       </c>
       <c r="D3" s="28" t="inlineStr">
         <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E3" s="27" t="inlineStr">
-        <is>
-          <t>Smartcredito</t>
-        </is>
-      </c>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E3" s="27" t="inlineStr"/>
       <c r="F3" s="29" t="n">
-        <v>-435</v>
+        <v>600</v>
       </c>
       <c r="G3" s="30">
         <f>G2+F3</f>
@@ -2040,7 +1996,7 @@
     </row>
     <row r="4">
       <c r="A4" s="25" t="n">
-        <v>46309</v>
+        <v>46308</v>
       </c>
       <c r="B4" s="26">
         <f>DATE(YEAR(A4),MONTH(A4),1)</f>
@@ -2048,18 +2004,21 @@
       </c>
       <c r="C4" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida hasta el 29 oct (estimado)</t>
+          <t>Smartcredito · pago hoy</t>
         </is>
       </c>
       <c r="D4" s="31" t="inlineStr">
         <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E4" s="27" t="inlineStr"/>
-      <c r="F4" s="32">
-        <f>-Supuestos!B6</f>
-        <v/>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr">
+        <is>
+          <t>Smartcredito</t>
+        </is>
+      </c>
+      <c r="F4" s="29" t="n">
+        <v>-435</v>
       </c>
       <c r="G4" s="30">
         <f>G3+F4</f>
@@ -2078,7 +2037,7 @@
     </row>
     <row r="5">
       <c r="A5" s="25" t="n">
-        <v>46324</v>
+        <v>46309</v>
       </c>
       <c r="B5" s="26">
         <f>DATE(YEAR(A5),MONTH(A5),1)</f>
@@ -2086,17 +2045,18 @@
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D5" s="33" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Gastos de vida hasta el 29 oct (estimado)</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="inlineStr">
+        <is>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E5" s="27" t="inlineStr"/>
-      <c r="F5" s="29" t="n">
-        <v>2645.44</v>
+      <c r="F5" s="33">
+        <f>-Supuestos!B6</f>
+        <v/>
       </c>
       <c r="G5" s="30">
         <f>G4+F5</f>
@@ -2115,7 +2075,7 @@
     </row>
     <row r="6">
       <c r="A6" s="25" t="n">
-        <v>46327</v>
+        <v>46324</v>
       </c>
       <c r="B6" s="26">
         <f>DATE(YEAR(A6),MONTH(A6),1)</f>
@@ -2123,17 +2083,17 @@
       </c>
       <c r="C6" s="27" t="inlineStr">
         <is>
-          <t>Moneyman: vuelvo a pedir (recibo 1.100 €)</t>
-        </is>
-      </c>
-      <c r="D6" s="33" t="inlineStr">
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
       </c>
       <c r="E6" s="27" t="inlineStr"/>
       <c r="F6" s="29" t="n">
-        <v>1100</v>
+        <v>2645.44</v>
       </c>
       <c r="G6" s="30">
         <f>G5+F6</f>
@@ -2160,10 +2120,10 @@
       </c>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>Moneyman</t>
-        </is>
-      </c>
-      <c r="D7" s="28" t="inlineStr">
+          <t>Moneyman · pago (sin volver a pedirlo)</t>
+        </is>
+      </c>
+      <c r="D7" s="31" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
@@ -2191,21 +2151,21 @@
       </c>
       <c r="C8" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Ama</t>
-        </is>
-      </c>
-      <c r="D8" s="36" t="inlineStr">
-        <is>
-          <t>Amigo</t>
+          <t>Vivus · cuota 1/4 (no aplazable)</t>
+        </is>
+      </c>
+      <c r="D8" s="31" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E8" s="27" t="inlineStr">
         <is>
-          <t>Ama</t>
+          <t>Vivus</t>
         </is>
       </c>
       <c r="F8" s="29" t="n">
-        <v>-600</v>
+        <v>-537</v>
       </c>
       <c r="G8" s="30">
         <f>G7+F8</f>
@@ -2227,21 +2187,17 @@
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>Vivus · cuota 1/4 (no aplazable)</t>
-        </is>
-      </c>
-      <c r="D9" s="28" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E9" s="27" t="inlineStr">
-        <is>
-          <t>Vivus</t>
-        </is>
-      </c>
+          <t>Pagolisto 1 · pagas 231,11 € y lo vuelves a pedir (neto 0)</t>
+        </is>
+      </c>
+      <c r="D9" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr"/>
       <c r="F9" s="29" t="n">
-        <v>-537</v>
+        <v>0</v>
       </c>
       <c r="G9" s="30">
         <f>G8+F9</f>
@@ -2258,10 +2214,10 @@
       </c>
       <c r="C10" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · pagas 231,11 € y lo vuelves a pedir (neto 0)</t>
-        </is>
-      </c>
-      <c r="D10" s="37" t="inlineStr">
+          <t>Pagolisto 2 · pagas 307,87 € y lo vuelves a pedir (neto 0)</t>
+        </is>
+      </c>
+      <c r="D10" s="36" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
@@ -2285,10 +2241,10 @@
       </c>
       <c r="C11" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · pagas 307,87 € y lo vuelves a pedir (neto 0)</t>
-        </is>
-      </c>
-      <c r="D11" s="37" t="inlineStr">
+          <t>Crédito Santander 1 · pagas 494,54 € y lo vuelves a pedir (neto 0)</t>
+        </is>
+      </c>
+      <c r="D11" s="36" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
@@ -2312,17 +2268,21 @@
       </c>
       <c r="C12" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · pagas 494,54 € y lo vuelves a pedir (neto 0)</t>
-        </is>
-      </c>
-      <c r="D12" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E12" s="27" t="inlineStr"/>
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D12" s="31" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E12" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
       <c r="F12" s="29" t="n">
-        <v>0</v>
+        <v>-96</v>
       </c>
       <c r="G12" s="30">
         <f>G11+F12</f>
@@ -2339,21 +2299,21 @@
       </c>
       <c r="C13" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D13" s="28" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D13" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E13" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Crédito Santander 2</t>
         </is>
       </c>
       <c r="F13" s="29" t="n">
-        <v>-96</v>
+        <v>-122.46</v>
       </c>
       <c r="G13" s="30">
         <f>G12+F13</f>
@@ -2370,21 +2330,18 @@
       </c>
       <c r="C14" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
-        </is>
-      </c>
-      <c r="D14" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E14" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F14" s="29" t="n">
-        <v>-122.46</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E14" s="27" t="inlineStr"/>
+      <c r="F14" s="33">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G14" s="30">
         <f>G13+F14</f>
@@ -2393,7 +2350,7 @@
     </row>
     <row r="15">
       <c r="A15" s="25" t="n">
-        <v>46327</v>
+        <v>46355</v>
       </c>
       <c r="B15" s="26">
         <f>DATE(YEAR(A15),MONTH(A15),1)</f>
@@ -2401,18 +2358,17 @@
       </c>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D15" s="31" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D15" s="28" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E15" s="27" t="inlineStr"/>
-      <c r="F15" s="32">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F15" s="29" t="n">
+        <v>3453.01</v>
       </c>
       <c r="G15" s="30">
         <f>G14+F15</f>
@@ -2429,17 +2385,21 @@
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D16" s="33" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E16" s="27" t="inlineStr"/>
+          <t>Vivus · liquidación del resto (total 1.500 € en vez de 2.148 €)</t>
+        </is>
+      </c>
+      <c r="D16" s="31" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E16" s="27" t="inlineStr">
+        <is>
+          <t>Vivus</t>
+        </is>
+      </c>
       <c r="F16" s="29" t="n">
-        <v>3453.01</v>
+        <v>-963</v>
       </c>
       <c r="G16" s="30">
         <f>G15+F16</f>
@@ -2456,21 +2416,21 @@
       </c>
       <c r="C17" s="27" t="inlineStr">
         <is>
-          <t>Vivus · liquidación del resto (total 1.500 € en vez de 2.148 €)</t>
-        </is>
-      </c>
-      <c r="D17" s="28" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Devolución a Ama</t>
+        </is>
+      </c>
+      <c r="D17" s="37" t="inlineStr">
+        <is>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E17" s="27" t="inlineStr">
         <is>
-          <t>Vivus</t>
+          <t>Ama</t>
         </is>
       </c>
       <c r="F17" s="29" t="n">
-        <v>-963</v>
+        <v>-600</v>
       </c>
       <c r="G17" s="30">
         <f>G16+F17</f>
@@ -2487,17 +2447,21 @@
       </c>
       <c r="C18" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · pagas 231,11 € y lo vuelves a pedir (neto 0)</t>
-        </is>
-      </c>
-      <c r="D18" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E18" s="27" t="inlineStr"/>
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D18" s="31" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E18" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
       <c r="F18" s="29" t="n">
-        <v>0</v>
+        <v>-96</v>
       </c>
       <c r="G18" s="30">
         <f>G17+F18</f>
@@ -2514,17 +2478,21 @@
       </c>
       <c r="C19" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · pagas 307,87 € y lo vuelves a pedir (neto 0)</t>
-        </is>
-      </c>
-      <c r="D19" s="37" t="inlineStr">
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D19" s="36" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
-      <c r="E19" s="27" t="inlineStr"/>
+      <c r="E19" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
       <c r="F19" s="29" t="n">
-        <v>0</v>
+        <v>-122.46</v>
       </c>
       <c r="G19" s="30">
         <f>G18+F19</f>
@@ -2541,17 +2509,21 @@
       </c>
       <c r="C20" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · pagas 494,54 € y lo vuelves a pedir (neto 0)</t>
-        </is>
-      </c>
-      <c r="D20" s="37" t="inlineStr">
+          <t>Pagolisto 1 · cuota 1/3</t>
+        </is>
+      </c>
+      <c r="D20" s="36" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
-      <c r="E20" s="27" t="inlineStr"/>
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>Pagolisto 1</t>
+        </is>
+      </c>
       <c r="F20" s="29" t="n">
-        <v>0</v>
+        <v>-231.11</v>
       </c>
       <c r="G20" s="30">
         <f>G19+F20</f>
@@ -2568,21 +2540,21 @@
       </c>
       <c r="C21" s="27" t="inlineStr">
         <is>
-          <t>Moneyman (vuelto a pedir)</t>
-        </is>
-      </c>
-      <c r="D21" s="28" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Pagolisto 2 · cuota 1/3</t>
+        </is>
+      </c>
+      <c r="D21" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E21" s="27" t="inlineStr">
         <is>
-          <t>Moneyman (vuelto a pedir)</t>
+          <t>Pagolisto 2</t>
         </is>
       </c>
       <c r="F21" s="29" t="n">
-        <v>-1400</v>
+        <v>-307.87</v>
       </c>
       <c r="G21" s="30">
         <f>G20+F21</f>
@@ -2599,21 +2571,21 @@
       </c>
       <c r="C22" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D22" s="28" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 1 · cuota 1/3</t>
+        </is>
+      </c>
+      <c r="D22" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E22" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Crédito Santander 1</t>
         </is>
       </c>
       <c r="F22" s="29" t="n">
-        <v>-96</v>
+        <v>-494.54</v>
       </c>
       <c r="G22" s="30">
         <f>G21+F22</f>
@@ -2630,21 +2602,18 @@
       </c>
       <c r="C23" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
-        </is>
-      </c>
-      <c r="D23" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E23" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F23" s="29" t="n">
-        <v>-122.46</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D23" s="32" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E23" s="27" t="inlineStr"/>
+      <c r="F23" s="33">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G23" s="30">
         <f>G22+F23</f>
@@ -2653,7 +2622,7 @@
     </row>
     <row r="24">
       <c r="A24" s="25" t="n">
-        <v>46357</v>
+        <v>46385</v>
       </c>
       <c r="B24" s="26">
         <f>DATE(YEAR(A24),MONTH(A24),1)</f>
@@ -2661,18 +2630,17 @@
       </c>
       <c r="C24" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D24" s="31" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D24" s="28" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E24" s="27" t="inlineStr"/>
-      <c r="F24" s="32">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F24" s="29" t="n">
+        <v>3453.01</v>
       </c>
       <c r="G24" s="30">
         <f>G23+F24</f>
@@ -2689,17 +2657,17 @@
       </c>
       <c r="C25" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D25" s="33" t="inlineStr">
+          <t>Paga extra de diciembre</t>
+        </is>
+      </c>
+      <c r="D25" s="28" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
       </c>
       <c r="E25" s="27" t="inlineStr"/>
       <c r="F25" s="29" t="n">
-        <v>3453.01</v>
+        <v>2014.69</v>
       </c>
       <c r="G25" s="30">
         <f>G24+F25</f>
@@ -2716,17 +2684,21 @@
       </c>
       <c r="C26" s="27" t="inlineStr">
         <is>
-          <t>Paga extra de diciembre</t>
-        </is>
-      </c>
-      <c r="D26" s="33" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E26" s="27" t="inlineStr"/>
+          <t>Devolución a Joserra (puente + lo anterior)</t>
+        </is>
+      </c>
+      <c r="D26" s="37" t="inlineStr">
+        <is>
+          <t>Amigo</t>
+        </is>
+      </c>
+      <c r="E26" s="27" t="inlineStr">
+        <is>
+          <t>Joserra</t>
+        </is>
+      </c>
       <c r="F26" s="29" t="n">
-        <v>2014.69</v>
+        <v>-1000</v>
       </c>
       <c r="G26" s="30">
         <f>G25+F26</f>
@@ -2746,7 +2718,7 @@
           <t>Santander (préstamo) · cuota</t>
         </is>
       </c>
-      <c r="D27" s="28" t="inlineStr">
+      <c r="D27" s="31" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
@@ -2777,7 +2749,7 @@
           <t>Crédito Santander 2 · cuota</t>
         </is>
       </c>
-      <c r="D28" s="37" t="inlineStr">
+      <c r="D28" s="36" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
@@ -2805,10 +2777,10 @@
       </c>
       <c r="C29" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 1/3</t>
-        </is>
-      </c>
-      <c r="D29" s="37" t="inlineStr">
+          <t>Pagolisto 1 · cuota 2/3</t>
+        </is>
+      </c>
+      <c r="D29" s="36" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
@@ -2836,10 +2808,10 @@
       </c>
       <c r="C30" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 1/3</t>
-        </is>
-      </c>
-      <c r="D30" s="37" t="inlineStr">
+          <t>Pagolisto 2 · cuota 2/3</t>
+        </is>
+      </c>
+      <c r="D30" s="36" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
@@ -2867,10 +2839,10 @@
       </c>
       <c r="C31" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 1/3</t>
-        </is>
-      </c>
-      <c r="D31" s="37" t="inlineStr">
+          <t>Crédito Santander 1 · cuota 2/3</t>
+        </is>
+      </c>
+      <c r="D31" s="36" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
@@ -2898,21 +2870,21 @@
       </c>
       <c r="C32" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Joserra</t>
-        </is>
-      </c>
-      <c r="D32" s="36" t="inlineStr">
+          <t>Devolución a Xabi</t>
+        </is>
+      </c>
+      <c r="D32" s="37" t="inlineStr">
         <is>
           <t>Amigo</t>
         </is>
       </c>
       <c r="E32" s="27" t="inlineStr">
         <is>
-          <t>Joserra</t>
+          <t>Xabi</t>
         </is>
       </c>
       <c r="F32" s="29" t="n">
-        <v>-400</v>
+        <v>-300</v>
       </c>
       <c r="G32" s="30">
         <f>G31+F32</f>
@@ -2929,21 +2901,18 @@
       </c>
       <c r="C33" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Xabi</t>
-        </is>
-      </c>
-      <c r="D33" s="36" t="inlineStr">
-        <is>
-          <t>Amigo</t>
-        </is>
-      </c>
-      <c r="E33" s="27" t="inlineStr">
-        <is>
-          <t>Xabi</t>
-        </is>
-      </c>
-      <c r="F33" s="29" t="n">
-        <v>-300</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D33" s="32" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E33" s="27" t="inlineStr"/>
+      <c r="F33" s="33">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G33" s="30">
         <f>G32+F33</f>
@@ -2952,7 +2921,7 @@
     </row>
     <row r="34">
       <c r="A34" s="25" t="n">
-        <v>46388</v>
+        <v>46416</v>
       </c>
       <c r="B34" s="26">
         <f>DATE(YEAR(A34),MONTH(A34),1)</f>
@@ -2960,18 +2929,17 @@
       </c>
       <c r="C34" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D34" s="31" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D34" s="28" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E34" s="27" t="inlineStr"/>
-      <c r="F34" s="32">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F34" s="29" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G34" s="30">
         <f>G33+F34</f>
@@ -2980,7 +2948,7 @@
     </row>
     <row r="35">
       <c r="A35" s="25" t="n">
-        <v>46416</v>
+        <v>46419</v>
       </c>
       <c r="B35" s="26">
         <f>DATE(YEAR(A35),MONTH(A35),1)</f>
@@ -2988,17 +2956,21 @@
       </c>
       <c r="C35" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D35" s="33" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E35" s="27" t="inlineStr"/>
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D35" s="31" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E35" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
       <c r="F35" s="29" t="n">
-        <v>3173.56</v>
+        <v>-96</v>
       </c>
       <c r="G35" s="30">
         <f>G34+F35</f>
@@ -3015,21 +2987,21 @@
       </c>
       <c r="C36" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D36" s="28" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D36" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E36" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Crédito Santander 2</t>
         </is>
       </c>
       <c r="F36" s="29" t="n">
-        <v>-96</v>
+        <v>-122.46</v>
       </c>
       <c r="G36" s="30">
         <f>G35+F36</f>
@@ -3046,21 +3018,21 @@
       </c>
       <c r="C37" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
-        </is>
-      </c>
-      <c r="D37" s="37" t="inlineStr">
+          <t>Pagolisto 1 · cuota 3/3</t>
+        </is>
+      </c>
+      <c r="D37" s="36" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E37" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Pagolisto 1</t>
         </is>
       </c>
       <c r="F37" s="29" t="n">
-        <v>-122.46</v>
+        <v>-231.12</v>
       </c>
       <c r="G37" s="30">
         <f>G36+F37</f>
@@ -3077,21 +3049,21 @@
       </c>
       <c r="C38" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 2/3</t>
-        </is>
-      </c>
-      <c r="D38" s="37" t="inlineStr">
+          <t>Pagolisto 2 · cuota 3/3</t>
+        </is>
+      </c>
+      <c r="D38" s="36" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E38" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1</t>
+          <t>Pagolisto 2</t>
         </is>
       </c>
       <c r="F38" s="29" t="n">
-        <v>-231.11</v>
+        <v>-307.87</v>
       </c>
       <c r="G38" s="30">
         <f>G37+F38</f>
@@ -3108,21 +3080,21 @@
       </c>
       <c r="C39" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 2/3</t>
-        </is>
-      </c>
-      <c r="D39" s="37" t="inlineStr">
+          <t>Crédito Santander 1 · cuota 3/3</t>
+        </is>
+      </c>
+      <c r="D39" s="36" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E39" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2</t>
+          <t>Crédito Santander 1</t>
         </is>
       </c>
       <c r="F39" s="29" t="n">
-        <v>-307.87</v>
+        <v>-494.55</v>
       </c>
       <c r="G39" s="30">
         <f>G38+F39</f>
@@ -3139,21 +3111,21 @@
       </c>
       <c r="C40" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 2/3</t>
+          <t>Devolución a Sergio</t>
         </is>
       </c>
       <c r="D40" s="37" t="inlineStr">
         <is>
-          <t>Aplazable</t>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E40" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1</t>
+          <t>Sergio</t>
         </is>
       </c>
       <c r="F40" s="29" t="n">
-        <v>-494.54</v>
+        <v>-1700</v>
       </c>
       <c r="G40" s="30">
         <f>G39+F40</f>
@@ -3170,21 +3142,18 @@
       </c>
       <c r="C41" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Sergio</t>
-        </is>
-      </c>
-      <c r="D41" s="36" t="inlineStr">
-        <is>
-          <t>Amigo</t>
-        </is>
-      </c>
-      <c r="E41" s="27" t="inlineStr">
-        <is>
-          <t>Sergio</t>
-        </is>
-      </c>
-      <c r="F41" s="29" t="n">
-        <v>-1700</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D41" s="32" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E41" s="27" t="inlineStr"/>
+      <c r="F41" s="33">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G41" s="30">
         <f>G40+F41</f>
@@ -3193,7 +3162,7 @@
     </row>
     <row r="42">
       <c r="A42" s="25" t="n">
-        <v>46419</v>
+        <v>46446</v>
       </c>
       <c r="B42" s="26">
         <f>DATE(YEAR(A42),MONTH(A42),1)</f>
@@ -3201,18 +3170,17 @@
       </c>
       <c r="C42" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D42" s="31" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D42" s="28" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E42" s="27" t="inlineStr"/>
-      <c r="F42" s="32">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F42" s="29" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G42" s="30">
         <f>G41+F42</f>
@@ -3229,17 +3197,17 @@
       </c>
       <c r="C43" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D43" s="33" t="inlineStr">
+          <t>Variable de febrero</t>
+        </is>
+      </c>
+      <c r="D43" s="28" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
       </c>
       <c r="E43" s="27" t="inlineStr"/>
       <c r="F43" s="29" t="n">
-        <v>3173.56</v>
+        <v>2114.45</v>
       </c>
       <c r="G43" s="30">
         <f>G42+F43</f>
@@ -3256,17 +3224,21 @@
       </c>
       <c r="C44" s="27" t="inlineStr">
         <is>
-          <t>Variable de febrero</t>
-        </is>
-      </c>
-      <c r="D44" s="33" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E44" s="27" t="inlineStr"/>
+          <t>Devolución a Txomin</t>
+        </is>
+      </c>
+      <c r="D44" s="37" t="inlineStr">
+        <is>
+          <t>Amigo</t>
+        </is>
+      </c>
+      <c r="E44" s="27" t="inlineStr">
+        <is>
+          <t>Txomin</t>
+        </is>
+      </c>
       <c r="F44" s="29" t="n">
-        <v>2114.45</v>
+        <v>-2500</v>
       </c>
       <c r="G44" s="30">
         <f>G43+F44</f>
@@ -3275,7 +3247,7 @@
     </row>
     <row r="45">
       <c r="A45" s="25" t="n">
-        <v>46446</v>
+        <v>46447</v>
       </c>
       <c r="B45" s="26">
         <f>DATE(YEAR(A45),MONTH(A45),1)</f>
@@ -3283,21 +3255,21 @@
       </c>
       <c r="C45" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Txomin</t>
-        </is>
-      </c>
-      <c r="D45" s="36" t="inlineStr">
-        <is>
-          <t>Amigo</t>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D45" s="31" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E45" s="27" t="inlineStr">
         <is>
-          <t>Txomin</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F45" s="29" t="n">
-        <v>-2500</v>
+        <v>-96</v>
       </c>
       <c r="G45" s="30">
         <f>G44+F45</f>
@@ -3314,21 +3286,21 @@
       </c>
       <c r="C46" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D46" s="28" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D46" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E46" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Crédito Santander 2</t>
         </is>
       </c>
       <c r="F46" s="29" t="n">
-        <v>-96</v>
+        <v>-404</v>
       </c>
       <c r="G46" s="30">
         <f>G45+F46</f>
@@ -3345,21 +3317,18 @@
       </c>
       <c r="C47" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
-        </is>
-      </c>
-      <c r="D47" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E47" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F47" s="29" t="n">
-        <v>-122.46</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D47" s="32" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E47" s="27" t="inlineStr"/>
+      <c r="F47" s="33">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G47" s="30">
         <f>G46+F47</f>
@@ -3368,7 +3337,7 @@
     </row>
     <row r="48">
       <c r="A48" s="25" t="n">
-        <v>46447</v>
+        <v>46475</v>
       </c>
       <c r="B48" s="26">
         <f>DATE(YEAR(A48),MONTH(A48),1)</f>
@@ -3376,21 +3345,17 @@
       </c>
       <c r="C48" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 3/3</t>
-        </is>
-      </c>
-      <c r="D48" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E48" s="27" t="inlineStr">
-        <is>
-          <t>Pagolisto 1</t>
-        </is>
-      </c>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D48" s="28" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E48" s="27" t="inlineStr"/>
       <c r="F48" s="29" t="n">
-        <v>-231.12</v>
+        <v>3173.56</v>
       </c>
       <c r="G48" s="30">
         <f>G47+F48</f>
@@ -3399,7 +3364,7 @@
     </row>
     <row r="49">
       <c r="A49" s="25" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="B49" s="26">
         <f>DATE(YEAR(A49),MONTH(A49),1)</f>
@@ -3407,21 +3372,21 @@
       </c>
       <c r="C49" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 3/3</t>
-        </is>
-      </c>
-      <c r="D49" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D49" s="31" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E49" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F49" s="29" t="n">
-        <v>-307.87</v>
+        <v>-96</v>
       </c>
       <c r="G49" s="30">
         <f>G48+F49</f>
@@ -3430,7 +3395,7 @@
     </row>
     <row r="50">
       <c r="A50" s="25" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="B50" s="26">
         <f>DATE(YEAR(A50),MONTH(A50),1)</f>
@@ -3438,21 +3403,21 @@
       </c>
       <c r="C50" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 3/3</t>
-        </is>
-      </c>
-      <c r="D50" s="37" t="inlineStr">
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D50" s="36" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E50" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1</t>
+          <t>Crédito Santander 2</t>
         </is>
       </c>
       <c r="F50" s="29" t="n">
-        <v>-494.55</v>
+        <v>-404</v>
       </c>
       <c r="G50" s="30">
         <f>G49+F50</f>
@@ -3461,7 +3426,7 @@
     </row>
     <row r="51">
       <c r="A51" s="25" t="n">
-        <v>46447</v>
+        <v>46478</v>
       </c>
       <c r="B51" s="26">
         <f>DATE(YEAR(A51),MONTH(A51),1)</f>
@@ -3472,13 +3437,13 @@
           <t>Gastos de vida</t>
         </is>
       </c>
-      <c r="D51" s="31" t="inlineStr">
+      <c r="D51" s="32" t="inlineStr">
         <is>
           <t>Gasto</t>
         </is>
       </c>
       <c r="E51" s="27" t="inlineStr"/>
-      <c r="F51" s="32">
+      <c r="F51" s="33">
         <f>-Supuestos!B7</f>
         <v/>
       </c>
@@ -3489,7 +3454,7 @@
     </row>
     <row r="52">
       <c r="A52" s="25" t="n">
-        <v>46475</v>
+        <v>46506</v>
       </c>
       <c r="B52" s="26">
         <f>DATE(YEAR(A52),MONTH(A52),1)</f>
@@ -3500,7 +3465,7 @@
           <t>Nómina</t>
         </is>
       </c>
-      <c r="D52" s="33" t="inlineStr">
+      <c r="D52" s="28" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
@@ -3516,7 +3481,7 @@
     </row>
     <row r="53">
       <c r="A53" s="25" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="B53" s="26">
         <f>DATE(YEAR(A53),MONTH(A53),1)</f>
@@ -3527,7 +3492,7 @@
           <t>Santander (préstamo) · plan 500 €/mes</t>
         </is>
       </c>
-      <c r="D53" s="28" t="inlineStr">
+      <c r="D53" s="31" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
@@ -3547,7 +3512,7 @@
     </row>
     <row r="54">
       <c r="A54" s="25" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="B54" s="26">
         <f>DATE(YEAR(A54),MONTH(A54),1)</f>
@@ -3558,7 +3523,7 @@
           <t>Crédito Santander 2 · plan 500 €/mes</t>
         </is>
       </c>
-      <c r="D54" s="37" t="inlineStr">
+      <c r="D54" s="36" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
@@ -3578,7 +3543,7 @@
     </row>
     <row r="55">
       <c r="A55" s="25" t="n">
-        <v>46478</v>
+        <v>46508</v>
       </c>
       <c r="B55" s="26">
         <f>DATE(YEAR(A55),MONTH(A55),1)</f>
@@ -3589,13 +3554,13 @@
           <t>Gastos de vida</t>
         </is>
       </c>
-      <c r="D55" s="31" t="inlineStr">
+      <c r="D55" s="32" t="inlineStr">
         <is>
           <t>Gasto</t>
         </is>
       </c>
       <c r="E55" s="27" t="inlineStr"/>
-      <c r="F55" s="32">
+      <c r="F55" s="33">
         <f>-Supuestos!B7</f>
         <v/>
       </c>
@@ -3606,7 +3571,7 @@
     </row>
     <row r="56">
       <c r="A56" s="25" t="n">
-        <v>46506</v>
+        <v>46536</v>
       </c>
       <c r="B56" s="26">
         <f>DATE(YEAR(A56),MONTH(A56),1)</f>
@@ -3617,7 +3582,7 @@
           <t>Nómina</t>
         </is>
       </c>
-      <c r="D56" s="33" t="inlineStr">
+      <c r="D56" s="28" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
@@ -3633,7 +3598,7 @@
     </row>
     <row r="57">
       <c r="A57" s="25" t="n">
-        <v>46508</v>
+        <v>46539</v>
       </c>
       <c r="B57" s="26">
         <f>DATE(YEAR(A57),MONTH(A57),1)</f>
@@ -3644,7 +3609,7 @@
           <t>Santander (préstamo) · plan 500 €/mes</t>
         </is>
       </c>
-      <c r="D57" s="28" t="inlineStr">
+      <c r="D57" s="31" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
@@ -3664,7 +3629,7 @@
     </row>
     <row r="58">
       <c r="A58" s="25" t="n">
-        <v>46508</v>
+        <v>46539</v>
       </c>
       <c r="B58" s="26">
         <f>DATE(YEAR(A58),MONTH(A58),1)</f>
@@ -3675,7 +3640,7 @@
           <t>Crédito Santander 2 · plan 500 €/mes</t>
         </is>
       </c>
-      <c r="D58" s="37" t="inlineStr">
+      <c r="D58" s="36" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
@@ -3695,7 +3660,7 @@
     </row>
     <row r="59">
       <c r="A59" s="25" t="n">
-        <v>46508</v>
+        <v>46539</v>
       </c>
       <c r="B59" s="26">
         <f>DATE(YEAR(A59),MONTH(A59),1)</f>
@@ -3706,13 +3671,13 @@
           <t>Gastos de vida</t>
         </is>
       </c>
-      <c r="D59" s="31" t="inlineStr">
+      <c r="D59" s="32" t="inlineStr">
         <is>
           <t>Gasto</t>
         </is>
       </c>
       <c r="E59" s="27" t="inlineStr"/>
-      <c r="F59" s="32">
+      <c r="F59" s="33">
         <f>-Supuestos!B7</f>
         <v/>
       </c>
@@ -3723,7 +3688,7 @@
     </row>
     <row r="60">
       <c r="A60" s="25" t="n">
-        <v>46536</v>
+        <v>46567</v>
       </c>
       <c r="B60" s="26">
         <f>DATE(YEAR(A60),MONTH(A60),1)</f>
@@ -3734,7 +3699,7 @@
           <t>Nómina</t>
         </is>
       </c>
-      <c r="D60" s="33" t="inlineStr">
+      <c r="D60" s="28" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
@@ -3750,7 +3715,7 @@
     </row>
     <row r="61">
       <c r="A61" s="25" t="n">
-        <v>46539</v>
+        <v>46567</v>
       </c>
       <c r="B61" s="26">
         <f>DATE(YEAR(A61),MONTH(A61),1)</f>
@@ -3758,21 +3723,17 @@
       </c>
       <c r="C61" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
+          <t>Paga extra de junio</t>
         </is>
       </c>
       <c r="D61" s="28" t="inlineStr">
         <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E61" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E61" s="27" t="inlineStr"/>
       <c r="F61" s="29" t="n">
-        <v>-96</v>
+        <v>1989.05</v>
       </c>
       <c r="G61" s="30">
         <f>G60+F61</f>
@@ -3781,7 +3742,7 @@
     </row>
     <row r="62">
       <c r="A62" s="25" t="n">
-        <v>46539</v>
+        <v>46569</v>
       </c>
       <c r="B62" s="26">
         <f>DATE(YEAR(A62),MONTH(A62),1)</f>
@@ -3789,21 +3750,21 @@
       </c>
       <c r="C62" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D62" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D62" s="31" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E62" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F62" s="29" t="n">
-        <v>-404</v>
+        <v>-279.08</v>
       </c>
       <c r="G62" s="30">
         <f>G61+F62</f>
@@ -3812,7 +3773,7 @@
     </row>
     <row r="63">
       <c r="A63" s="25" t="n">
-        <v>46539</v>
+        <v>46569</v>
       </c>
       <c r="B63" s="26">
         <f>DATE(YEAR(A63),MONTH(A63),1)</f>
@@ -3820,18 +3781,21 @@
       </c>
       <c r="C63" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D63" s="31" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E63" s="27" t="inlineStr"/>
-      <c r="F63" s="32">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D63" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E63" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F63" s="29" t="n">
+        <v>-220.92</v>
       </c>
       <c r="G63" s="30">
         <f>G62+F63</f>
@@ -3840,7 +3804,7 @@
     </row>
     <row r="64">
       <c r="A64" s="25" t="n">
-        <v>46567</v>
+        <v>46569</v>
       </c>
       <c r="B64" s="26">
         <f>DATE(YEAR(A64),MONTH(A64),1)</f>
@@ -3848,17 +3812,18 @@
       </c>
       <c r="C64" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D64" s="33" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D64" s="32" t="inlineStr">
+        <is>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E64" s="27" t="inlineStr"/>
-      <c r="F64" s="29" t="n">
-        <v>3173.56</v>
+      <c r="F64" s="33">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G64" s="30">
         <f>G63+F64</f>
@@ -3867,7 +3832,7 @@
     </row>
     <row r="65">
       <c r="A65" s="25" t="n">
-        <v>46567</v>
+        <v>46597</v>
       </c>
       <c r="B65" s="26">
         <f>DATE(YEAR(A65),MONTH(A65),1)</f>
@@ -3875,17 +3840,17 @@
       </c>
       <c r="C65" s="27" t="inlineStr">
         <is>
-          <t>Paga extra de junio</t>
-        </is>
-      </c>
-      <c r="D65" s="33" t="inlineStr">
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D65" s="28" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
       </c>
       <c r="E65" s="27" t="inlineStr"/>
       <c r="F65" s="29" t="n">
-        <v>1989.05</v>
+        <v>3173.56</v>
       </c>
       <c r="G65" s="30">
         <f>G64+F65</f>
@@ -3894,7 +3859,7 @@
     </row>
     <row r="66">
       <c r="A66" s="25" t="n">
-        <v>46569</v>
+        <v>46600</v>
       </c>
       <c r="B66" s="26">
         <f>DATE(YEAR(A66),MONTH(A66),1)</f>
@@ -3905,7 +3870,7 @@
           <t>Santander (préstamo) · plan 500 €/mes</t>
         </is>
       </c>
-      <c r="D66" s="28" t="inlineStr">
+      <c r="D66" s="31" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
@@ -3916,7 +3881,7 @@
         </is>
       </c>
       <c r="F66" s="29" t="n">
-        <v>-96</v>
+        <v>-500</v>
       </c>
       <c r="G66" s="30">
         <f>G65+F66</f>
@@ -3925,7 +3890,7 @@
     </row>
     <row r="67">
       <c r="A67" s="25" t="n">
-        <v>46569</v>
+        <v>46600</v>
       </c>
       <c r="B67" s="26">
         <f>DATE(YEAR(A67),MONTH(A67),1)</f>
@@ -3933,21 +3898,18 @@
       </c>
       <c r="C67" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D67" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E67" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F67" s="29" t="n">
-        <v>-404</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D67" s="32" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E67" s="27" t="inlineStr"/>
+      <c r="F67" s="33">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G67" s="30">
         <f>G66+F67</f>
@@ -3956,7 +3918,7 @@
     </row>
     <row r="68">
       <c r="A68" s="25" t="n">
-        <v>46569</v>
+        <v>46628</v>
       </c>
       <c r="B68" s="26">
         <f>DATE(YEAR(A68),MONTH(A68),1)</f>
@@ -3964,18 +3926,17 @@
       </c>
       <c r="C68" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D68" s="31" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D68" s="28" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E68" s="27" t="inlineStr"/>
-      <c r="F68" s="32">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F68" s="29" t="n">
+        <v>2280.25</v>
       </c>
       <c r="G68" s="30">
         <f>G67+F68</f>
@@ -3984,7 +3945,7 @@
     </row>
     <row r="69">
       <c r="A69" s="25" t="n">
-        <v>46597</v>
+        <v>46631</v>
       </c>
       <c r="B69" s="26">
         <f>DATE(YEAR(A69),MONTH(A69),1)</f>
@@ -3992,17 +3953,21 @@
       </c>
       <c r="C69" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D69" s="33" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E69" s="27" t="inlineStr"/>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D69" s="31" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E69" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
       <c r="F69" s="29" t="n">
-        <v>3173.56</v>
+        <v>-447.85</v>
       </c>
       <c r="G69" s="30">
         <f>G68+F69</f>
@@ -4011,7 +3976,7 @@
     </row>
     <row r="70">
       <c r="A70" s="25" t="n">
-        <v>46600</v>
+        <v>46631</v>
       </c>
       <c r="B70" s="26">
         <f>DATE(YEAR(A70),MONTH(A70),1)</f>
@@ -4019,21 +3984,18 @@
       </c>
       <c r="C70" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D70" s="28" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E70" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F70" s="29" t="n">
-        <v>-401.54</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D70" s="32" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E70" s="27" t="inlineStr"/>
+      <c r="F70" s="33">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G70" s="30">
         <f>G69+F70</f>
@@ -4042,7 +4004,7 @@
     </row>
     <row r="71">
       <c r="A71" s="25" t="n">
-        <v>46600</v>
+        <v>46659</v>
       </c>
       <c r="B71" s="26">
         <f>DATE(YEAR(A71),MONTH(A71),1)</f>
@@ -4050,21 +4012,17 @@
       </c>
       <c r="C71" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D71" s="37" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E71" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D71" s="28" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E71" s="27" t="inlineStr"/>
       <c r="F71" s="29" t="n">
-        <v>-98.45999999999999</v>
+        <v>3173.56</v>
       </c>
       <c r="G71" s="30">
         <f>G70+F71</f>
@@ -4073,7 +4031,7 @@
     </row>
     <row r="72">
       <c r="A72" s="25" t="n">
-        <v>46600</v>
+        <v>46661</v>
       </c>
       <c r="B72" s="26">
         <f>DATE(YEAR(A72),MONTH(A72),1)</f>
@@ -4084,13 +4042,13 @@
           <t>Gastos de vida</t>
         </is>
       </c>
-      <c r="D72" s="31" t="inlineStr">
+      <c r="D72" s="32" t="inlineStr">
         <is>
           <t>Gasto</t>
         </is>
       </c>
       <c r="E72" s="27" t="inlineStr"/>
-      <c r="F72" s="32">
+      <c r="F72" s="33">
         <f>-Supuestos!B7</f>
         <v/>
       </c>
@@ -4101,7 +4059,7 @@
     </row>
     <row r="73">
       <c r="A73" s="25" t="n">
-        <v>46628</v>
+        <v>46689</v>
       </c>
       <c r="B73" s="26">
         <f>DATE(YEAR(A73),MONTH(A73),1)</f>
@@ -4112,195 +4070,23 @@
           <t>Nómina</t>
         </is>
       </c>
-      <c r="D73" s="33" t="inlineStr">
+      <c r="D73" s="28" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
       </c>
       <c r="E73" s="27" t="inlineStr"/>
       <c r="F73" s="29" t="n">
-        <v>2280.25</v>
+        <v>2490.44</v>
       </c>
       <c r="G73" s="30">
         <f>G72+F73</f>
         <v/>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="25" t="n">
-        <v>46631</v>
-      </c>
-      <c r="B74" s="26">
-        <f>DATE(YEAR(A74),MONTH(A74),1)</f>
-        <v/>
-      </c>
-      <c r="C74" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D74" s="28" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E74" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F74" s="29" t="n">
-        <v>-500</v>
-      </c>
-      <c r="G74" s="30">
-        <f>G73+F74</f>
-        <v/>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="25" t="n">
-        <v>46631</v>
-      </c>
-      <c r="B75" s="26">
-        <f>DATE(YEAR(A75),MONTH(A75),1)</f>
-        <v/>
-      </c>
-      <c r="C75" s="27" t="inlineStr">
-        <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D75" s="31" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E75" s="27" t="inlineStr"/>
-      <c r="F75" s="32">
-        <f>-Supuestos!B7</f>
-        <v/>
-      </c>
-      <c r="G75" s="30">
-        <f>G74+F75</f>
-        <v/>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="25" t="n">
-        <v>46659</v>
-      </c>
-      <c r="B76" s="26">
-        <f>DATE(YEAR(A76),MONTH(A76),1)</f>
-        <v/>
-      </c>
-      <c r="C76" s="27" t="inlineStr">
-        <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D76" s="33" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E76" s="27" t="inlineStr"/>
-      <c r="F76" s="29" t="n">
-        <v>3173.56</v>
-      </c>
-      <c r="G76" s="30">
-        <f>G75+F76</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="25" t="n">
-        <v>46661</v>
-      </c>
-      <c r="B77" s="26">
-        <f>DATE(YEAR(A77),MONTH(A77),1)</f>
-        <v/>
-      </c>
-      <c r="C77" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D77" s="28" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E77" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F77" s="29" t="n">
-        <v>-229.39</v>
-      </c>
-      <c r="G77" s="30">
-        <f>G76+F77</f>
-        <v/>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="25" t="n">
-        <v>46661</v>
-      </c>
-      <c r="B78" s="26">
-        <f>DATE(YEAR(A78),MONTH(A78),1)</f>
-        <v/>
-      </c>
-      <c r="C78" s="27" t="inlineStr">
-        <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D78" s="31" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E78" s="27" t="inlineStr"/>
-      <c r="F78" s="32">
-        <f>-Supuestos!B7</f>
-        <v/>
-      </c>
-      <c r="G78" s="30">
-        <f>G77+F78</f>
-        <v/>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="25" t="n">
-        <v>46689</v>
-      </c>
-      <c r="B79" s="26">
-        <f>DATE(YEAR(A79),MONTH(A79),1)</f>
-        <v/>
-      </c>
-      <c r="C79" s="27" t="inlineStr">
-        <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D79" s="33" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E79" s="27" t="inlineStr"/>
-      <c r="F79" s="29" t="n">
-        <v>2490.44</v>
-      </c>
-      <c r="G79" s="30">
-        <f>G78+F79</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G79"/>
-  <conditionalFormatting sqref="G2:G79">
+  <autoFilter ref="A1:G73"/>
+  <conditionalFormatting sqref="G2:G73">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="1">
       <formula>0</formula>
     </cfRule>
@@ -4374,11 +4160,11 @@
         </is>
       </c>
       <c r="B6" s="41" t="n">
-        <v>150</v>
+        <v>300</v>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>Tras pagar Smartcredito te quedan 165 €: máximo disponible hasta la nómina</t>
+          <t>Con el puente de Joserra tienes 765 €; para llegar al 1 nov, máximo ~550 €</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4186,7 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Pago mensual al bloque Santander desde abr 2027 (€)</t>
+          <t>Pago mensual al bloque Santander desde mar 2027 (€)</t>
         </is>
       </c>
       <c r="B8" s="41" t="n">
@@ -4436,7 +4222,7 @@
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Escenario: hoy pagas Smartcredito; el 1 nov pagas Moneyman y lo vuelves a pedir (1.100 €) para pagar a Ama y la cuota de Vivus; el 29 nov liquidas el resto de Vivus. Aplazables: pagar y volver a pedir en nov y dic.</t>
+          <t>Escenario: hoy pagas Smartcredito y Joserra te deja 600 € (se le devuelven 1.000 € el 29 dic). Sin volver a pedir Moneyman ni Smartcredito. Ama el 29 nov.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan: saldo 600 €, nómina de octubre 3100 €, Smartcredito el 14 nov y sin préstamos puente
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JEd5Mo2HQL6TrpXUCZoFXP
</commit_message>
<xml_diff>
--- a/excel/plan_de_pagos.xlsx
+++ b/excel/plan_de_pagos.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Supuestos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Calendario'!$A$1:$G$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Calendario'!$A$1:$G$72</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -95,17 +95,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00F3F4F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00DCFCE7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FDE2E2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
     <fill>
@@ -150,7 +150,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -173,13 +173,13 @@
     <xf numFmtId="167" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -653,23 +653,23 @@
         <v>46296</v>
       </c>
       <c r="B2" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A2)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A2)</f>
         <v/>
       </c>
       <c r="C2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A2)</f>
         <v/>
       </c>
       <c r="D2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A2)</f>
         <v/>
       </c>
       <c r="E2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A2)</f>
         <v/>
       </c>
       <c r="F2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A2)</f>
         <v/>
       </c>
       <c r="G2" s="3">
@@ -690,23 +690,23 @@
         <v>46327</v>
       </c>
       <c r="B3" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A3)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A3)</f>
         <v/>
       </c>
       <c r="C3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A3)</f>
         <v/>
       </c>
       <c r="D3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A3)</f>
         <v/>
       </c>
       <c r="E3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A3)</f>
         <v/>
       </c>
       <c r="F3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A3)</f>
         <v/>
       </c>
       <c r="G3" s="3">
@@ -727,23 +727,23 @@
         <v>46357</v>
       </c>
       <c r="B4" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A4)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A4)</f>
         <v/>
       </c>
       <c r="C4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A4)</f>
         <v/>
       </c>
       <c r="D4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A4)</f>
         <v/>
       </c>
       <c r="E4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A4)</f>
         <v/>
       </c>
       <c r="F4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A4)</f>
         <v/>
       </c>
       <c r="G4" s="3">
@@ -764,23 +764,23 @@
         <v>46388</v>
       </c>
       <c r="B5" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A5)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A5)</f>
         <v/>
       </c>
       <c r="C5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A5)</f>
         <v/>
       </c>
       <c r="D5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A5)</f>
         <v/>
       </c>
       <c r="E5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A5)</f>
         <v/>
       </c>
       <c r="F5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A5)</f>
         <v/>
       </c>
       <c r="G5" s="3">
@@ -801,23 +801,23 @@
         <v>46419</v>
       </c>
       <c r="B6" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A6)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A6)</f>
         <v/>
       </c>
       <c r="C6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A6)</f>
         <v/>
       </c>
       <c r="D6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A6)</f>
         <v/>
       </c>
       <c r="E6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A6)</f>
         <v/>
       </c>
       <c r="F6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A6)</f>
         <v/>
       </c>
       <c r="G6" s="3">
@@ -838,23 +838,23 @@
         <v>46447</v>
       </c>
       <c r="B7" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A7)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A7)</f>
         <v/>
       </c>
       <c r="C7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A7)</f>
         <v/>
       </c>
       <c r="D7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A7)</f>
         <v/>
       </c>
       <c r="E7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A7)</f>
         <v/>
       </c>
       <c r="F7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A7)</f>
         <v/>
       </c>
       <c r="G7" s="3">
@@ -875,23 +875,23 @@
         <v>46478</v>
       </c>
       <c r="B8" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A8)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A8)</f>
         <v/>
       </c>
       <c r="C8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A8)</f>
         <v/>
       </c>
       <c r="D8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A8)</f>
         <v/>
       </c>
       <c r="E8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A8)</f>
         <v/>
       </c>
       <c r="F8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A8)</f>
         <v/>
       </c>
       <c r="G8" s="3">
@@ -912,23 +912,23 @@
         <v>46508</v>
       </c>
       <c r="B9" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A9)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A9)</f>
         <v/>
       </c>
       <c r="C9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A9)</f>
         <v/>
       </c>
       <c r="D9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A9)</f>
         <v/>
       </c>
       <c r="E9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A9)</f>
         <v/>
       </c>
       <c r="F9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A9)</f>
         <v/>
       </c>
       <c r="G9" s="3">
@@ -949,23 +949,23 @@
         <v>46539</v>
       </c>
       <c r="B10" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A10)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A10)</f>
         <v/>
       </c>
       <c r="C10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A10)</f>
         <v/>
       </c>
       <c r="D10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A10)</f>
         <v/>
       </c>
       <c r="E10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A10)</f>
         <v/>
       </c>
       <c r="F10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A10)</f>
         <v/>
       </c>
       <c r="G10" s="3">
@@ -986,23 +986,23 @@
         <v>46569</v>
       </c>
       <c r="B11" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A11)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A11)</f>
         <v/>
       </c>
       <c r="C11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A11)</f>
         <v/>
       </c>
       <c r="D11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A11)</f>
         <v/>
       </c>
       <c r="E11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A11)</f>
         <v/>
       </c>
       <c r="F11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A11)</f>
         <v/>
       </c>
       <c r="G11" s="3">
@@ -1023,23 +1023,23 @@
         <v>46600</v>
       </c>
       <c r="B12" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A12)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A12)</f>
         <v/>
       </c>
       <c r="C12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A12)</f>
         <v/>
       </c>
       <c r="D12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A12)</f>
         <v/>
       </c>
       <c r="E12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A12)</f>
         <v/>
       </c>
       <c r="F12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A12)</f>
         <v/>
       </c>
       <c r="G12" s="3">
@@ -1060,23 +1060,23 @@
         <v>46631</v>
       </c>
       <c r="B13" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A13)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A13)</f>
         <v/>
       </c>
       <c r="C13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A13)</f>
         <v/>
       </c>
       <c r="D13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A13)</f>
         <v/>
       </c>
       <c r="E13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A13)</f>
         <v/>
       </c>
       <c r="F13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A13)</f>
         <v/>
       </c>
       <c r="G13" s="3">
@@ -1097,23 +1097,23 @@
         <v>46661</v>
       </c>
       <c r="B14" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Ingreso",Calendario!$B$3:$B$73,A14)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A14)</f>
         <v/>
       </c>
       <c r="C14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Gasto",Calendario!$B$3:$B$73,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A14)</f>
         <v/>
       </c>
       <c r="D14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Fijo",Calendario!$B$3:$B$73,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A14)</f>
         <v/>
       </c>
       <c r="E14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Aplazable",Calendario!$B$3:$B$73,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A14)</f>
         <v/>
       </c>
       <c r="F14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$D$3:$D$73,"Amigo",Calendario!$B$3:$B$73,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A14)</f>
         <v/>
       </c>
       <c r="G14" s="3">
@@ -1171,7 +1171,7 @@
         </is>
       </c>
       <c r="C17" s="4">
-        <f>MIN(Calendario!G2:G73)</f>
+        <f>MIN(Calendario!G2:G72)</f>
         <v/>
       </c>
     </row>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="C18" s="7">
-        <f>INDEX(Calendario!A2:A73,MATCH(C17,Calendario!G2:G73,0))</f>
+        <f>INDEX(Calendario!A2:A72,MATCH(C17,Calendario!G2:G72,0))</f>
         <v/>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
         <v>1400</v>
       </c>
       <c r="E2" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A2)</f>
         <v/>
       </c>
       <c r="F2" s="3">
@@ -1291,7 +1291,7 @@
         <v/>
       </c>
       <c r="G2" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A2)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A2)</f>
         <v/>
       </c>
       <c r="H2" s="13" t="inlineStr">
@@ -1323,7 +1323,7 @@
         <v>2148</v>
       </c>
       <c r="E3" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A3)</f>
         <v/>
       </c>
       <c r="F3" s="3">
@@ -1331,7 +1331,7 @@
         <v/>
       </c>
       <c r="G3" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A3)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A3)</f>
         <v/>
       </c>
       <c r="H3" s="13" t="inlineStr">
@@ -1363,7 +1363,7 @@
         <v>435</v>
       </c>
       <c r="E4" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A4)</f>
         <v/>
       </c>
       <c r="F4" s="3">
@@ -1371,12 +1371,12 @@
         <v/>
       </c>
       <c r="G4" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A4)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A4)</f>
         <v/>
       </c>
       <c r="H4" s="13" t="inlineStr">
         <is>
-          <t>Pago único hoy (13 oct). Volver a pedirlo cuesta: recibes 300 €, devuelves 435 €</t>
+          <t>Pago único el 14 nov. Volver a pedirlo cuesta: recibes 300 €, devuelves 435 €</t>
         </is>
       </c>
       <c r="I4" s="10" t="n">
@@ -1403,7 +1403,7 @@
         <v>1994.93</v>
       </c>
       <c r="E5" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A5)</f>
         <v/>
       </c>
       <c r="F5" s="3">
@@ -1411,7 +1411,7 @@
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A5)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A5)</f>
         <v/>
       </c>
       <c r="H5" s="13" t="inlineStr">
@@ -1443,7 +1443,7 @@
         <v>693.34</v>
       </c>
       <c r="E6" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A6)</f>
         <v/>
       </c>
       <c r="F6" s="3">
@@ -1451,7 +1451,7 @@
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A6)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A6)</f>
         <v/>
       </c>
       <c r="H6" s="13" t="inlineStr">
@@ -1483,7 +1483,7 @@
         <v>923.61</v>
       </c>
       <c r="E7" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A7)</f>
         <v/>
       </c>
       <c r="F7" s="3">
@@ -1491,7 +1491,7 @@
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A7)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A7)</f>
         <v/>
       </c>
       <c r="H7" s="13" t="inlineStr">
@@ -1523,7 +1523,7 @@
         <v>1483.63</v>
       </c>
       <c r="E8" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A8)</f>
         <v/>
       </c>
       <c r="F8" s="3">
@@ -1531,7 +1531,7 @@
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A8)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A8)</f>
         <v/>
       </c>
       <c r="H8" s="13" t="inlineStr">
@@ -1563,7 +1563,7 @@
         <v>2326.76</v>
       </c>
       <c r="E9" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A9)</f>
         <v/>
       </c>
       <c r="F9" s="3">
@@ -1571,7 +1571,7 @@
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A9)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A9)</f>
         <v/>
       </c>
       <c r="H9" s="13" t="inlineStr">
@@ -1603,7 +1603,7 @@
         <v>600</v>
       </c>
       <c r="E10" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A10)</f>
         <v/>
       </c>
       <c r="F10" s="3">
@@ -1611,7 +1611,7 @@
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A10)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A10)</f>
         <v/>
       </c>
       <c r="H10" s="13" t="inlineStr">
@@ -1640,10 +1640,10 @@
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>1000</v>
+        <v>400</v>
       </c>
       <c r="E11" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A11)</f>
         <v/>
       </c>
       <c r="F11" s="3">
@@ -1651,12 +1651,12 @@
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A11)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A11)</f>
         <v/>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>400 € anteriores + 600 € de puente el 13 oct. Se devuelve todo antes de fin de año</t>
+          <t>Sin plazo ni interés. Se devuelve antes de fin de año</t>
         </is>
       </c>
       <c r="I11" s="10" t="n">
@@ -1683,7 +1683,7 @@
         <v>300</v>
       </c>
       <c r="E12" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A12)</f>
         <v/>
       </c>
       <c r="F12" s="3">
@@ -1691,7 +1691,7 @@
         <v/>
       </c>
       <c r="G12" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A12)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A12)</f>
         <v/>
       </c>
       <c r="H12" s="13" t="inlineStr">
@@ -1723,7 +1723,7 @@
         <v>1700</v>
       </c>
       <c r="E13" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A13)</f>
         <v/>
       </c>
       <c r="F13" s="3">
@@ -1731,7 +1731,7 @@
         <v/>
       </c>
       <c r="G13" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A13)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A13)</f>
         <v/>
       </c>
       <c r="H13" s="13" t="inlineStr">
@@ -1763,7 +1763,7 @@
         <v>2500</v>
       </c>
       <c r="E14" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$73,Calendario!$E$3:$E$73,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A14)</f>
         <v/>
       </c>
       <c r="F14" s="3">
@@ -1771,7 +1771,7 @@
         <v/>
       </c>
       <c r="G14" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$73,Calendario!$E$3:$E$73,A14)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A14)</f>
         <v/>
       </c>
       <c r="H14" s="13" t="inlineStr">
@@ -1869,7 +1869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:J72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1959,7 +1959,7 @@
     </row>
     <row r="3">
       <c r="A3" s="25" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B3" s="26">
         <f>DATE(YEAR(A3),MONTH(A3),1)</f>
@@ -1967,17 +1967,18 @@
       </c>
       <c r="C3" s="27" t="inlineStr">
         <is>
-          <t>Préstamo puente de Joserra (sin intereses)</t>
+          <t>Gastos de vida hasta el 29 oct (estimado)</t>
         </is>
       </c>
       <c r="D3" s="28" t="inlineStr">
         <is>
-          <t>Ingreso</t>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E3" s="27" t="inlineStr"/>
-      <c r="F3" s="29" t="n">
-        <v>600</v>
+      <c r="F3" s="29">
+        <f>-Supuestos!B6</f>
+        <v/>
       </c>
       <c r="G3" s="30">
         <f>G2+F3</f>
@@ -1996,7 +1997,7 @@
     </row>
     <row r="4">
       <c r="A4" s="25" t="n">
-        <v>46308</v>
+        <v>46324</v>
       </c>
       <c r="B4" s="26">
         <f>DATE(YEAR(A4),MONTH(A4),1)</f>
@@ -2004,21 +2005,17 @@
       </c>
       <c r="C4" s="27" t="inlineStr">
         <is>
-          <t>Smartcredito · pago hoy</t>
+          <t>Nómina</t>
         </is>
       </c>
       <c r="D4" s="31" t="inlineStr">
         <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E4" s="27" t="inlineStr">
-        <is>
-          <t>Smartcredito</t>
-        </is>
-      </c>
-      <c r="F4" s="29" t="n">
-        <v>-435</v>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr"/>
+      <c r="F4" s="32" t="n">
+        <v>3100</v>
       </c>
       <c r="G4" s="30">
         <f>G3+F4</f>
@@ -2037,7 +2034,7 @@
     </row>
     <row r="5">
       <c r="A5" s="25" t="n">
-        <v>46309</v>
+        <v>46327</v>
       </c>
       <c r="B5" s="26">
         <f>DATE(YEAR(A5),MONTH(A5),1)</f>
@@ -2045,18 +2042,21 @@
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida hasta el 29 oct (estimado)</t>
-        </is>
-      </c>
-      <c r="D5" s="32" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E5" s="27" t="inlineStr"/>
-      <c r="F5" s="33">
-        <f>-Supuestos!B6</f>
-        <v/>
+          <t>Moneyman · pago (sin volver a pedirlo)</t>
+        </is>
+      </c>
+      <c r="D5" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr">
+        <is>
+          <t>Moneyman</t>
+        </is>
+      </c>
+      <c r="F5" s="32" t="n">
+        <v>-1400</v>
       </c>
       <c r="G5" s="30">
         <f>G4+F5</f>
@@ -2075,7 +2075,7 @@
     </row>
     <row r="6">
       <c r="A6" s="25" t="n">
-        <v>46324</v>
+        <v>46327</v>
       </c>
       <c r="B6" s="26">
         <f>DATE(YEAR(A6),MONTH(A6),1)</f>
@@ -2083,17 +2083,21 @@
       </c>
       <c r="C6" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D6" s="28" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E6" s="27" t="inlineStr"/>
-      <c r="F6" s="29" t="n">
-        <v>2645.44</v>
+          <t>Vivus · cuota 1/4 (no aplazable)</t>
+        </is>
+      </c>
+      <c r="D6" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>Vivus</t>
+        </is>
+      </c>
+      <c r="F6" s="32" t="n">
+        <v>-537</v>
       </c>
       <c r="G6" s="30">
         <f>G5+F6</f>
@@ -2120,21 +2124,17 @@
       </c>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>Moneyman · pago (sin volver a pedirlo)</t>
-        </is>
-      </c>
-      <c r="D7" s="31" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E7" s="27" t="inlineStr">
-        <is>
-          <t>Moneyman</t>
-        </is>
-      </c>
-      <c r="F7" s="29" t="n">
-        <v>-1400</v>
+          <t>Pagolisto 1 · pagas 231,11 € y lo vuelves a pedir (neto 0)</t>
+        </is>
+      </c>
+      <c r="D7" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr"/>
+      <c r="F7" s="32" t="n">
+        <v>0</v>
       </c>
       <c r="G7" s="30">
         <f>G6+F7</f>
@@ -2151,21 +2151,17 @@
       </c>
       <c r="C8" s="27" t="inlineStr">
         <is>
-          <t>Vivus · cuota 1/4 (no aplazable)</t>
-        </is>
-      </c>
-      <c r="D8" s="31" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E8" s="27" t="inlineStr">
-        <is>
-          <t>Vivus</t>
-        </is>
-      </c>
-      <c r="F8" s="29" t="n">
-        <v>-537</v>
+          <t>Pagolisto 2 · pagas 307,87 € y lo vuelves a pedir (neto 0)</t>
+        </is>
+      </c>
+      <c r="D8" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr"/>
+      <c r="F8" s="32" t="n">
+        <v>0</v>
       </c>
       <c r="G8" s="30">
         <f>G7+F8</f>
@@ -2187,7 +2183,7 @@
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · pagas 231,11 € y lo vuelves a pedir (neto 0)</t>
+          <t>Crédito Santander 1 · pagas 494,54 € y lo vuelves a pedir (neto 0)</t>
         </is>
       </c>
       <c r="D9" s="36" t="inlineStr">
@@ -2196,7 +2192,7 @@
         </is>
       </c>
       <c r="E9" s="27" t="inlineStr"/>
-      <c r="F9" s="29" t="n">
+      <c r="F9" s="32" t="n">
         <v>0</v>
       </c>
       <c r="G9" s="30">
@@ -2214,17 +2210,21 @@
       </c>
       <c r="C10" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · pagas 307,87 € y lo vuelves a pedir (neto 0)</t>
-        </is>
-      </c>
-      <c r="D10" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E10" s="27" t="inlineStr"/>
-      <c r="F10" s="29" t="n">
-        <v>0</v>
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D10" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F10" s="32" t="n">
+        <v>-96</v>
       </c>
       <c r="G10" s="30">
         <f>G9+F10</f>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="C11" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · pagas 494,54 € y lo vuelves a pedir (neto 0)</t>
+          <t>Crédito Santander 2 · cuota</t>
         </is>
       </c>
       <c r="D11" s="36" t="inlineStr">
@@ -2249,9 +2249,13 @@
           <t>Aplazable</t>
         </is>
       </c>
-      <c r="E11" s="27" t="inlineStr"/>
-      <c r="F11" s="29" t="n">
-        <v>0</v>
+      <c r="E11" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F11" s="32" t="n">
+        <v>-122.46</v>
       </c>
       <c r="G11" s="30">
         <f>G10+F11</f>
@@ -2268,21 +2272,18 @@
       </c>
       <c r="C12" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D12" s="31" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E12" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F12" s="29" t="n">
-        <v>-96</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D12" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E12" s="27" t="inlineStr"/>
+      <c r="F12" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G12" s="30">
         <f>G11+F12</f>
@@ -2291,7 +2292,7 @@
     </row>
     <row r="13">
       <c r="A13" s="25" t="n">
-        <v>46327</v>
+        <v>46340</v>
       </c>
       <c r="B13" s="26">
         <f>DATE(YEAR(A13),MONTH(A13),1)</f>
@@ -2299,21 +2300,21 @@
       </c>
       <c r="C13" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
-        </is>
-      </c>
-      <c r="D13" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Smartcredito · pago único</t>
+        </is>
+      </c>
+      <c r="D13" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E13" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F13" s="29" t="n">
-        <v>-122.46</v>
+          <t>Smartcredito</t>
+        </is>
+      </c>
+      <c r="F13" s="32" t="n">
+        <v>-435</v>
       </c>
       <c r="G13" s="30">
         <f>G12+F13</f>
@@ -2322,7 +2323,7 @@
     </row>
     <row r="14">
       <c r="A14" s="25" t="n">
-        <v>46327</v>
+        <v>46355</v>
       </c>
       <c r="B14" s="26">
         <f>DATE(YEAR(A14),MONTH(A14),1)</f>
@@ -2330,18 +2331,17 @@
       </c>
       <c r="C14" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D14" s="32" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D14" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E14" s="27" t="inlineStr"/>
-      <c r="F14" s="33">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F14" s="32" t="n">
+        <v>3453.01</v>
       </c>
       <c r="G14" s="30">
         <f>G13+F14</f>
@@ -2358,17 +2358,21 @@
       </c>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D15" s="28" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E15" s="27" t="inlineStr"/>
-      <c r="F15" s="29" t="n">
-        <v>3453.01</v>
+          <t>Vivus · liquidación del resto (total 1.500 € en vez de 2.148 €)</t>
+        </is>
+      </c>
+      <c r="D15" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E15" s="27" t="inlineStr">
+        <is>
+          <t>Vivus</t>
+        </is>
+      </c>
+      <c r="F15" s="32" t="n">
+        <v>-963</v>
       </c>
       <c r="G15" s="30">
         <f>G14+F15</f>
@@ -2385,21 +2389,21 @@
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
-          <t>Vivus · liquidación del resto (total 1.500 € en vez de 2.148 €)</t>
-        </is>
-      </c>
-      <c r="D16" s="31" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Devolución a Ama</t>
+        </is>
+      </c>
+      <c r="D16" s="37" t="inlineStr">
+        <is>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E16" s="27" t="inlineStr">
         <is>
-          <t>Vivus</t>
-        </is>
-      </c>
-      <c r="F16" s="29" t="n">
-        <v>-963</v>
+          <t>Ama</t>
+        </is>
+      </c>
+      <c r="F16" s="32" t="n">
+        <v>-600</v>
       </c>
       <c r="G16" s="30">
         <f>G15+F16</f>
@@ -2408,7 +2412,7 @@
     </row>
     <row r="17">
       <c r="A17" s="25" t="n">
-        <v>46355</v>
+        <v>46357</v>
       </c>
       <c r="B17" s="26">
         <f>DATE(YEAR(A17),MONTH(A17),1)</f>
@@ -2416,21 +2420,21 @@
       </c>
       <c r="C17" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Ama</t>
-        </is>
-      </c>
-      <c r="D17" s="37" t="inlineStr">
-        <is>
-          <t>Amigo</t>
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D17" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E17" s="27" t="inlineStr">
         <is>
-          <t>Ama</t>
-        </is>
-      </c>
-      <c r="F17" s="29" t="n">
-        <v>-600</v>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F17" s="32" t="n">
+        <v>-96</v>
       </c>
       <c r="G17" s="30">
         <f>G16+F17</f>
@@ -2447,21 +2451,21 @@
       </c>
       <c r="C18" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D18" s="31" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D18" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E18" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F18" s="29" t="n">
-        <v>-96</v>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F18" s="32" t="n">
+        <v>-122.46</v>
       </c>
       <c r="G18" s="30">
         <f>G17+F18</f>
@@ -2478,7 +2482,7 @@
       </c>
       <c r="C19" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
+          <t>Pagolisto 1 · cuota 1/3</t>
         </is>
       </c>
       <c r="D19" s="36" t="inlineStr">
@@ -2488,11 +2492,11 @@
       </c>
       <c r="E19" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F19" s="29" t="n">
-        <v>-122.46</v>
+          <t>Pagolisto 1</t>
+        </is>
+      </c>
+      <c r="F19" s="32" t="n">
+        <v>-231.11</v>
       </c>
       <c r="G19" s="30">
         <f>G18+F19</f>
@@ -2509,7 +2513,7 @@
       </c>
       <c r="C20" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 1/3</t>
+          <t>Pagolisto 2 · cuota 1/3</t>
         </is>
       </c>
       <c r="D20" s="36" t="inlineStr">
@@ -2519,11 +2523,11 @@
       </c>
       <c r="E20" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1</t>
-        </is>
-      </c>
-      <c r="F20" s="29" t="n">
-        <v>-231.11</v>
+          <t>Pagolisto 2</t>
+        </is>
+      </c>
+      <c r="F20" s="32" t="n">
+        <v>-307.87</v>
       </c>
       <c r="G20" s="30">
         <f>G19+F20</f>
@@ -2540,7 +2544,7 @@
       </c>
       <c r="C21" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 1/3</t>
+          <t>Crédito Santander 1 · cuota 1/3</t>
         </is>
       </c>
       <c r="D21" s="36" t="inlineStr">
@@ -2550,11 +2554,11 @@
       </c>
       <c r="E21" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2</t>
-        </is>
-      </c>
-      <c r="F21" s="29" t="n">
-        <v>-307.87</v>
+          <t>Crédito Santander 1</t>
+        </is>
+      </c>
+      <c r="F21" s="32" t="n">
+        <v>-494.54</v>
       </c>
       <c r="G21" s="30">
         <f>G20+F21</f>
@@ -2571,21 +2575,18 @@
       </c>
       <c r="C22" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 1/3</t>
-        </is>
-      </c>
-      <c r="D22" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E22" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 1</t>
-        </is>
-      </c>
-      <c r="F22" s="29" t="n">
-        <v>-494.54</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D22" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E22" s="27" t="inlineStr"/>
+      <c r="F22" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G22" s="30">
         <f>G21+F22</f>
@@ -2594,7 +2595,7 @@
     </row>
     <row r="23">
       <c r="A23" s="25" t="n">
-        <v>46357</v>
+        <v>46385</v>
       </c>
       <c r="B23" s="26">
         <f>DATE(YEAR(A23),MONTH(A23),1)</f>
@@ -2602,18 +2603,17 @@
       </c>
       <c r="C23" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D23" s="32" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D23" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E23" s="27" t="inlineStr"/>
-      <c r="F23" s="33">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F23" s="32" t="n">
+        <v>3453.01</v>
       </c>
       <c r="G23" s="30">
         <f>G22+F23</f>
@@ -2630,17 +2630,17 @@
       </c>
       <c r="C24" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D24" s="28" t="inlineStr">
+          <t>Paga extra de diciembre</t>
+        </is>
+      </c>
+      <c r="D24" s="31" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
       </c>
       <c r="E24" s="27" t="inlineStr"/>
-      <c r="F24" s="29" t="n">
-        <v>3453.01</v>
+      <c r="F24" s="32" t="n">
+        <v>2014.69</v>
       </c>
       <c r="G24" s="30">
         <f>G23+F24</f>
@@ -2657,17 +2657,21 @@
       </c>
       <c r="C25" s="27" t="inlineStr">
         <is>
-          <t>Paga extra de diciembre</t>
-        </is>
-      </c>
-      <c r="D25" s="28" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E25" s="27" t="inlineStr"/>
-      <c r="F25" s="29" t="n">
-        <v>2014.69</v>
+          <t>Devolución a Joserra</t>
+        </is>
+      </c>
+      <c r="D25" s="37" t="inlineStr">
+        <is>
+          <t>Amigo</t>
+        </is>
+      </c>
+      <c r="E25" s="27" t="inlineStr">
+        <is>
+          <t>Joserra</t>
+        </is>
+      </c>
+      <c r="F25" s="32" t="n">
+        <v>-400</v>
       </c>
       <c r="G25" s="30">
         <f>G24+F25</f>
@@ -2676,7 +2680,7 @@
     </row>
     <row r="26">
       <c r="A26" s="25" t="n">
-        <v>46385</v>
+        <v>46388</v>
       </c>
       <c r="B26" s="26">
         <f>DATE(YEAR(A26),MONTH(A26),1)</f>
@@ -2684,21 +2688,21 @@
       </c>
       <c r="C26" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Joserra (puente + lo anterior)</t>
-        </is>
-      </c>
-      <c r="D26" s="37" t="inlineStr">
-        <is>
-          <t>Amigo</t>
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D26" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E26" s="27" t="inlineStr">
         <is>
-          <t>Joserra</t>
-        </is>
-      </c>
-      <c r="F26" s="29" t="n">
-        <v>-1000</v>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F26" s="32" t="n">
+        <v>-96</v>
       </c>
       <c r="G26" s="30">
         <f>G25+F26</f>
@@ -2715,21 +2719,21 @@
       </c>
       <c r="C27" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D27" s="31" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D27" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E27" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F27" s="29" t="n">
-        <v>-96</v>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F27" s="32" t="n">
+        <v>-122.46</v>
       </c>
       <c r="G27" s="30">
         <f>G26+F27</f>
@@ -2746,7 +2750,7 @@
       </c>
       <c r="C28" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
+          <t>Pagolisto 1 · cuota 2/3</t>
         </is>
       </c>
       <c r="D28" s="36" t="inlineStr">
@@ -2756,11 +2760,11 @@
       </c>
       <c r="E28" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F28" s="29" t="n">
-        <v>-122.46</v>
+          <t>Pagolisto 1</t>
+        </is>
+      </c>
+      <c r="F28" s="32" t="n">
+        <v>-231.11</v>
       </c>
       <c r="G28" s="30">
         <f>G27+F28</f>
@@ -2777,7 +2781,7 @@
       </c>
       <c r="C29" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 2/3</t>
+          <t>Pagolisto 2 · cuota 2/3</t>
         </is>
       </c>
       <c r="D29" s="36" t="inlineStr">
@@ -2787,11 +2791,11 @@
       </c>
       <c r="E29" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1</t>
-        </is>
-      </c>
-      <c r="F29" s="29" t="n">
-        <v>-231.11</v>
+          <t>Pagolisto 2</t>
+        </is>
+      </c>
+      <c r="F29" s="32" t="n">
+        <v>-307.87</v>
       </c>
       <c r="G29" s="30">
         <f>G28+F29</f>
@@ -2808,7 +2812,7 @@
       </c>
       <c r="C30" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 2/3</t>
+          <t>Crédito Santander 1 · cuota 2/3</t>
         </is>
       </c>
       <c r="D30" s="36" t="inlineStr">
@@ -2818,11 +2822,11 @@
       </c>
       <c r="E30" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2</t>
-        </is>
-      </c>
-      <c r="F30" s="29" t="n">
-        <v>-307.87</v>
+          <t>Crédito Santander 1</t>
+        </is>
+      </c>
+      <c r="F30" s="32" t="n">
+        <v>-494.54</v>
       </c>
       <c r="G30" s="30">
         <f>G29+F30</f>
@@ -2839,21 +2843,21 @@
       </c>
       <c r="C31" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 2/3</t>
-        </is>
-      </c>
-      <c r="D31" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Devolución a Xabi</t>
+        </is>
+      </c>
+      <c r="D31" s="37" t="inlineStr">
+        <is>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E31" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1</t>
-        </is>
-      </c>
-      <c r="F31" s="29" t="n">
-        <v>-494.54</v>
+          <t>Xabi</t>
+        </is>
+      </c>
+      <c r="F31" s="32" t="n">
+        <v>-300</v>
       </c>
       <c r="G31" s="30">
         <f>G30+F31</f>
@@ -2870,21 +2874,18 @@
       </c>
       <c r="C32" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Xabi</t>
-        </is>
-      </c>
-      <c r="D32" s="37" t="inlineStr">
-        <is>
-          <t>Amigo</t>
-        </is>
-      </c>
-      <c r="E32" s="27" t="inlineStr">
-        <is>
-          <t>Xabi</t>
-        </is>
-      </c>
-      <c r="F32" s="29" t="n">
-        <v>-300</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D32" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E32" s="27" t="inlineStr"/>
+      <c r="F32" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G32" s="30">
         <f>G31+F32</f>
@@ -2893,7 +2894,7 @@
     </row>
     <row r="33">
       <c r="A33" s="25" t="n">
-        <v>46388</v>
+        <v>46416</v>
       </c>
       <c r="B33" s="26">
         <f>DATE(YEAR(A33),MONTH(A33),1)</f>
@@ -2901,18 +2902,17 @@
       </c>
       <c r="C33" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D33" s="32" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D33" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E33" s="27" t="inlineStr"/>
-      <c r="F33" s="33">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F33" s="32" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G33" s="30">
         <f>G32+F33</f>
@@ -2921,7 +2921,7 @@
     </row>
     <row r="34">
       <c r="A34" s="25" t="n">
-        <v>46416</v>
+        <v>46419</v>
       </c>
       <c r="B34" s="26">
         <f>DATE(YEAR(A34),MONTH(A34),1)</f>
@@ -2929,17 +2929,21 @@
       </c>
       <c r="C34" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D34" s="28" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E34" s="27" t="inlineStr"/>
-      <c r="F34" s="29" t="n">
-        <v>3173.56</v>
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D34" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E34" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F34" s="32" t="n">
+        <v>-96</v>
       </c>
       <c r="G34" s="30">
         <f>G33+F34</f>
@@ -2956,21 +2960,21 @@
       </c>
       <c r="C35" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D35" s="31" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D35" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E35" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F35" s="29" t="n">
-        <v>-96</v>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F35" s="32" t="n">
+        <v>-122.46</v>
       </c>
       <c r="G35" s="30">
         <f>G34+F35</f>
@@ -2987,7 +2991,7 @@
       </c>
       <c r="C36" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
+          <t>Pagolisto 1 · cuota 3/3</t>
         </is>
       </c>
       <c r="D36" s="36" t="inlineStr">
@@ -2997,11 +3001,11 @@
       </c>
       <c r="E36" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F36" s="29" t="n">
-        <v>-122.46</v>
+          <t>Pagolisto 1</t>
+        </is>
+      </c>
+      <c r="F36" s="32" t="n">
+        <v>-231.12</v>
       </c>
       <c r="G36" s="30">
         <f>G35+F36</f>
@@ -3018,7 +3022,7 @@
       </c>
       <c r="C37" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 3/3</t>
+          <t>Pagolisto 2 · cuota 3/3</t>
         </is>
       </c>
       <c r="D37" s="36" t="inlineStr">
@@ -3028,11 +3032,11 @@
       </c>
       <c r="E37" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1</t>
-        </is>
-      </c>
-      <c r="F37" s="29" t="n">
-        <v>-231.12</v>
+          <t>Pagolisto 2</t>
+        </is>
+      </c>
+      <c r="F37" s="32" t="n">
+        <v>-307.87</v>
       </c>
       <c r="G37" s="30">
         <f>G36+F37</f>
@@ -3049,7 +3053,7 @@
       </c>
       <c r="C38" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 3/3</t>
+          <t>Crédito Santander 1 · cuota 3/3</t>
         </is>
       </c>
       <c r="D38" s="36" t="inlineStr">
@@ -3059,11 +3063,11 @@
       </c>
       <c r="E38" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2</t>
-        </is>
-      </c>
-      <c r="F38" s="29" t="n">
-        <v>-307.87</v>
+          <t>Crédito Santander 1</t>
+        </is>
+      </c>
+      <c r="F38" s="32" t="n">
+        <v>-494.55</v>
       </c>
       <c r="G38" s="30">
         <f>G37+F38</f>
@@ -3080,21 +3084,21 @@
       </c>
       <c r="C39" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 3/3</t>
-        </is>
-      </c>
-      <c r="D39" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
+          <t>Devolución a Sergio</t>
+        </is>
+      </c>
+      <c r="D39" s="37" t="inlineStr">
+        <is>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E39" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1</t>
-        </is>
-      </c>
-      <c r="F39" s="29" t="n">
-        <v>-494.55</v>
+          <t>Sergio</t>
+        </is>
+      </c>
+      <c r="F39" s="32" t="n">
+        <v>-1700</v>
       </c>
       <c r="G39" s="30">
         <f>G38+F39</f>
@@ -3111,21 +3115,18 @@
       </c>
       <c r="C40" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Sergio</t>
-        </is>
-      </c>
-      <c r="D40" s="37" t="inlineStr">
-        <is>
-          <t>Amigo</t>
-        </is>
-      </c>
-      <c r="E40" s="27" t="inlineStr">
-        <is>
-          <t>Sergio</t>
-        </is>
-      </c>
-      <c r="F40" s="29" t="n">
-        <v>-1700</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D40" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E40" s="27" t="inlineStr"/>
+      <c r="F40" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G40" s="30">
         <f>G39+F40</f>
@@ -3134,7 +3135,7 @@
     </row>
     <row r="41">
       <c r="A41" s="25" t="n">
-        <v>46419</v>
+        <v>46446</v>
       </c>
       <c r="B41" s="26">
         <f>DATE(YEAR(A41),MONTH(A41),1)</f>
@@ -3142,18 +3143,17 @@
       </c>
       <c r="C41" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D41" s="32" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D41" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E41" s="27" t="inlineStr"/>
-      <c r="F41" s="33">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F41" s="32" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G41" s="30">
         <f>G40+F41</f>
@@ -3170,17 +3170,17 @@
       </c>
       <c r="C42" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D42" s="28" t="inlineStr">
+          <t>Variable de febrero</t>
+        </is>
+      </c>
+      <c r="D42" s="31" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
       </c>
       <c r="E42" s="27" t="inlineStr"/>
-      <c r="F42" s="29" t="n">
-        <v>3173.56</v>
+      <c r="F42" s="32" t="n">
+        <v>2114.45</v>
       </c>
       <c r="G42" s="30">
         <f>G41+F42</f>
@@ -3197,17 +3197,21 @@
       </c>
       <c r="C43" s="27" t="inlineStr">
         <is>
-          <t>Variable de febrero</t>
-        </is>
-      </c>
-      <c r="D43" s="28" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E43" s="27" t="inlineStr"/>
-      <c r="F43" s="29" t="n">
-        <v>2114.45</v>
+          <t>Devolución a Txomin</t>
+        </is>
+      </c>
+      <c r="D43" s="37" t="inlineStr">
+        <is>
+          <t>Amigo</t>
+        </is>
+      </c>
+      <c r="E43" s="27" t="inlineStr">
+        <is>
+          <t>Txomin</t>
+        </is>
+      </c>
+      <c r="F43" s="32" t="n">
+        <v>-2500</v>
       </c>
       <c r="G43" s="30">
         <f>G42+F43</f>
@@ -3216,7 +3220,7 @@
     </row>
     <row r="44">
       <c r="A44" s="25" t="n">
-        <v>46446</v>
+        <v>46447</v>
       </c>
       <c r="B44" s="26">
         <f>DATE(YEAR(A44),MONTH(A44),1)</f>
@@ -3224,21 +3228,21 @@
       </c>
       <c r="C44" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Txomin</t>
-        </is>
-      </c>
-      <c r="D44" s="37" t="inlineStr">
-        <is>
-          <t>Amigo</t>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D44" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E44" s="27" t="inlineStr">
         <is>
-          <t>Txomin</t>
-        </is>
-      </c>
-      <c r="F44" s="29" t="n">
-        <v>-2500</v>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F44" s="32" t="n">
+        <v>-96</v>
       </c>
       <c r="G44" s="30">
         <f>G43+F44</f>
@@ -3255,21 +3259,21 @@
       </c>
       <c r="C45" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D45" s="31" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D45" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E45" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F45" s="29" t="n">
-        <v>-96</v>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F45" s="32" t="n">
+        <v>-404</v>
       </c>
       <c r="G45" s="30">
         <f>G44+F45</f>
@@ -3286,21 +3290,18 @@
       </c>
       <c r="C46" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D46" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E46" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F46" s="29" t="n">
-        <v>-404</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D46" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E46" s="27" t="inlineStr"/>
+      <c r="F46" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G46" s="30">
         <f>G45+F46</f>
@@ -3309,7 +3310,7 @@
     </row>
     <row r="47">
       <c r="A47" s="25" t="n">
-        <v>46447</v>
+        <v>46475</v>
       </c>
       <c r="B47" s="26">
         <f>DATE(YEAR(A47),MONTH(A47),1)</f>
@@ -3317,18 +3318,17 @@
       </c>
       <c r="C47" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D47" s="32" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D47" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E47" s="27" t="inlineStr"/>
-      <c r="F47" s="33">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F47" s="32" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G47" s="30">
         <f>G46+F47</f>
@@ -3337,7 +3337,7 @@
     </row>
     <row r="48">
       <c r="A48" s="25" t="n">
-        <v>46475</v>
+        <v>46478</v>
       </c>
       <c r="B48" s="26">
         <f>DATE(YEAR(A48),MONTH(A48),1)</f>
@@ -3345,17 +3345,21 @@
       </c>
       <c r="C48" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D48" s="28" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E48" s="27" t="inlineStr"/>
-      <c r="F48" s="29" t="n">
-        <v>3173.56</v>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D48" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E48" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F48" s="32" t="n">
+        <v>-96</v>
       </c>
       <c r="G48" s="30">
         <f>G47+F48</f>
@@ -3372,21 +3376,21 @@
       </c>
       <c r="C49" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D49" s="31" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D49" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E49" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F49" s="29" t="n">
-        <v>-96</v>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F49" s="32" t="n">
+        <v>-404</v>
       </c>
       <c r="G49" s="30">
         <f>G48+F49</f>
@@ -3403,21 +3407,18 @@
       </c>
       <c r="C50" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D50" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E50" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F50" s="29" t="n">
-        <v>-404</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D50" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E50" s="27" t="inlineStr"/>
+      <c r="F50" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G50" s="30">
         <f>G49+F50</f>
@@ -3426,7 +3427,7 @@
     </row>
     <row r="51">
       <c r="A51" s="25" t="n">
-        <v>46478</v>
+        <v>46506</v>
       </c>
       <c r="B51" s="26">
         <f>DATE(YEAR(A51),MONTH(A51),1)</f>
@@ -3434,18 +3435,17 @@
       </c>
       <c r="C51" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D51" s="32" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D51" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E51" s="27" t="inlineStr"/>
-      <c r="F51" s="33">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F51" s="32" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G51" s="30">
         <f>G50+F51</f>
@@ -3454,7 +3454,7 @@
     </row>
     <row r="52">
       <c r="A52" s="25" t="n">
-        <v>46506</v>
+        <v>46508</v>
       </c>
       <c r="B52" s="26">
         <f>DATE(YEAR(A52),MONTH(A52),1)</f>
@@ -3462,17 +3462,21 @@
       </c>
       <c r="C52" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D52" s="28" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E52" s="27" t="inlineStr"/>
-      <c r="F52" s="29" t="n">
-        <v>3173.56</v>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D52" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E52" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F52" s="32" t="n">
+        <v>-96</v>
       </c>
       <c r="G52" s="30">
         <f>G51+F52</f>
@@ -3489,21 +3493,21 @@
       </c>
       <c r="C53" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D53" s="31" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D53" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E53" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F53" s="29" t="n">
-        <v>-96</v>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F53" s="32" t="n">
+        <v>-404</v>
       </c>
       <c r="G53" s="30">
         <f>G52+F53</f>
@@ -3520,21 +3524,18 @@
       </c>
       <c r="C54" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D54" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E54" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F54" s="29" t="n">
-        <v>-404</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D54" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E54" s="27" t="inlineStr"/>
+      <c r="F54" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G54" s="30">
         <f>G53+F54</f>
@@ -3543,7 +3544,7 @@
     </row>
     <row r="55">
       <c r="A55" s="25" t="n">
-        <v>46508</v>
+        <v>46536</v>
       </c>
       <c r="B55" s="26">
         <f>DATE(YEAR(A55),MONTH(A55),1)</f>
@@ -3551,18 +3552,17 @@
       </c>
       <c r="C55" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D55" s="32" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D55" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E55" s="27" t="inlineStr"/>
-      <c r="F55" s="33">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F55" s="32" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G55" s="30">
         <f>G54+F55</f>
@@ -3571,7 +3571,7 @@
     </row>
     <row r="56">
       <c r="A56" s="25" t="n">
-        <v>46536</v>
+        <v>46539</v>
       </c>
       <c r="B56" s="26">
         <f>DATE(YEAR(A56),MONTH(A56),1)</f>
@@ -3579,17 +3579,21 @@
       </c>
       <c r="C56" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D56" s="28" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E56" s="27" t="inlineStr"/>
-      <c r="F56" s="29" t="n">
-        <v>3173.56</v>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D56" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E56" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F56" s="32" t="n">
+        <v>-96</v>
       </c>
       <c r="G56" s="30">
         <f>G55+F56</f>
@@ -3606,21 +3610,21 @@
       </c>
       <c r="C57" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D57" s="31" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D57" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E57" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F57" s="29" t="n">
-        <v>-96</v>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F57" s="32" t="n">
+        <v>-404</v>
       </c>
       <c r="G57" s="30">
         <f>G56+F57</f>
@@ -3637,21 +3641,18 @@
       </c>
       <c r="C58" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D58" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E58" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F58" s="29" t="n">
-        <v>-404</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D58" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E58" s="27" t="inlineStr"/>
+      <c r="F58" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G58" s="30">
         <f>G57+F58</f>
@@ -3660,7 +3661,7 @@
     </row>
     <row r="59">
       <c r="A59" s="25" t="n">
-        <v>46539</v>
+        <v>46567</v>
       </c>
       <c r="B59" s="26">
         <f>DATE(YEAR(A59),MONTH(A59),1)</f>
@@ -3668,18 +3669,17 @@
       </c>
       <c r="C59" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D59" s="32" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D59" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E59" s="27" t="inlineStr"/>
-      <c r="F59" s="33">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F59" s="32" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G59" s="30">
         <f>G58+F59</f>
@@ -3696,17 +3696,17 @@
       </c>
       <c r="C60" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D60" s="28" t="inlineStr">
+          <t>Paga extra de junio</t>
+        </is>
+      </c>
+      <c r="D60" s="31" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
       </c>
       <c r="E60" s="27" t="inlineStr"/>
-      <c r="F60" s="29" t="n">
-        <v>3173.56</v>
+      <c r="F60" s="32" t="n">
+        <v>1989.05</v>
       </c>
       <c r="G60" s="30">
         <f>G59+F60</f>
@@ -3715,7 +3715,7 @@
     </row>
     <row r="61">
       <c r="A61" s="25" t="n">
-        <v>46567</v>
+        <v>46569</v>
       </c>
       <c r="B61" s="26">
         <f>DATE(YEAR(A61),MONTH(A61),1)</f>
@@ -3723,17 +3723,21 @@
       </c>
       <c r="C61" s="27" t="inlineStr">
         <is>
-          <t>Paga extra de junio</t>
-        </is>
-      </c>
-      <c r="D61" s="28" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E61" s="27" t="inlineStr"/>
-      <c r="F61" s="29" t="n">
-        <v>1989.05</v>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D61" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E61" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F61" s="32" t="n">
+        <v>-279.08</v>
       </c>
       <c r="G61" s="30">
         <f>G60+F61</f>
@@ -3750,21 +3754,21 @@
       </c>
       <c r="C62" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D62" s="31" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D62" s="36" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E62" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F62" s="29" t="n">
-        <v>-279.08</v>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F62" s="32" t="n">
+        <v>-220.92</v>
       </c>
       <c r="G62" s="30">
         <f>G61+F62</f>
@@ -3781,21 +3785,18 @@
       </c>
       <c r="C63" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D63" s="36" t="inlineStr">
-        <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E63" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
-      <c r="F63" s="29" t="n">
-        <v>-220.92</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D63" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E63" s="27" t="inlineStr"/>
+      <c r="F63" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G63" s="30">
         <f>G62+F63</f>
@@ -3804,7 +3805,7 @@
     </row>
     <row r="64">
       <c r="A64" s="25" t="n">
-        <v>46569</v>
+        <v>46597</v>
       </c>
       <c r="B64" s="26">
         <f>DATE(YEAR(A64),MONTH(A64),1)</f>
@@ -3812,18 +3813,17 @@
       </c>
       <c r="C64" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D64" s="32" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D64" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E64" s="27" t="inlineStr"/>
-      <c r="F64" s="33">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F64" s="32" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G64" s="30">
         <f>G63+F64</f>
@@ -3832,7 +3832,7 @@
     </row>
     <row r="65">
       <c r="A65" s="25" t="n">
-        <v>46597</v>
+        <v>46600</v>
       </c>
       <c r="B65" s="26">
         <f>DATE(YEAR(A65),MONTH(A65),1)</f>
@@ -3840,17 +3840,21 @@
       </c>
       <c r="C65" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D65" s="28" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E65" s="27" t="inlineStr"/>
-      <c r="F65" s="29" t="n">
-        <v>3173.56</v>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D65" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E65" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F65" s="32" t="n">
+        <v>-500</v>
       </c>
       <c r="G65" s="30">
         <f>G64+F65</f>
@@ -3867,21 +3871,18 @@
       </c>
       <c r="C66" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D66" s="31" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E66" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F66" s="29" t="n">
-        <v>-500</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D66" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E66" s="27" t="inlineStr"/>
+      <c r="F66" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G66" s="30">
         <f>G65+F66</f>
@@ -3890,7 +3891,7 @@
     </row>
     <row r="67">
       <c r="A67" s="25" t="n">
-        <v>46600</v>
+        <v>46628</v>
       </c>
       <c r="B67" s="26">
         <f>DATE(YEAR(A67),MONTH(A67),1)</f>
@@ -3898,18 +3899,17 @@
       </c>
       <c r="C67" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D67" s="32" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D67" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E67" s="27" t="inlineStr"/>
-      <c r="F67" s="33">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F67" s="32" t="n">
+        <v>2280.25</v>
       </c>
       <c r="G67" s="30">
         <f>G66+F67</f>
@@ -3918,7 +3918,7 @@
     </row>
     <row r="68">
       <c r="A68" s="25" t="n">
-        <v>46628</v>
+        <v>46631</v>
       </c>
       <c r="B68" s="26">
         <f>DATE(YEAR(A68),MONTH(A68),1)</f>
@@ -3926,17 +3926,21 @@
       </c>
       <c r="C68" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D68" s="28" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E68" s="27" t="inlineStr"/>
-      <c r="F68" s="29" t="n">
-        <v>2280.25</v>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D68" s="33" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E68" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F68" s="32" t="n">
+        <v>-447.85</v>
       </c>
       <c r="G68" s="30">
         <f>G67+F68</f>
@@ -3953,21 +3957,18 @@
       </c>
       <c r="C69" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D69" s="31" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E69" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
-      <c r="F69" s="29" t="n">
-        <v>-447.85</v>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D69" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E69" s="27" t="inlineStr"/>
+      <c r="F69" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G69" s="30">
         <f>G68+F69</f>
@@ -3976,7 +3977,7 @@
     </row>
     <row r="70">
       <c r="A70" s="25" t="n">
-        <v>46631</v>
+        <v>46659</v>
       </c>
       <c r="B70" s="26">
         <f>DATE(YEAR(A70),MONTH(A70),1)</f>
@@ -3984,18 +3985,17 @@
       </c>
       <c r="C70" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D70" s="32" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D70" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E70" s="27" t="inlineStr"/>
-      <c r="F70" s="33">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F70" s="32" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G70" s="30">
         <f>G69+F70</f>
@@ -4004,7 +4004,7 @@
     </row>
     <row r="71">
       <c r="A71" s="25" t="n">
-        <v>46659</v>
+        <v>46661</v>
       </c>
       <c r="B71" s="26">
         <f>DATE(YEAR(A71),MONTH(A71),1)</f>
@@ -4012,17 +4012,18 @@
       </c>
       <c r="C71" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
+          <t>Gastos de vida</t>
         </is>
       </c>
       <c r="D71" s="28" t="inlineStr">
         <is>
-          <t>Ingreso</t>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E71" s="27" t="inlineStr"/>
-      <c r="F71" s="29" t="n">
-        <v>3173.56</v>
+      <c r="F71" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G71" s="30">
         <f>G70+F71</f>
@@ -4031,7 +4032,7 @@
     </row>
     <row r="72">
       <c r="A72" s="25" t="n">
-        <v>46661</v>
+        <v>46689</v>
       </c>
       <c r="B72" s="26">
         <f>DATE(YEAR(A72),MONTH(A72),1)</f>
@@ -4039,54 +4040,26 @@
       </c>
       <c r="C72" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D72" s="32" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D72" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E72" s="27" t="inlineStr"/>
-      <c r="F72" s="33">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F72" s="32" t="n">
+        <v>2490.44</v>
       </c>
       <c r="G72" s="30">
         <f>G71+F72</f>
         <v/>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="25" t="n">
-        <v>46689</v>
-      </c>
-      <c r="B73" s="26">
-        <f>DATE(YEAR(A73),MONTH(A73),1)</f>
-        <v/>
-      </c>
-      <c r="C73" s="27" t="inlineStr">
-        <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D73" s="28" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E73" s="27" t="inlineStr"/>
-      <c r="F73" s="29" t="n">
-        <v>2490.44</v>
-      </c>
-      <c r="G73" s="30">
-        <f>G72+F73</f>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G73"/>
-  <conditionalFormatting sqref="G2:G73">
+  <autoFilter ref="A1:G72"/>
+  <conditionalFormatting sqref="G2:G72">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="1">
       <formula>0</formula>
     </cfRule>
@@ -4130,7 +4103,7 @@
         </is>
       </c>
       <c r="B4" s="40" t="n">
-        <v>46308</v>
+        <v>46312</v>
       </c>
       <c r="C4" s="13" t="inlineStr">
         <is>
@@ -4149,7 +4122,7 @@
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>Saldo en cuenta el 13 oct 2026, según el usuario</t>
+          <t>Saldo en cuenta el 17 oct 2026, según el usuario</t>
         </is>
       </c>
     </row>
@@ -4164,7 +4137,7 @@
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>Con el puente de Joserra tienes 765 €; para llegar al 1 nov, máximo ~550 €</t>
+          <t>Estimación. Con más de ~350 € el 1 dic queda en negativo (salvo que aplaces los aplazables ese mes)</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4174,7 @@
     <row r="10">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>Nóminas, pagas extra y variable: netas, según la previsión del desplazamiento.</t>
+          <t>Nóminas, pagas extra y variable: netas, según la previsión del desplazamiento (octubre: 3.100 €, confirmado por el usuario).</t>
         </is>
       </c>
     </row>
@@ -4222,7 +4195,7 @@
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Escenario: hoy pagas Smartcredito y Joserra te deja 600 € (se le devuelven 1.000 € el 29 dic). Sin volver a pedir Moneyman ni Smartcredito. Ama el 29 nov.</t>
+          <t>Escenario: nómina de octubre de 3.100 €, Smartcredito el 14 nov, sin préstamos puente ni volver a pedir Moneyman. Ama el 29 nov, Vivus liquidado el 29 nov.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plan: Ama son 800 € y se pagan el 29 oct; escenario con puente de 600 € de Joserra
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JEd5Mo2HQL6TrpXUCZoFXP
</commit_message>
<xml_diff>
--- a/excel/plan_de_pagos.xlsx
+++ b/excel/plan_de_pagos.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Supuestos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Calendario'!$A$1:$G$72</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Calendario'!$A$1:$G$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -105,17 +105,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FDE2E2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DBEAFE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
   </fills>
@@ -150,14 +150,14 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -177,8 +177,8 @@
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -653,23 +653,23 @@
         <v>46296</v>
       </c>
       <c r="B2" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A2)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Ingreso",Calendario!$B$3:$B$74,A2)</f>
         <v/>
       </c>
       <c r="C2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Gasto",Calendario!$B$3:$B$74,A2)</f>
         <v/>
       </c>
       <c r="D2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Fijo",Calendario!$B$3:$B$74,A2)</f>
         <v/>
       </c>
       <c r="E2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Aplazable",Calendario!$B$3:$B$74,A2)</f>
         <v/>
       </c>
       <c r="F2" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Amigo",Calendario!$B$3:$B$74,A2)</f>
         <v/>
       </c>
       <c r="G2" s="3">
@@ -690,23 +690,23 @@
         <v>46327</v>
       </c>
       <c r="B3" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A3)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Ingreso",Calendario!$B$3:$B$74,A3)</f>
         <v/>
       </c>
       <c r="C3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Gasto",Calendario!$B$3:$B$74,A3)</f>
         <v/>
       </c>
       <c r="D3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Fijo",Calendario!$B$3:$B$74,A3)</f>
         <v/>
       </c>
       <c r="E3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Aplazable",Calendario!$B$3:$B$74,A3)</f>
         <v/>
       </c>
       <c r="F3" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Amigo",Calendario!$B$3:$B$74,A3)</f>
         <v/>
       </c>
       <c r="G3" s="3">
@@ -727,23 +727,23 @@
         <v>46357</v>
       </c>
       <c r="B4" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A4)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Ingreso",Calendario!$B$3:$B$74,A4)</f>
         <v/>
       </c>
       <c r="C4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Gasto",Calendario!$B$3:$B$74,A4)</f>
         <v/>
       </c>
       <c r="D4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Fijo",Calendario!$B$3:$B$74,A4)</f>
         <v/>
       </c>
       <c r="E4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Aplazable",Calendario!$B$3:$B$74,A4)</f>
         <v/>
       </c>
       <c r="F4" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Amigo",Calendario!$B$3:$B$74,A4)</f>
         <v/>
       </c>
       <c r="G4" s="3">
@@ -764,23 +764,23 @@
         <v>46388</v>
       </c>
       <c r="B5" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A5)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Ingreso",Calendario!$B$3:$B$74,A5)</f>
         <v/>
       </c>
       <c r="C5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Gasto",Calendario!$B$3:$B$74,A5)</f>
         <v/>
       </c>
       <c r="D5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Fijo",Calendario!$B$3:$B$74,A5)</f>
         <v/>
       </c>
       <c r="E5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Aplazable",Calendario!$B$3:$B$74,A5)</f>
         <v/>
       </c>
       <c r="F5" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Amigo",Calendario!$B$3:$B$74,A5)</f>
         <v/>
       </c>
       <c r="G5" s="3">
@@ -801,23 +801,23 @@
         <v>46419</v>
       </c>
       <c r="B6" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A6)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Ingreso",Calendario!$B$3:$B$74,A6)</f>
         <v/>
       </c>
       <c r="C6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Gasto",Calendario!$B$3:$B$74,A6)</f>
         <v/>
       </c>
       <c r="D6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Fijo",Calendario!$B$3:$B$74,A6)</f>
         <v/>
       </c>
       <c r="E6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Aplazable",Calendario!$B$3:$B$74,A6)</f>
         <v/>
       </c>
       <c r="F6" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Amigo",Calendario!$B$3:$B$74,A6)</f>
         <v/>
       </c>
       <c r="G6" s="3">
@@ -838,23 +838,23 @@
         <v>46447</v>
       </c>
       <c r="B7" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A7)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Ingreso",Calendario!$B$3:$B$74,A7)</f>
         <v/>
       </c>
       <c r="C7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Gasto",Calendario!$B$3:$B$74,A7)</f>
         <v/>
       </c>
       <c r="D7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Fijo",Calendario!$B$3:$B$74,A7)</f>
         <v/>
       </c>
       <c r="E7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Aplazable",Calendario!$B$3:$B$74,A7)</f>
         <v/>
       </c>
       <c r="F7" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Amigo",Calendario!$B$3:$B$74,A7)</f>
         <v/>
       </c>
       <c r="G7" s="3">
@@ -875,23 +875,23 @@
         <v>46478</v>
       </c>
       <c r="B8" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A8)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Ingreso",Calendario!$B$3:$B$74,A8)</f>
         <v/>
       </c>
       <c r="C8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Gasto",Calendario!$B$3:$B$74,A8)</f>
         <v/>
       </c>
       <c r="D8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Fijo",Calendario!$B$3:$B$74,A8)</f>
         <v/>
       </c>
       <c r="E8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Aplazable",Calendario!$B$3:$B$74,A8)</f>
         <v/>
       </c>
       <c r="F8" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Amigo",Calendario!$B$3:$B$74,A8)</f>
         <v/>
       </c>
       <c r="G8" s="3">
@@ -912,23 +912,23 @@
         <v>46508</v>
       </c>
       <c r="B9" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A9)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Ingreso",Calendario!$B$3:$B$74,A9)</f>
         <v/>
       </c>
       <c r="C9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Gasto",Calendario!$B$3:$B$74,A9)</f>
         <v/>
       </c>
       <c r="D9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Fijo",Calendario!$B$3:$B$74,A9)</f>
         <v/>
       </c>
       <c r="E9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Aplazable",Calendario!$B$3:$B$74,A9)</f>
         <v/>
       </c>
       <c r="F9" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Amigo",Calendario!$B$3:$B$74,A9)</f>
         <v/>
       </c>
       <c r="G9" s="3">
@@ -949,23 +949,23 @@
         <v>46539</v>
       </c>
       <c r="B10" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A10)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Ingreso",Calendario!$B$3:$B$74,A10)</f>
         <v/>
       </c>
       <c r="C10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Gasto",Calendario!$B$3:$B$74,A10)</f>
         <v/>
       </c>
       <c r="D10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Fijo",Calendario!$B$3:$B$74,A10)</f>
         <v/>
       </c>
       <c r="E10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Aplazable",Calendario!$B$3:$B$74,A10)</f>
         <v/>
       </c>
       <c r="F10" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Amigo",Calendario!$B$3:$B$74,A10)</f>
         <v/>
       </c>
       <c r="G10" s="3">
@@ -986,23 +986,23 @@
         <v>46569</v>
       </c>
       <c r="B11" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A11)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Ingreso",Calendario!$B$3:$B$74,A11)</f>
         <v/>
       </c>
       <c r="C11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Gasto",Calendario!$B$3:$B$74,A11)</f>
         <v/>
       </c>
       <c r="D11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Fijo",Calendario!$B$3:$B$74,A11)</f>
         <v/>
       </c>
       <c r="E11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Aplazable",Calendario!$B$3:$B$74,A11)</f>
         <v/>
       </c>
       <c r="F11" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Amigo",Calendario!$B$3:$B$74,A11)</f>
         <v/>
       </c>
       <c r="G11" s="3">
@@ -1023,23 +1023,23 @@
         <v>46600</v>
       </c>
       <c r="B12" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A12)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Ingreso",Calendario!$B$3:$B$74,A12)</f>
         <v/>
       </c>
       <c r="C12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Gasto",Calendario!$B$3:$B$74,A12)</f>
         <v/>
       </c>
       <c r="D12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Fijo",Calendario!$B$3:$B$74,A12)</f>
         <v/>
       </c>
       <c r="E12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Aplazable",Calendario!$B$3:$B$74,A12)</f>
         <v/>
       </c>
       <c r="F12" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Amigo",Calendario!$B$3:$B$74,A12)</f>
         <v/>
       </c>
       <c r="G12" s="3">
@@ -1060,23 +1060,23 @@
         <v>46631</v>
       </c>
       <c r="B13" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A13)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Ingreso",Calendario!$B$3:$B$74,A13)</f>
         <v/>
       </c>
       <c r="C13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Gasto",Calendario!$B$3:$B$74,A13)</f>
         <v/>
       </c>
       <c r="D13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Fijo",Calendario!$B$3:$B$74,A13)</f>
         <v/>
       </c>
       <c r="E13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Aplazable",Calendario!$B$3:$B$74,A13)</f>
         <v/>
       </c>
       <c r="F13" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Amigo",Calendario!$B$3:$B$74,A13)</f>
         <v/>
       </c>
       <c r="G13" s="3">
@@ -1097,23 +1097,23 @@
         <v>46661</v>
       </c>
       <c r="B14" s="3">
-        <f>SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Ingreso",Calendario!$B$3:$B$72,A14)</f>
+        <f>SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Ingreso",Calendario!$B$3:$B$74,A14)</f>
         <v/>
       </c>
       <c r="C14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Gasto",Calendario!$B$3:$B$72,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Gasto",Calendario!$B$3:$B$74,A14)</f>
         <v/>
       </c>
       <c r="D14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Fijo",Calendario!$B$3:$B$72,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Fijo",Calendario!$B$3:$B$74,A14)</f>
         <v/>
       </c>
       <c r="E14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Aplazable",Calendario!$B$3:$B$72,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Aplazable",Calendario!$B$3:$B$74,A14)</f>
         <v/>
       </c>
       <c r="F14" s="3">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$D$3:$D$72,"Amigo",Calendario!$B$3:$B$72,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$D$3:$D$74,"Amigo",Calendario!$B$3:$B$74,A14)</f>
         <v/>
       </c>
       <c r="G14" s="3">
@@ -1171,7 +1171,7 @@
         </is>
       </c>
       <c r="C17" s="4">
-        <f>MIN(Calendario!G2:G72)</f>
+        <f>MIN(Calendario!G2:G74)</f>
         <v/>
       </c>
     </row>
@@ -1182,7 +1182,7 @@
         </is>
       </c>
       <c r="C18" s="7">
-        <f>INDEX(Calendario!A2:A72,MATCH(C17,Calendario!G2:G72,0))</f>
+        <f>INDEX(Calendario!A2:A74,MATCH(C17,Calendario!G2:G74,0))</f>
         <v/>
       </c>
     </row>
@@ -1283,7 +1283,7 @@
         <v>1400</v>
       </c>
       <c r="E2" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A2)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$E$3:$E$74,A2)</f>
         <v/>
       </c>
       <c r="F2" s="3">
@@ -1291,7 +1291,7 @@
         <v/>
       </c>
       <c r="G2" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A2)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$74,Calendario!$E$3:$E$74,A2)</f>
         <v/>
       </c>
       <c r="H2" s="13" t="inlineStr">
@@ -1323,7 +1323,7 @@
         <v>2148</v>
       </c>
       <c r="E3" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A3)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$E$3:$E$74,A3)</f>
         <v/>
       </c>
       <c r="F3" s="3">
@@ -1331,7 +1331,7 @@
         <v/>
       </c>
       <c r="G3" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A3)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$74,Calendario!$E$3:$E$74,A3)</f>
         <v/>
       </c>
       <c r="H3" s="13" t="inlineStr">
@@ -1363,7 +1363,7 @@
         <v>435</v>
       </c>
       <c r="E4" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A4)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$E$3:$E$74,A4)</f>
         <v/>
       </c>
       <c r="F4" s="3">
@@ -1371,7 +1371,7 @@
         <v/>
       </c>
       <c r="G4" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A4)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$74,Calendario!$E$3:$E$74,A4)</f>
         <v/>
       </c>
       <c r="H4" s="13" t="inlineStr">
@@ -1403,7 +1403,7 @@
         <v>1994.93</v>
       </c>
       <c r="E5" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A5)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$E$3:$E$74,A5)</f>
         <v/>
       </c>
       <c r="F5" s="3">
@@ -1411,7 +1411,7 @@
         <v/>
       </c>
       <c r="G5" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A5)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$74,Calendario!$E$3:$E$74,A5)</f>
         <v/>
       </c>
       <c r="H5" s="13" t="inlineStr">
@@ -1443,7 +1443,7 @@
         <v>693.34</v>
       </c>
       <c r="E6" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A6)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$E$3:$E$74,A6)</f>
         <v/>
       </c>
       <c r="F6" s="3">
@@ -1451,7 +1451,7 @@
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A6)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$74,Calendario!$E$3:$E$74,A6)</f>
         <v/>
       </c>
       <c r="H6" s="13" t="inlineStr">
@@ -1483,7 +1483,7 @@
         <v>923.61</v>
       </c>
       <c r="E7" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A7)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$E$3:$E$74,A7)</f>
         <v/>
       </c>
       <c r="F7" s="3">
@@ -1491,7 +1491,7 @@
         <v/>
       </c>
       <c r="G7" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A7)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$74,Calendario!$E$3:$E$74,A7)</f>
         <v/>
       </c>
       <c r="H7" s="13" t="inlineStr">
@@ -1523,7 +1523,7 @@
         <v>1483.63</v>
       </c>
       <c r="E8" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A8)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$E$3:$E$74,A8)</f>
         <v/>
       </c>
       <c r="F8" s="3">
@@ -1531,7 +1531,7 @@
         <v/>
       </c>
       <c r="G8" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A8)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$74,Calendario!$E$3:$E$74,A8)</f>
         <v/>
       </c>
       <c r="H8" s="13" t="inlineStr">
@@ -1563,7 +1563,7 @@
         <v>2326.76</v>
       </c>
       <c r="E9" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A9)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$E$3:$E$74,A9)</f>
         <v/>
       </c>
       <c r="F9" s="3">
@@ -1571,7 +1571,7 @@
         <v/>
       </c>
       <c r="G9" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A9)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$74,Calendario!$E$3:$E$74,A9)</f>
         <v/>
       </c>
       <c r="H9" s="13" t="inlineStr">
@@ -1600,10 +1600,10 @@
         </is>
       </c>
       <c r="D10" s="10" t="n">
-        <v>600</v>
+        <v>800</v>
       </c>
       <c r="E10" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A10)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$E$3:$E$74,A10)</f>
         <v/>
       </c>
       <c r="F10" s="3">
@@ -1611,12 +1611,12 @@
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A10)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$74,Calendario!$E$3:$E$74,A10)</f>
         <v/>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>Prioridad: 29 nov, con la nómina</t>
+          <t>Fundamental en octubre: 29 oct, con la nómina</t>
         </is>
       </c>
       <c r="I10" s="10" t="n">
@@ -1640,10 +1640,10 @@
         </is>
       </c>
       <c r="D11" s="10" t="n">
-        <v>400</v>
+        <v>1000</v>
       </c>
       <c r="E11" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A11)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$E$3:$E$74,A11)</f>
         <v/>
       </c>
       <c r="F11" s="3">
@@ -1651,12 +1651,12 @@
         <v/>
       </c>
       <c r="G11" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A11)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$74,Calendario!$E$3:$E$74,A11)</f>
         <v/>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>Sin plazo ni interés. Se devuelve antes de fin de año</t>
+          <t>400 € anteriores + 600 € de puente (17 oct). Todo se devuelve el 29 dic</t>
         </is>
       </c>
       <c r="I11" s="10" t="n">
@@ -1683,7 +1683,7 @@
         <v>300</v>
       </c>
       <c r="E12" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A12)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$E$3:$E$74,A12)</f>
         <v/>
       </c>
       <c r="F12" s="3">
@@ -1691,7 +1691,7 @@
         <v/>
       </c>
       <c r="G12" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A12)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$74,Calendario!$E$3:$E$74,A12)</f>
         <v/>
       </c>
       <c r="H12" s="13" t="inlineStr">
@@ -1723,7 +1723,7 @@
         <v>1700</v>
       </c>
       <c r="E13" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A13)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$E$3:$E$74,A13)</f>
         <v/>
       </c>
       <c r="F13" s="3">
@@ -1731,7 +1731,7 @@
         <v/>
       </c>
       <c r="G13" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A13)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$74,Calendario!$E$3:$E$74,A13)</f>
         <v/>
       </c>
       <c r="H13" s="13" t="inlineStr">
@@ -1763,7 +1763,7 @@
         <v>2500</v>
       </c>
       <c r="E14" s="11">
-        <f>-SUMIFS(Calendario!$F$3:$F$72,Calendario!$E$3:$E$72,A14)</f>
+        <f>-SUMIFS(Calendario!$F$3:$F$74,Calendario!$E$3:$E$74,A14)</f>
         <v/>
       </c>
       <c r="F14" s="3">
@@ -1771,7 +1771,7 @@
         <v/>
       </c>
       <c r="G14" s="12">
-        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$72,Calendario!$E$3:$E$72,A14)</f>
+        <f>_xlfn.MAXIFS(Calendario!$A$3:$A$74,Calendario!$E$3:$E$74,A14)</f>
         <v/>
       </c>
       <c r="H14" s="13" t="inlineStr">
@@ -1869,7 +1869,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J72"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1997,7 +1997,7 @@
     </row>
     <row r="4">
       <c r="A4" s="25" t="n">
-        <v>46324</v>
+        <v>46312</v>
       </c>
       <c r="B4" s="26">
         <f>DATE(YEAR(A4),MONTH(A4),1)</f>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="C4" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
+          <t>Préstamo puente de Joserra (sin intereses)</t>
         </is>
       </c>
       <c r="D4" s="31" t="inlineStr">
@@ -2015,7 +2015,7 @@
       </c>
       <c r="E4" s="27" t="inlineStr"/>
       <c r="F4" s="32" t="n">
-        <v>3100</v>
+        <v>600</v>
       </c>
       <c r="G4" s="30">
         <f>G3+F4</f>
@@ -2034,7 +2034,7 @@
     </row>
     <row r="5">
       <c r="A5" s="25" t="n">
-        <v>46327</v>
+        <v>46324</v>
       </c>
       <c r="B5" s="26">
         <f>DATE(YEAR(A5),MONTH(A5),1)</f>
@@ -2042,27 +2042,23 @@
       </c>
       <c r="C5" s="27" t="inlineStr">
         <is>
-          <t>Moneyman · pago (sin volver a pedirlo)</t>
-        </is>
-      </c>
-      <c r="D5" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E5" s="27" t="inlineStr">
-        <is>
-          <t>Moneyman</t>
-        </is>
-      </c>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D5" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr"/>
       <c r="F5" s="32" t="n">
-        <v>-1400</v>
+        <v>3100</v>
       </c>
       <c r="G5" s="30">
         <f>G4+F5</f>
         <v/>
       </c>
-      <c r="I5" s="34" t="inlineStr">
+      <c r="I5" s="33" t="inlineStr">
         <is>
           <t>Ingreso</t>
         </is>
@@ -2075,7 +2071,7 @@
     </row>
     <row r="6">
       <c r="A6" s="25" t="n">
-        <v>46327</v>
+        <v>46324</v>
       </c>
       <c r="B6" s="26">
         <f>DATE(YEAR(A6),MONTH(A6),1)</f>
@@ -2083,21 +2079,21 @@
       </c>
       <c r="C6" s="27" t="inlineStr">
         <is>
-          <t>Vivus · cuota 1/4 (no aplazable)</t>
-        </is>
-      </c>
-      <c r="D6" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Devolución a Ama</t>
+        </is>
+      </c>
+      <c r="D6" s="34" t="inlineStr">
+        <is>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E6" s="27" t="inlineStr">
         <is>
-          <t>Vivus</t>
+          <t>Ama</t>
         </is>
       </c>
       <c r="F6" s="32" t="n">
-        <v>-537</v>
+        <v>-800</v>
       </c>
       <c r="G6" s="30">
         <f>G5+F6</f>
@@ -2124,17 +2120,21 @@
       </c>
       <c r="C7" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · pagas 231,11 € y lo vuelves a pedir (neto 0)</t>
+          <t>Moneyman · pago (sin volver a pedirlo)</t>
         </is>
       </c>
       <c r="D7" s="36" t="inlineStr">
         <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E7" s="27" t="inlineStr"/>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>Moneyman</t>
+        </is>
+      </c>
       <c r="F7" s="32" t="n">
-        <v>0</v>
+        <v>-1400</v>
       </c>
       <c r="G7" s="30">
         <f>G6+F7</f>
@@ -2151,17 +2151,21 @@
       </c>
       <c r="C8" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · pagas 307,87 € y lo vuelves a pedir (neto 0)</t>
+          <t>Vivus · cuota 1/4 (no aplazable)</t>
         </is>
       </c>
       <c r="D8" s="36" t="inlineStr">
         <is>
-          <t>Aplazable</t>
-        </is>
-      </c>
-      <c r="E8" s="27" t="inlineStr"/>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>Vivus</t>
+        </is>
+      </c>
       <c r="F8" s="32" t="n">
-        <v>0</v>
+        <v>-537</v>
       </c>
       <c r="G8" s="30">
         <f>G7+F8</f>
@@ -2183,10 +2187,10 @@
       </c>
       <c r="C9" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · pagas 494,54 € y lo vuelves a pedir (neto 0)</t>
-        </is>
-      </c>
-      <c r="D9" s="36" t="inlineStr">
+          <t>Pagolisto 1 · pagas 231,11 € y lo vuelves a pedir (neto 0)</t>
+        </is>
+      </c>
+      <c r="D9" s="37" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
@@ -2210,21 +2214,17 @@
       </c>
       <c r="C10" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D10" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E10" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
+          <t>Pagolisto 2 · pagas 307,87 € y lo vuelves a pedir (neto 0)</t>
+        </is>
+      </c>
+      <c r="D10" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr"/>
       <c r="F10" s="32" t="n">
-        <v>-96</v>
+        <v>0</v>
       </c>
       <c r="G10" s="30">
         <f>G9+F10</f>
@@ -2241,21 +2241,17 @@
       </c>
       <c r="C11" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
-        </is>
-      </c>
-      <c r="D11" s="36" t="inlineStr">
+          <t>Crédito Santander 1 · pagas 494,54 € y lo vuelves a pedir (neto 0)</t>
+        </is>
+      </c>
+      <c r="D11" s="37" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
-      <c r="E11" s="27" t="inlineStr">
-        <is>
-          <t>Crédito Santander 2</t>
-        </is>
-      </c>
+      <c r="E11" s="27" t="inlineStr"/>
       <c r="F11" s="32" t="n">
-        <v>-122.46</v>
+        <v>0</v>
       </c>
       <c r="G11" s="30">
         <f>G10+F11</f>
@@ -2272,18 +2268,17 @@
       </c>
       <c r="C12" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D12" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Crédito Santander 2 · pagas 122,46 € y lo vuelves a pedir (neto 0)</t>
+        </is>
+      </c>
+      <c r="D12" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E12" s="27" t="inlineStr"/>
-      <c r="F12" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F12" s="32" t="n">
+        <v>0</v>
       </c>
       <c r="G12" s="30">
         <f>G11+F12</f>
@@ -2292,7 +2287,7 @@
     </row>
     <row r="13">
       <c r="A13" s="25" t="n">
-        <v>46340</v>
+        <v>46327</v>
       </c>
       <c r="B13" s="26">
         <f>DATE(YEAR(A13),MONTH(A13),1)</f>
@@ -2300,21 +2295,21 @@
       </c>
       <c r="C13" s="27" t="inlineStr">
         <is>
-          <t>Smartcredito · pago único</t>
-        </is>
-      </c>
-      <c r="D13" s="33" t="inlineStr">
+          <t>Santander (préstamo) · cuota</t>
+        </is>
+      </c>
+      <c r="D13" s="36" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
       </c>
       <c r="E13" s="27" t="inlineStr">
         <is>
-          <t>Smartcredito</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F13" s="32" t="n">
-        <v>-435</v>
+        <v>-96</v>
       </c>
       <c r="G13" s="30">
         <f>G12+F13</f>
@@ -2323,7 +2318,7 @@
     </row>
     <row r="14">
       <c r="A14" s="25" t="n">
-        <v>46355</v>
+        <v>46327</v>
       </c>
       <c r="B14" s="26">
         <f>DATE(YEAR(A14),MONTH(A14),1)</f>
@@ -2331,17 +2326,18 @@
       </c>
       <c r="C14" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D14" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D14" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E14" s="27" t="inlineStr"/>
-      <c r="F14" s="32" t="n">
-        <v>3453.01</v>
+      <c r="F14" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G14" s="30">
         <f>G13+F14</f>
@@ -2350,7 +2346,7 @@
     </row>
     <row r="15">
       <c r="A15" s="25" t="n">
-        <v>46355</v>
+        <v>46340</v>
       </c>
       <c r="B15" s="26">
         <f>DATE(YEAR(A15),MONTH(A15),1)</f>
@@ -2358,21 +2354,21 @@
       </c>
       <c r="C15" s="27" t="inlineStr">
         <is>
-          <t>Vivus · liquidación del resto (total 1.500 € en vez de 2.148 €)</t>
-        </is>
-      </c>
-      <c r="D15" s="33" t="inlineStr">
+          <t>Smartcredito · pago único</t>
+        </is>
+      </c>
+      <c r="D15" s="36" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
       </c>
       <c r="E15" s="27" t="inlineStr">
         <is>
-          <t>Vivus</t>
+          <t>Smartcredito</t>
         </is>
       </c>
       <c r="F15" s="32" t="n">
-        <v>-963</v>
+        <v>-435</v>
       </c>
       <c r="G15" s="30">
         <f>G14+F15</f>
@@ -2389,21 +2385,17 @@
       </c>
       <c r="C16" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Ama</t>
-        </is>
-      </c>
-      <c r="D16" s="37" t="inlineStr">
-        <is>
-          <t>Amigo</t>
-        </is>
-      </c>
-      <c r="E16" s="27" t="inlineStr">
-        <is>
-          <t>Ama</t>
-        </is>
-      </c>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D16" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E16" s="27" t="inlineStr"/>
       <c r="F16" s="32" t="n">
-        <v>-600</v>
+        <v>3453.01</v>
       </c>
       <c r="G16" s="30">
         <f>G15+F16</f>
@@ -2412,7 +2404,7 @@
     </row>
     <row r="17">
       <c r="A17" s="25" t="n">
-        <v>46357</v>
+        <v>46355</v>
       </c>
       <c r="B17" s="26">
         <f>DATE(YEAR(A17),MONTH(A17),1)</f>
@@ -2420,21 +2412,21 @@
       </c>
       <c r="C17" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D17" s="33" t="inlineStr">
+          <t>Vivus · liquidación del resto (total 1.500 € en vez de 2.148 €)</t>
+        </is>
+      </c>
+      <c r="D17" s="36" t="inlineStr">
         <is>
           <t>Fijo</t>
         </is>
       </c>
       <c r="E17" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Vivus</t>
         </is>
       </c>
       <c r="F17" s="32" t="n">
-        <v>-96</v>
+        <v>-963</v>
       </c>
       <c r="G17" s="30">
         <f>G16+F17</f>
@@ -2451,21 +2443,21 @@
       </c>
       <c r="C18" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
+          <t>Santander (préstamo) · cuota</t>
         </is>
       </c>
       <c r="D18" s="36" t="inlineStr">
         <is>
-          <t>Aplazable</t>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E18" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F18" s="32" t="n">
-        <v>-122.46</v>
+        <v>-96</v>
       </c>
       <c r="G18" s="30">
         <f>G17+F18</f>
@@ -2482,21 +2474,21 @@
       </c>
       <c r="C19" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 1/3</t>
-        </is>
-      </c>
-      <c r="D19" s="36" t="inlineStr">
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D19" s="37" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E19" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1</t>
+          <t>Crédito Santander 2</t>
         </is>
       </c>
       <c r="F19" s="32" t="n">
-        <v>-231.11</v>
+        <v>-122.46</v>
       </c>
       <c r="G19" s="30">
         <f>G18+F19</f>
@@ -2513,21 +2505,21 @@
       </c>
       <c r="C20" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 1/3</t>
-        </is>
-      </c>
-      <c r="D20" s="36" t="inlineStr">
+          <t>Pagolisto 1 · cuota 1/3</t>
+        </is>
+      </c>
+      <c r="D20" s="37" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E20" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2</t>
+          <t>Pagolisto 1</t>
         </is>
       </c>
       <c r="F20" s="32" t="n">
-        <v>-307.87</v>
+        <v>-231.11</v>
       </c>
       <c r="G20" s="30">
         <f>G19+F20</f>
@@ -2544,21 +2536,21 @@
       </c>
       <c r="C21" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 1/3</t>
-        </is>
-      </c>
-      <c r="D21" s="36" t="inlineStr">
+          <t>Pagolisto 2 · cuota 1/3</t>
+        </is>
+      </c>
+      <c r="D21" s="37" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E21" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1</t>
+          <t>Pagolisto 2</t>
         </is>
       </c>
       <c r="F21" s="32" t="n">
-        <v>-494.54</v>
+        <v>-307.87</v>
       </c>
       <c r="G21" s="30">
         <f>G20+F21</f>
@@ -2575,18 +2567,21 @@
       </c>
       <c r="C22" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D22" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E22" s="27" t="inlineStr"/>
-      <c r="F22" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Crédito Santander 1 · cuota 1/3</t>
+        </is>
+      </c>
+      <c r="D22" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E22" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 1</t>
+        </is>
+      </c>
+      <c r="F22" s="32" t="n">
+        <v>-494.54</v>
       </c>
       <c r="G22" s="30">
         <f>G21+F22</f>
@@ -2595,7 +2590,7 @@
     </row>
     <row r="23">
       <c r="A23" s="25" t="n">
-        <v>46385</v>
+        <v>46357</v>
       </c>
       <c r="B23" s="26">
         <f>DATE(YEAR(A23),MONTH(A23),1)</f>
@@ -2603,17 +2598,18 @@
       </c>
       <c r="C23" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D23" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D23" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E23" s="27" t="inlineStr"/>
-      <c r="F23" s="32" t="n">
-        <v>3453.01</v>
+      <c r="F23" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G23" s="30">
         <f>G22+F23</f>
@@ -2630,7 +2626,7 @@
       </c>
       <c r="C24" s="27" t="inlineStr">
         <is>
-          <t>Paga extra de diciembre</t>
+          <t>Nómina</t>
         </is>
       </c>
       <c r="D24" s="31" t="inlineStr">
@@ -2640,7 +2636,7 @@
       </c>
       <c r="E24" s="27" t="inlineStr"/>
       <c r="F24" s="32" t="n">
-        <v>2014.69</v>
+        <v>3453.01</v>
       </c>
       <c r="G24" s="30">
         <f>G23+F24</f>
@@ -2657,21 +2653,17 @@
       </c>
       <c r="C25" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Joserra</t>
-        </is>
-      </c>
-      <c r="D25" s="37" t="inlineStr">
-        <is>
-          <t>Amigo</t>
-        </is>
-      </c>
-      <c r="E25" s="27" t="inlineStr">
-        <is>
-          <t>Joserra</t>
-        </is>
-      </c>
+          <t>Paga extra de diciembre</t>
+        </is>
+      </c>
+      <c r="D25" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E25" s="27" t="inlineStr"/>
       <c r="F25" s="32" t="n">
-        <v>-400</v>
+        <v>2014.69</v>
       </c>
       <c r="G25" s="30">
         <f>G24+F25</f>
@@ -2680,7 +2672,7 @@
     </row>
     <row r="26">
       <c r="A26" s="25" t="n">
-        <v>46388</v>
+        <v>46385</v>
       </c>
       <c r="B26" s="26">
         <f>DATE(YEAR(A26),MONTH(A26),1)</f>
@@ -2688,21 +2680,21 @@
       </c>
       <c r="C26" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D26" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Devolución a Joserra (puente + lo anterior)</t>
+        </is>
+      </c>
+      <c r="D26" s="34" t="inlineStr">
+        <is>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E26" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Joserra</t>
         </is>
       </c>
       <c r="F26" s="32" t="n">
-        <v>-96</v>
+        <v>-1000</v>
       </c>
       <c r="G26" s="30">
         <f>G25+F26</f>
@@ -2719,21 +2711,21 @@
       </c>
       <c r="C27" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
+          <t>Santander (préstamo) · cuota</t>
         </is>
       </c>
       <c r="D27" s="36" t="inlineStr">
         <is>
-          <t>Aplazable</t>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E27" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F27" s="32" t="n">
-        <v>-122.46</v>
+        <v>-96</v>
       </c>
       <c r="G27" s="30">
         <f>G26+F27</f>
@@ -2750,21 +2742,21 @@
       </c>
       <c r="C28" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 2/3</t>
-        </is>
-      </c>
-      <c r="D28" s="36" t="inlineStr">
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D28" s="37" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E28" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1</t>
+          <t>Crédito Santander 2</t>
         </is>
       </c>
       <c r="F28" s="32" t="n">
-        <v>-231.11</v>
+        <v>-122.46</v>
       </c>
       <c r="G28" s="30">
         <f>G27+F28</f>
@@ -2781,21 +2773,21 @@
       </c>
       <c r="C29" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 2/3</t>
-        </is>
-      </c>
-      <c r="D29" s="36" t="inlineStr">
+          <t>Pagolisto 1 · cuota 2/3</t>
+        </is>
+      </c>
+      <c r="D29" s="37" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E29" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2</t>
+          <t>Pagolisto 1</t>
         </is>
       </c>
       <c r="F29" s="32" t="n">
-        <v>-307.87</v>
+        <v>-231.11</v>
       </c>
       <c r="G29" s="30">
         <f>G28+F29</f>
@@ -2812,21 +2804,21 @@
       </c>
       <c r="C30" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 2/3</t>
-        </is>
-      </c>
-      <c r="D30" s="36" t="inlineStr">
+          <t>Pagolisto 2 · cuota 2/3</t>
+        </is>
+      </c>
+      <c r="D30" s="37" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E30" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1</t>
+          <t>Pagolisto 2</t>
         </is>
       </c>
       <c r="F30" s="32" t="n">
-        <v>-494.54</v>
+        <v>-307.87</v>
       </c>
       <c r="G30" s="30">
         <f>G29+F30</f>
@@ -2843,21 +2835,21 @@
       </c>
       <c r="C31" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Xabi</t>
+          <t>Crédito Santander 1 · cuota 2/3</t>
         </is>
       </c>
       <c r="D31" s="37" t="inlineStr">
         <is>
-          <t>Amigo</t>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E31" s="27" t="inlineStr">
         <is>
-          <t>Xabi</t>
+          <t>Crédito Santander 1</t>
         </is>
       </c>
       <c r="F31" s="32" t="n">
-        <v>-300</v>
+        <v>-494.54</v>
       </c>
       <c r="G31" s="30">
         <f>G30+F31</f>
@@ -2874,18 +2866,21 @@
       </c>
       <c r="C32" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D32" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E32" s="27" t="inlineStr"/>
-      <c r="F32" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Devolución a Xabi</t>
+        </is>
+      </c>
+      <c r="D32" s="34" t="inlineStr">
+        <is>
+          <t>Amigo</t>
+        </is>
+      </c>
+      <c r="E32" s="27" t="inlineStr">
+        <is>
+          <t>Xabi</t>
+        </is>
+      </c>
+      <c r="F32" s="32" t="n">
+        <v>-300</v>
       </c>
       <c r="G32" s="30">
         <f>G31+F32</f>
@@ -2894,7 +2889,7 @@
     </row>
     <row r="33">
       <c r="A33" s="25" t="n">
-        <v>46416</v>
+        <v>46388</v>
       </c>
       <c r="B33" s="26">
         <f>DATE(YEAR(A33),MONTH(A33),1)</f>
@@ -2902,17 +2897,18 @@
       </c>
       <c r="C33" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D33" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D33" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E33" s="27" t="inlineStr"/>
-      <c r="F33" s="32" t="n">
-        <v>3173.56</v>
+      <c r="F33" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G33" s="30">
         <f>G32+F33</f>
@@ -2921,7 +2917,7 @@
     </row>
     <row r="34">
       <c r="A34" s="25" t="n">
-        <v>46419</v>
+        <v>46416</v>
       </c>
       <c r="B34" s="26">
         <f>DATE(YEAR(A34),MONTH(A34),1)</f>
@@ -2929,21 +2925,17 @@
       </c>
       <c r="C34" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · cuota</t>
-        </is>
-      </c>
-      <c r="D34" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E34" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D34" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E34" s="27" t="inlineStr"/>
       <c r="F34" s="32" t="n">
-        <v>-96</v>
+        <v>3173.56</v>
       </c>
       <c r="G34" s="30">
         <f>G33+F34</f>
@@ -2960,21 +2952,21 @@
       </c>
       <c r="C35" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · cuota</t>
+          <t>Santander (préstamo) · cuota</t>
         </is>
       </c>
       <c r="D35" s="36" t="inlineStr">
         <is>
-          <t>Aplazable</t>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E35" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F35" s="32" t="n">
-        <v>-122.46</v>
+        <v>-96</v>
       </c>
       <c r="G35" s="30">
         <f>G34+F35</f>
@@ -2991,21 +2983,21 @@
       </c>
       <c r="C36" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1 · cuota 3/3</t>
-        </is>
-      </c>
-      <c r="D36" s="36" t="inlineStr">
+          <t>Crédito Santander 2 · cuota</t>
+        </is>
+      </c>
+      <c r="D36" s="37" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E36" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 1</t>
+          <t>Crédito Santander 2</t>
         </is>
       </c>
       <c r="F36" s="32" t="n">
-        <v>-231.12</v>
+        <v>-122.46</v>
       </c>
       <c r="G36" s="30">
         <f>G35+F36</f>
@@ -3022,21 +3014,21 @@
       </c>
       <c r="C37" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2 · cuota 3/3</t>
-        </is>
-      </c>
-      <c r="D37" s="36" t="inlineStr">
+          <t>Pagolisto 1 · cuota 3/3</t>
+        </is>
+      </c>
+      <c r="D37" s="37" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E37" s="27" t="inlineStr">
         <is>
-          <t>Pagolisto 2</t>
+          <t>Pagolisto 1</t>
         </is>
       </c>
       <c r="F37" s="32" t="n">
-        <v>-307.87</v>
+        <v>-231.12</v>
       </c>
       <c r="G37" s="30">
         <f>G36+F37</f>
@@ -3053,21 +3045,21 @@
       </c>
       <c r="C38" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1 · cuota 3/3</t>
-        </is>
-      </c>
-      <c r="D38" s="36" t="inlineStr">
+          <t>Pagolisto 2 · cuota 3/3</t>
+        </is>
+      </c>
+      <c r="D38" s="37" t="inlineStr">
         <is>
           <t>Aplazable</t>
         </is>
       </c>
       <c r="E38" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 1</t>
+          <t>Pagolisto 2</t>
         </is>
       </c>
       <c r="F38" s="32" t="n">
-        <v>-494.55</v>
+        <v>-307.87</v>
       </c>
       <c r="G38" s="30">
         <f>G37+F38</f>
@@ -3084,21 +3076,21 @@
       </c>
       <c r="C39" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Sergio</t>
+          <t>Crédito Santander 1 · cuota 3/3</t>
         </is>
       </c>
       <c r="D39" s="37" t="inlineStr">
         <is>
-          <t>Amigo</t>
+          <t>Aplazable</t>
         </is>
       </c>
       <c r="E39" s="27" t="inlineStr">
         <is>
-          <t>Sergio</t>
+          <t>Crédito Santander 1</t>
         </is>
       </c>
       <c r="F39" s="32" t="n">
-        <v>-1700</v>
+        <v>-494.55</v>
       </c>
       <c r="G39" s="30">
         <f>G38+F39</f>
@@ -3115,18 +3107,21 @@
       </c>
       <c r="C40" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D40" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E40" s="27" t="inlineStr"/>
-      <c r="F40" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Devolución a Sergio</t>
+        </is>
+      </c>
+      <c r="D40" s="34" t="inlineStr">
+        <is>
+          <t>Amigo</t>
+        </is>
+      </c>
+      <c r="E40" s="27" t="inlineStr">
+        <is>
+          <t>Sergio</t>
+        </is>
+      </c>
+      <c r="F40" s="32" t="n">
+        <v>-1700</v>
       </c>
       <c r="G40" s="30">
         <f>G39+F40</f>
@@ -3135,7 +3130,7 @@
     </row>
     <row r="41">
       <c r="A41" s="25" t="n">
-        <v>46446</v>
+        <v>46419</v>
       </c>
       <c r="B41" s="26">
         <f>DATE(YEAR(A41),MONTH(A41),1)</f>
@@ -3143,17 +3138,18 @@
       </c>
       <c r="C41" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D41" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D41" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E41" s="27" t="inlineStr"/>
-      <c r="F41" s="32" t="n">
-        <v>3173.56</v>
+      <c r="F41" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G41" s="30">
         <f>G40+F41</f>
@@ -3170,7 +3166,7 @@
       </c>
       <c r="C42" s="27" t="inlineStr">
         <is>
-          <t>Variable de febrero</t>
+          <t>Nómina</t>
         </is>
       </c>
       <c r="D42" s="31" t="inlineStr">
@@ -3180,7 +3176,7 @@
       </c>
       <c r="E42" s="27" t="inlineStr"/>
       <c r="F42" s="32" t="n">
-        <v>2114.45</v>
+        <v>3173.56</v>
       </c>
       <c r="G42" s="30">
         <f>G41+F42</f>
@@ -3197,21 +3193,17 @@
       </c>
       <c r="C43" s="27" t="inlineStr">
         <is>
-          <t>Devolución a Txomin</t>
-        </is>
-      </c>
-      <c r="D43" s="37" t="inlineStr">
-        <is>
-          <t>Amigo</t>
-        </is>
-      </c>
-      <c r="E43" s="27" t="inlineStr">
-        <is>
-          <t>Txomin</t>
-        </is>
-      </c>
+          <t>Variable de febrero</t>
+        </is>
+      </c>
+      <c r="D43" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E43" s="27" t="inlineStr"/>
       <c r="F43" s="32" t="n">
-        <v>-2500</v>
+        <v>2114.45</v>
       </c>
       <c r="G43" s="30">
         <f>G42+F43</f>
@@ -3220,7 +3212,7 @@
     </row>
     <row r="44">
       <c r="A44" s="25" t="n">
-        <v>46447</v>
+        <v>46446</v>
       </c>
       <c r="B44" s="26">
         <f>DATE(YEAR(A44),MONTH(A44),1)</f>
@@ -3228,21 +3220,21 @@
       </c>
       <c r="C44" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D44" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
+          <t>Devolución a Txomin</t>
+        </is>
+      </c>
+      <c r="D44" s="34" t="inlineStr">
+        <is>
+          <t>Amigo</t>
         </is>
       </c>
       <c r="E44" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo)</t>
+          <t>Txomin</t>
         </is>
       </c>
       <c r="F44" s="32" t="n">
-        <v>-96</v>
+        <v>-2500</v>
       </c>
       <c r="G44" s="30">
         <f>G43+F44</f>
@@ -3259,21 +3251,21 @@
       </c>
       <c r="C45" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
         </is>
       </c>
       <c r="D45" s="36" t="inlineStr">
         <is>
-          <t>Aplazable</t>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E45" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F45" s="32" t="n">
-        <v>-404</v>
+        <v>-96</v>
       </c>
       <c r="G45" s="30">
         <f>G44+F45</f>
@@ -3290,18 +3282,21 @@
       </c>
       <c r="C46" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D46" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E46" s="27" t="inlineStr"/>
-      <c r="F46" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D46" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E46" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F46" s="32" t="n">
+        <v>-404</v>
       </c>
       <c r="G46" s="30">
         <f>G45+F46</f>
@@ -3310,7 +3305,7 @@
     </row>
     <row r="47">
       <c r="A47" s="25" t="n">
-        <v>46475</v>
+        <v>46447</v>
       </c>
       <c r="B47" s="26">
         <f>DATE(YEAR(A47),MONTH(A47),1)</f>
@@ -3318,17 +3313,18 @@
       </c>
       <c r="C47" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D47" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D47" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E47" s="27" t="inlineStr"/>
-      <c r="F47" s="32" t="n">
-        <v>3173.56</v>
+      <c r="F47" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G47" s="30">
         <f>G46+F47</f>
@@ -3337,7 +3333,7 @@
     </row>
     <row r="48">
       <c r="A48" s="25" t="n">
-        <v>46478</v>
+        <v>46475</v>
       </c>
       <c r="B48" s="26">
         <f>DATE(YEAR(A48),MONTH(A48),1)</f>
@@ -3345,21 +3341,17 @@
       </c>
       <c r="C48" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D48" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E48" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D48" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E48" s="27" t="inlineStr"/>
       <c r="F48" s="32" t="n">
-        <v>-96</v>
+        <v>3173.56</v>
       </c>
       <c r="G48" s="30">
         <f>G47+F48</f>
@@ -3376,21 +3368,21 @@
       </c>
       <c r="C49" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
         </is>
       </c>
       <c r="D49" s="36" t="inlineStr">
         <is>
-          <t>Aplazable</t>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E49" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F49" s="32" t="n">
-        <v>-404</v>
+        <v>-96</v>
       </c>
       <c r="G49" s="30">
         <f>G48+F49</f>
@@ -3407,18 +3399,21 @@
       </c>
       <c r="C50" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D50" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E50" s="27" t="inlineStr"/>
-      <c r="F50" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D50" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E50" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F50" s="32" t="n">
+        <v>-404</v>
       </c>
       <c r="G50" s="30">
         <f>G49+F50</f>
@@ -3427,7 +3422,7 @@
     </row>
     <row r="51">
       <c r="A51" s="25" t="n">
-        <v>46506</v>
+        <v>46478</v>
       </c>
       <c r="B51" s="26">
         <f>DATE(YEAR(A51),MONTH(A51),1)</f>
@@ -3435,17 +3430,18 @@
       </c>
       <c r="C51" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D51" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D51" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E51" s="27" t="inlineStr"/>
-      <c r="F51" s="32" t="n">
-        <v>3173.56</v>
+      <c r="F51" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G51" s="30">
         <f>G50+F51</f>
@@ -3454,7 +3450,7 @@
     </row>
     <row r="52">
       <c r="A52" s="25" t="n">
-        <v>46508</v>
+        <v>46506</v>
       </c>
       <c r="B52" s="26">
         <f>DATE(YEAR(A52),MONTH(A52),1)</f>
@@ -3462,21 +3458,17 @@
       </c>
       <c r="C52" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D52" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E52" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D52" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E52" s="27" t="inlineStr"/>
       <c r="F52" s="32" t="n">
-        <v>-96</v>
+        <v>3173.56</v>
       </c>
       <c r="G52" s="30">
         <f>G51+F52</f>
@@ -3493,21 +3485,21 @@
       </c>
       <c r="C53" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
         </is>
       </c>
       <c r="D53" s="36" t="inlineStr">
         <is>
-          <t>Aplazable</t>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E53" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F53" s="32" t="n">
-        <v>-404</v>
+        <v>-96</v>
       </c>
       <c r="G53" s="30">
         <f>G52+F53</f>
@@ -3524,18 +3516,21 @@
       </c>
       <c r="C54" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D54" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E54" s="27" t="inlineStr"/>
-      <c r="F54" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D54" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E54" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F54" s="32" t="n">
+        <v>-404</v>
       </c>
       <c r="G54" s="30">
         <f>G53+F54</f>
@@ -3544,7 +3539,7 @@
     </row>
     <row r="55">
       <c r="A55" s="25" t="n">
-        <v>46536</v>
+        <v>46508</v>
       </c>
       <c r="B55" s="26">
         <f>DATE(YEAR(A55),MONTH(A55),1)</f>
@@ -3552,17 +3547,18 @@
       </c>
       <c r="C55" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D55" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D55" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E55" s="27" t="inlineStr"/>
-      <c r="F55" s="32" t="n">
-        <v>3173.56</v>
+      <c r="F55" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G55" s="30">
         <f>G54+F55</f>
@@ -3571,7 +3567,7 @@
     </row>
     <row r="56">
       <c r="A56" s="25" t="n">
-        <v>46539</v>
+        <v>46536</v>
       </c>
       <c r="B56" s="26">
         <f>DATE(YEAR(A56),MONTH(A56),1)</f>
@@ -3579,21 +3575,17 @@
       </c>
       <c r="C56" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D56" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E56" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D56" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E56" s="27" t="inlineStr"/>
       <c r="F56" s="32" t="n">
-        <v>-96</v>
+        <v>3173.56</v>
       </c>
       <c r="G56" s="30">
         <f>G55+F56</f>
@@ -3610,21 +3602,21 @@
       </c>
       <c r="C57" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
         </is>
       </c>
       <c r="D57" s="36" t="inlineStr">
         <is>
-          <t>Aplazable</t>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E57" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F57" s="32" t="n">
-        <v>-404</v>
+        <v>-96</v>
       </c>
       <c r="G57" s="30">
         <f>G56+F57</f>
@@ -3641,18 +3633,21 @@
       </c>
       <c r="C58" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D58" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E58" s="27" t="inlineStr"/>
-      <c r="F58" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D58" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E58" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F58" s="32" t="n">
+        <v>-404</v>
       </c>
       <c r="G58" s="30">
         <f>G57+F58</f>
@@ -3661,7 +3656,7 @@
     </row>
     <row r="59">
       <c r="A59" s="25" t="n">
-        <v>46567</v>
+        <v>46539</v>
       </c>
       <c r="B59" s="26">
         <f>DATE(YEAR(A59),MONTH(A59),1)</f>
@@ -3669,17 +3664,18 @@
       </c>
       <c r="C59" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D59" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D59" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E59" s="27" t="inlineStr"/>
-      <c r="F59" s="32" t="n">
-        <v>3173.56</v>
+      <c r="F59" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G59" s="30">
         <f>G58+F59</f>
@@ -3696,7 +3692,7 @@
       </c>
       <c r="C60" s="27" t="inlineStr">
         <is>
-          <t>Paga extra de junio</t>
+          <t>Nómina</t>
         </is>
       </c>
       <c r="D60" s="31" t="inlineStr">
@@ -3706,7 +3702,7 @@
       </c>
       <c r="E60" s="27" t="inlineStr"/>
       <c r="F60" s="32" t="n">
-        <v>1989.05</v>
+        <v>3173.56</v>
       </c>
       <c r="G60" s="30">
         <f>G59+F60</f>
@@ -3715,7 +3711,7 @@
     </row>
     <row r="61">
       <c r="A61" s="25" t="n">
-        <v>46569</v>
+        <v>46567</v>
       </c>
       <c r="B61" s="26">
         <f>DATE(YEAR(A61),MONTH(A61),1)</f>
@@ -3723,21 +3719,17 @@
       </c>
       <c r="C61" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D61" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E61" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
+          <t>Paga extra de junio</t>
+        </is>
+      </c>
+      <c r="D61" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E61" s="27" t="inlineStr"/>
       <c r="F61" s="32" t="n">
-        <v>-279.08</v>
+        <v>1989.05</v>
       </c>
       <c r="G61" s="30">
         <f>G60+F61</f>
@@ -3754,21 +3746,21 @@
       </c>
       <c r="C62" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2 · plan 500 €/mes</t>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
         </is>
       </c>
       <c r="D62" s="36" t="inlineStr">
         <is>
-          <t>Aplazable</t>
+          <t>Fijo</t>
         </is>
       </c>
       <c r="E62" s="27" t="inlineStr">
         <is>
-          <t>Crédito Santander 2</t>
+          <t>Santander (préstamo)</t>
         </is>
       </c>
       <c r="F62" s="32" t="n">
-        <v>-220.92</v>
+        <v>-156.62</v>
       </c>
       <c r="G62" s="30">
         <f>G61+F62</f>
@@ -3785,18 +3777,21 @@
       </c>
       <c r="C63" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D63" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E63" s="27" t="inlineStr"/>
-      <c r="F63" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Crédito Santander 2 · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D63" s="37" t="inlineStr">
+        <is>
+          <t>Aplazable</t>
+        </is>
+      </c>
+      <c r="E63" s="27" t="inlineStr">
+        <is>
+          <t>Crédito Santander 2</t>
+        </is>
+      </c>
+      <c r="F63" s="32" t="n">
+        <v>-343.38</v>
       </c>
       <c r="G63" s="30">
         <f>G62+F63</f>
@@ -3805,7 +3800,7 @@
     </row>
     <row r="64">
       <c r="A64" s="25" t="n">
-        <v>46597</v>
+        <v>46569</v>
       </c>
       <c r="B64" s="26">
         <f>DATE(YEAR(A64),MONTH(A64),1)</f>
@@ -3813,17 +3808,18 @@
       </c>
       <c r="C64" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D64" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D64" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E64" s="27" t="inlineStr"/>
-      <c r="F64" s="32" t="n">
-        <v>3173.56</v>
+      <c r="F64" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G64" s="30">
         <f>G63+F64</f>
@@ -3832,7 +3828,7 @@
     </row>
     <row r="65">
       <c r="A65" s="25" t="n">
-        <v>46600</v>
+        <v>46597</v>
       </c>
       <c r="B65" s="26">
         <f>DATE(YEAR(A65),MONTH(A65),1)</f>
@@ -3840,21 +3836,17 @@
       </c>
       <c r="C65" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D65" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E65" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D65" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E65" s="27" t="inlineStr"/>
       <c r="F65" s="32" t="n">
-        <v>-500</v>
+        <v>3173.56</v>
       </c>
       <c r="G65" s="30">
         <f>G64+F65</f>
@@ -3871,18 +3863,21 @@
       </c>
       <c r="C66" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D66" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E66" s="27" t="inlineStr"/>
-      <c r="F66" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D66" s="36" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E66" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F66" s="32" t="n">
+        <v>-500</v>
       </c>
       <c r="G66" s="30">
         <f>G65+F66</f>
@@ -3891,7 +3886,7 @@
     </row>
     <row r="67">
       <c r="A67" s="25" t="n">
-        <v>46628</v>
+        <v>46600</v>
       </c>
       <c r="B67" s="26">
         <f>DATE(YEAR(A67),MONTH(A67),1)</f>
@@ -3899,17 +3894,18 @@
       </c>
       <c r="C67" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D67" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D67" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E67" s="27" t="inlineStr"/>
-      <c r="F67" s="32" t="n">
-        <v>2280.25</v>
+      <c r="F67" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G67" s="30">
         <f>G66+F67</f>
@@ -3918,7 +3914,7 @@
     </row>
     <row r="68">
       <c r="A68" s="25" t="n">
-        <v>46631</v>
+        <v>46628</v>
       </c>
       <c r="B68" s="26">
         <f>DATE(YEAR(A68),MONTH(A68),1)</f>
@@ -3926,21 +3922,17 @@
       </c>
       <c r="C68" s="27" t="inlineStr">
         <is>
-          <t>Santander (préstamo) · plan 500 €/mes</t>
-        </is>
-      </c>
-      <c r="D68" s="33" t="inlineStr">
-        <is>
-          <t>Fijo</t>
-        </is>
-      </c>
-      <c r="E68" s="27" t="inlineStr">
-        <is>
-          <t>Santander (préstamo)</t>
-        </is>
-      </c>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D68" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E68" s="27" t="inlineStr"/>
       <c r="F68" s="32" t="n">
-        <v>-447.85</v>
+        <v>2280.25</v>
       </c>
       <c r="G68" s="30">
         <f>G67+F68</f>
@@ -3957,18 +3949,21 @@
       </c>
       <c r="C69" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D69" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
-        </is>
-      </c>
-      <c r="E69" s="27" t="inlineStr"/>
-      <c r="F69" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D69" s="36" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E69" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
+      <c r="F69" s="32" t="n">
+        <v>-500</v>
       </c>
       <c r="G69" s="30">
         <f>G68+F69</f>
@@ -3977,7 +3972,7 @@
     </row>
     <row r="70">
       <c r="A70" s="25" t="n">
-        <v>46659</v>
+        <v>46631</v>
       </c>
       <c r="B70" s="26">
         <f>DATE(YEAR(A70),MONTH(A70),1)</f>
@@ -3985,17 +3980,18 @@
       </c>
       <c r="C70" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D70" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D70" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
         </is>
       </c>
       <c r="E70" s="27" t="inlineStr"/>
-      <c r="F70" s="32" t="n">
-        <v>3173.56</v>
+      <c r="F70" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
       </c>
       <c r="G70" s="30">
         <f>G69+F70</f>
@@ -4004,7 +4000,7 @@
     </row>
     <row r="71">
       <c r="A71" s="25" t="n">
-        <v>46661</v>
+        <v>46659</v>
       </c>
       <c r="B71" s="26">
         <f>DATE(YEAR(A71),MONTH(A71),1)</f>
@@ -4012,18 +4008,17 @@
       </c>
       <c r="C71" s="27" t="inlineStr">
         <is>
-          <t>Gastos de vida</t>
-        </is>
-      </c>
-      <c r="D71" s="28" t="inlineStr">
-        <is>
-          <t>Gasto</t>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D71" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
         </is>
       </c>
       <c r="E71" s="27" t="inlineStr"/>
-      <c r="F71" s="29">
-        <f>-Supuestos!B7</f>
-        <v/>
+      <c r="F71" s="32" t="n">
+        <v>3173.56</v>
       </c>
       <c r="G71" s="30">
         <f>G70+F71</f>
@@ -4032,7 +4027,7 @@
     </row>
     <row r="72">
       <c r="A72" s="25" t="n">
-        <v>46689</v>
+        <v>46661</v>
       </c>
       <c r="B72" s="26">
         <f>DATE(YEAR(A72),MONTH(A72),1)</f>
@@ -4040,26 +4035,85 @@
       </c>
       <c r="C72" s="27" t="inlineStr">
         <is>
-          <t>Nómina</t>
-        </is>
-      </c>
-      <c r="D72" s="31" t="inlineStr">
-        <is>
-          <t>Ingreso</t>
-        </is>
-      </c>
-      <c r="E72" s="27" t="inlineStr"/>
+          <t>Santander (préstamo) · plan 500 €/mes</t>
+        </is>
+      </c>
+      <c r="D72" s="36" t="inlineStr">
+        <is>
+          <t>Fijo</t>
+        </is>
+      </c>
+      <c r="E72" s="27" t="inlineStr">
+        <is>
+          <t>Santander (préstamo)</t>
+        </is>
+      </c>
       <c r="F72" s="32" t="n">
-        <v>2490.44</v>
+        <v>-70.31</v>
       </c>
       <c r="G72" s="30">
         <f>G71+F72</f>
         <v/>
       </c>
     </row>
+    <row r="73">
+      <c r="A73" s="25" t="n">
+        <v>46661</v>
+      </c>
+      <c r="B73" s="26">
+        <f>DATE(YEAR(A73),MONTH(A73),1)</f>
+        <v/>
+      </c>
+      <c r="C73" s="27" t="inlineStr">
+        <is>
+          <t>Gastos de vida</t>
+        </is>
+      </c>
+      <c r="D73" s="28" t="inlineStr">
+        <is>
+          <t>Gasto</t>
+        </is>
+      </c>
+      <c r="E73" s="27" t="inlineStr"/>
+      <c r="F73" s="29">
+        <f>-Supuestos!B7</f>
+        <v/>
+      </c>
+      <c r="G73" s="30">
+        <f>G72+F73</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="25" t="n">
+        <v>46689</v>
+      </c>
+      <c r="B74" s="26">
+        <f>DATE(YEAR(A74),MONTH(A74),1)</f>
+        <v/>
+      </c>
+      <c r="C74" s="27" t="inlineStr">
+        <is>
+          <t>Nómina</t>
+        </is>
+      </c>
+      <c r="D74" s="31" t="inlineStr">
+        <is>
+          <t>Ingreso</t>
+        </is>
+      </c>
+      <c r="E74" s="27" t="inlineStr"/>
+      <c r="F74" s="32" t="n">
+        <v>2490.44</v>
+      </c>
+      <c r="G74" s="30">
+        <f>G73+F74</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G72"/>
-  <conditionalFormatting sqref="G2:G72">
+  <autoFilter ref="A1:G74"/>
+  <conditionalFormatting sqref="G2:G74">
     <cfRule type="cellIs" priority="1" operator="lessThan" dxfId="1">
       <formula>0</formula>
     </cfRule>
@@ -4133,11 +4187,11 @@
         </is>
       </c>
       <c r="B6" s="41" t="n">
-        <v>300</v>
+        <v>200</v>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>Estimación. Con más de ~350 € el 1 dic queda en negativo (salvo que aplaces los aplazables ese mes)</t>
+          <t>Máximo recomendado: con más de ~330 € el 14 nov (Smartcredito) queda en negativo</t>
         </is>
       </c>
     </row>
@@ -4195,7 +4249,7 @@
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Escenario: nómina de octubre de 3.100 €, Smartcredito el 14 nov, sin préstamos puente ni volver a pedir Moneyman. Ama el 29 nov, Vivus liquidado el 29 nov.</t>
+          <t>Escenario: Joserra presta 600 € (17 oct) y se le devuelven 1.000 € el 29 dic. Ama (800 €) el 29 oct. En nov los aplazables (incluido Crédito Santander 2) se pagan y se vuelven a pedir. Sin volver a pedir Moneyman ni Smartcredito.</t>
         </is>
       </c>
     </row>

</xml_diff>